<commit_message>
deliverable: publish completed customer master
</commit_message>
<xml_diff>
--- a/deliverables/tape-masking-film-customer-master.xlsx
+++ b/deliverables/tape-masking-film-customer-master.xlsx
@@ -2,7 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="Ra7a84bf2eeee4eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="Ra17befd378a0476e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本与流程" sheetId="2" r:id="R8bdb0886f8d2416b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R05c792e53b1b481f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,14 +15,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
     <x:numFmt numFmtId="203" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="204" formatCode="0%"/>
+    <x:numFmt numFmtId="205" formatCode="¥0.00"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -57,6 +60,18 @@
     <x:font>
       <x:sz val="9"/>
       <x:color rgb="FF1F1F1F"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -109,7 +124,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="43">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -186,6 +201,23 @@
     <x:xf numFmtId="204" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -227,9 +259,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerMasterTable" displayName="CustomerMasterTable" ref="A6:AN41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:AN41"/>
-  <x:tableColumns count="40">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerMasterTable" displayName="CustomerMasterTable" ref="A6:AO41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:AO41"/>
+  <x:tableColumns count="41">
     <x:tableColumn id="1" name="研究状态"/>
     <x:tableColumn id="2" name="市场优先级"/>
     <x:tableColumn id="3" name="品类"/>
@@ -254,22 +286,23 @@
     <x:tableColumn id="22" name="官网补充邮箱"/>
     <x:tableColumn id="23" name="API电话"/>
     <x:tableColumn id="24" name="官网补充电话"/>
-    <x:tableColumn id="25" name="WhatsApp"/>
-    <x:tableColumn id="26" name="社交媒体"/>
-    <x:tableColumn id="27" name="官网联系渠道"/>
-    <x:tableColumn id="28" name="API邮箱验证详情"/>
-    <x:tableColumn id="29" name="产品名称"/>
-    <x:tableColumn id="30" name="产品标签"/>
-    <x:tableColumn id="31" name="产品描述/命中证据"/>
-    <x:tableColumn id="32" name="产品别名"/>
-    <x:tableColumn id="33" name="上游词"/>
-    <x:tableColumn id="34" name="下游词"/>
-    <x:tableColumn id="35" name="搜索词"/>
-    <x:tableColumn id="36" name="搜索原始来源"/>
-    <x:tableColumn id="37" name="API联系方式来源"/>
-    <x:tableColumn id="38" name="官网核验来源"/>
-    <x:tableColumn id="39" name="官网核验说明"/>
-    <x:tableColumn id="40" name="最后核验日期"/>
+    <x:tableColumn id="25" name="电话验证详情"/>
+    <x:tableColumn id="26" name="WhatsApp"/>
+    <x:tableColumn id="27" name="社交媒体"/>
+    <x:tableColumn id="28" name="官网联系渠道"/>
+    <x:tableColumn id="29" name="邮箱验证详情"/>
+    <x:tableColumn id="30" name="产品名称"/>
+    <x:tableColumn id="31" name="产品标签"/>
+    <x:tableColumn id="32" name="产品描述/命中证据"/>
+    <x:tableColumn id="33" name="产品别名"/>
+    <x:tableColumn id="34" name="上游词"/>
+    <x:tableColumn id="35" name="下游词"/>
+    <x:tableColumn id="36" name="搜索词"/>
+    <x:tableColumn id="37" name="搜索原始来源"/>
+    <x:tableColumn id="38" name="API联系方式来源"/>
+    <x:tableColumn id="39" name="官网核验来源"/>
+    <x:tableColumn id="40" name="官网核验说明"/>
+    <x:tableColumn id="41" name="最后核验日期"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -494,22 +527,23 @@
     <x:col min="22" max="22" width="35" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="24" hidden="0" customWidth="1"/>
     <x:col min="24" max="24" width="24" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="22" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="32" hidden="0" customWidth="1"/>
-    <x:col min="27" max="27" width="25" hidden="0" customWidth="1"/>
-    <x:col min="28" max="28" width="38" hidden="0" customWidth="1"/>
-    <x:col min="29" max="29" width="30" hidden="0" customWidth="1"/>
-    <x:col min="30" max="30" width="28" hidden="0" customWidth="1"/>
-    <x:col min="31" max="31" width="55" hidden="0" customWidth="1"/>
-    <x:col min="32" max="32" width="35" hidden="0" customWidth="1"/>
-    <x:col min="33" max="33" width="28" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="42" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="22" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="32" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="25" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="38" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="30" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="28" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="55" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="35" hidden="0" customWidth="1"/>
     <x:col min="34" max="34" width="28" hidden="0" customWidth="1"/>
-    <x:col min="35" max="35" width="20" hidden="0" customWidth="1"/>
-    <x:col min="36" max="36" width="32" hidden="0" customWidth="1"/>
-    <x:col min="37" max="37" width="34" hidden="0" customWidth="1"/>
-    <x:col min="38" max="38" width="42" hidden="0" customWidth="1"/>
-    <x:col min="39" max="39" width="50" hidden="0" customWidth="1"/>
-    <x:col min="40" max="40" width="14" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="28" hidden="0" customWidth="1"/>
+    <x:col min="36" max="36" width="20" hidden="0" customWidth="1"/>
+    <x:col min="37" max="37" width="32" hidden="0" customWidth="1"/>
+    <x:col min="38" max="38" width="34" hidden="0" customWidth="1"/>
+    <x:col min="39" max="39" width="42" hidden="0" customWidth="1"/>
+    <x:col min="40" max="40" width="50" hidden="0" customWidth="1"/>
+    <x:col min="41" max="41" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -555,6 +589,7 @@
       <x:c r="AL1" s="7"/>
       <x:c r="AM1" s="7"/>
       <x:c r="AN1" s="7"/>
+      <x:c r="AO1" s="7"/>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="11" t="str">
@@ -599,6 +634,7 @@
       <x:c r="AL2" s="11"/>
       <x:c r="AM2" s="11"/>
       <x:c r="AN2" s="11"/>
+      <x:c r="AO2" s="11"/>
     </x:row>
     <x:row r="3" ht="27" customHeight="1">
       <x:c r="A3" s="15" t="str">
@@ -628,33 +664,33 @@
       <x:c r="O3" s="16"/>
       <x:c r="P3" s="16"/>
       <x:c r="Q3" s="15" t="str">
-        <x:v>已验证邮箱</x:v>
+        <x:v>有效邮箱公司</x:v>
       </x:c>
       <x:c r="R3" s="15"/>
       <x:c r="S3" s="15"/>
       <x:c r="T3" s="15"/>
       <x:c r="U3" s="16" t="n">
-        <x:f>COUNTIF(H7:H41,"*已*验*")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF(H7:H41,"已验证有效")</x:f>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="V3" s="16"/>
       <x:c r="W3" s="16"/>
       <x:c r="X3" s="16"/>
       <x:c r="Y3" s="15" t="str">
-        <x:v>平均联系完整度</x:v>
+        <x:v>有效电话公司</x:v>
       </x:c>
       <x:c r="Z3" s="15"/>
       <x:c r="AA3" s="15"/>
       <x:c r="AB3" s="15"/>
       <x:c r="AC3" s="16" t="n">
-        <x:f>AVERAGE(K7:K41)</x:f>
-        <x:v>0.7571428571428572</x:v>
+        <x:f>COUNTIF(Y7:Y41,"*状态1*")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AD3" s="16"/>
       <x:c r="AE3" s="16"/>
       <x:c r="AF3" s="16"/>
       <x:c r="AG3" s="17" t="str">
-        <x:v>OpenAPI 累计费用：¥49.50（前期上限 ¥50）</x:v>
+        <x:v>OpenAPI 累计费用：¥81.60 / 上限 ¥100.00</x:v>
       </x:c>
       <x:c r="AH3" s="17"/>
       <x:c r="AI3" s="17"/>
@@ -663,10 +699,11 @@
       <x:c r="AL3" s="17"/>
       <x:c r="AM3" s="17"/>
       <x:c r="AN3" s="17"/>
+      <x:c r="AO3" s="17"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="22" t="str">
-        <x:v>使用：先按“市场优先级”和“邮箱可用状态”筛选；“跟进状态/负责人”为人工维护列。邮箱状态 0=未检测，1=有效，2=无效，3=不确定。完整原始数据见 data/raw/。</x:v>
+        <x:v>使用：先筛选“市场优先级”和“邮箱可用状态”。邮箱 1=有效、2=无效、3=不确定、0=接口已调用但未能检测；电话详情为 状态/类型/WhatsApp。原始证据见 data/raw/。</x:v>
       </x:c>
       <x:c r="B4" s="22"/>
       <x:c r="C4" s="22"/>
@@ -707,6 +744,7 @@
       <x:c r="AL4" s="22"/>
       <x:c r="AM4" s="22"/>
       <x:c r="AN4" s="22"/>
+      <x:c r="AO4" s="22"/>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
       <x:c r="A6" s="27" t="str">
@@ -782,51 +820,54 @@
         <x:v>官网补充电话</x:v>
       </x:c>
       <x:c r="Y6" s="27" t="str">
+        <x:v>电话验证详情</x:v>
+      </x:c>
+      <x:c r="Z6" s="27" t="str">
         <x:v>WhatsApp</x:v>
       </x:c>
-      <x:c r="Z6" s="27" t="str">
+      <x:c r="AA6" s="27" t="str">
         <x:v>社交媒体</x:v>
       </x:c>
-      <x:c r="AA6" s="27" t="str">
+      <x:c r="AB6" s="27" t="str">
         <x:v>官网联系渠道</x:v>
       </x:c>
-      <x:c r="AB6" s="27" t="str">
-        <x:v>API邮箱验证详情</x:v>
-      </x:c>
       <x:c r="AC6" s="27" t="str">
+        <x:v>邮箱验证详情</x:v>
+      </x:c>
+      <x:c r="AD6" s="27" t="str">
         <x:v>产品名称</x:v>
       </x:c>
-      <x:c r="AD6" s="27" t="str">
+      <x:c r="AE6" s="27" t="str">
         <x:v>产品标签</x:v>
       </x:c>
-      <x:c r="AE6" s="27" t="str">
+      <x:c r="AF6" s="27" t="str">
         <x:v>产品描述/命中证据</x:v>
       </x:c>
-      <x:c r="AF6" s="27" t="str">
+      <x:c r="AG6" s="27" t="str">
         <x:v>产品别名</x:v>
       </x:c>
-      <x:c r="AG6" s="27" t="str">
+      <x:c r="AH6" s="27" t="str">
         <x:v>上游词</x:v>
       </x:c>
-      <x:c r="AH6" s="27" t="str">
+      <x:c r="AI6" s="27" t="str">
         <x:v>下游词</x:v>
       </x:c>
-      <x:c r="AI6" s="27" t="str">
+      <x:c r="AJ6" s="27" t="str">
         <x:v>搜索词</x:v>
       </x:c>
-      <x:c r="AJ6" s="27" t="str">
+      <x:c r="AK6" s="27" t="str">
         <x:v>搜索原始来源</x:v>
       </x:c>
-      <x:c r="AK6" s="27" t="str">
+      <x:c r="AL6" s="27" t="str">
         <x:v>API联系方式来源</x:v>
       </x:c>
-      <x:c r="AL6" s="27" t="str">
+      <x:c r="AM6" s="27" t="str">
         <x:v>官网核验来源</x:v>
       </x:c>
-      <x:c r="AM6" s="27" t="str">
+      <x:c r="AN6" s="27" t="str">
         <x:v>官网核验说明</x:v>
       </x:c>
-      <x:c r="AN6" s="27" t="str">
+      <x:c r="AO6" s="27" t="str">
         <x:v>最后核验日期</x:v>
       </x:c>
     </x:row>
@@ -850,19 +891,16 @@
         <x:v>GB</x:v>
       </x:c>
       <x:c r="G7" s="30" t="str">
-        <x:f>IF(V7&lt;&gt;"",V7,U7)</x:f>
         <x:v>echrisman@polifilm.us</x:v>
       </x:c>
       <x:c r="H7" s="30" t="str">
-        <x:f>IF(V7&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB7)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
-      </x:c>
-      <x:c r="I7" s="30" t="str">
-        <x:f>IF(X7&lt;&gt;"",X7,W7)</x:f>
-      </x:c>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC7)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC7)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC7)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC7)),"判定无效",IF(V7&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
+      </x:c>
+      <x:c r="I7" s="30" t="str"/>
       <x:c r="J7" s="30" t="str"/>
       <x:c r="K7" s="35" t="n">
-        <x:f>ROUND((IF(G7&lt;&gt;"",40,0)+IF(I7&lt;&gt;"",25,0)+IF(J7&lt;&gt;"",20,0)+IF(Z7&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H7="已验证有效",40,IF(V7&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y7)),25,0)+IF(J7&lt;&gt;"",20,0)+IF(AA7&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="L7" s="30" t="str">
@@ -895,29 +933,30 @@
       <x:c r="Y7" s="30" t="str"/>
       <x:c r="Z7" s="30" t="str"/>
       <x:c r="AA7" s="30" t="str"/>
-      <x:c r="AB7" s="30" t="str">
+      <x:c r="AB7" s="30" t="str"/>
+      <x:c r="AC7" s="30" t="str">
         <x:v>echrisman@polifilm.us:1</x:v>
       </x:c>
-      <x:c r="AC7" s="30" t="str"/>
       <x:c r="AD7" s="30" t="str"/>
-      <x:c r="AE7" s="30" t="str">
+      <x:c r="AE7" s="30" t="str"/>
+      <x:c r="AF7" s="30" t="str">
         <x:v>168 ROLLS OF POLYETHYLENE MASKING FILM (HS#39 20.10)P ACKED ONTO 28 PALLETS REF #103354 IR S NUMBER:36-3437 757</x:v>
       </x:c>
-      <x:c r="AF7" s="30" t="str"/>
       <x:c r="AG7" s="30" t="str"/>
       <x:c r="AH7" s="30" t="str"/>
-      <x:c r="AI7" s="30" t="str">
+      <x:c r="AI7" s="30" t="str"/>
+      <x:c r="AJ7" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ7" s="30" t="str">
+      <x:c r="AK7" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK7" s="30" t="str">
+      <x:c r="AL7" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL7" s="30" t="str"/>
       <x:c r="AM7" s="30" t="str"/>
-      <x:c r="AN7" s="34" t="n">
+      <x:c r="AN7" s="30" t="str"/>
+      <x:c r="AO7" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -941,21 +980,18 @@
         <x:v>US</x:v>
       </x:c>
       <x:c r="G8" s="30" t="str">
-        <x:f>IF(V8&lt;&gt;"",V8,U8)</x:f>
         <x:v>restrada@poli-film.net</x:v>
       </x:c>
       <x:c r="H8" s="30" t="str">
-        <x:f>IF(V8&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB8)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
-      </x:c>
-      <x:c r="I8" s="30" t="str">
-        <x:f>IF(X8&lt;&gt;"",X8,W8)</x:f>
-      </x:c>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC8)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC8)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC8)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC8)),"判定无效",IF(V8&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
+      </x:c>
+      <x:c r="I8" s="30" t="str"/>
       <x:c r="J8" s="30" t="str">
         <x:v>http://www.polifilmamerica.com/</x:v>
       </x:c>
       <x:c r="K8" s="35" t="n">
-        <x:f>ROUND((IF(G8&lt;&gt;"",40,0)+IF(I8&lt;&gt;"",25,0)+IF(J8&lt;&gt;"",20,0)+IF(Z8&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H8="已验证有效",40,IF(V8&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y8)),25,0)+IF(J8&lt;&gt;"",20,0)+IF(AA8&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="L8" s="30" t="str">
@@ -990,31 +1026,32 @@
       <x:c r="Y8" s="30" t="str"/>
       <x:c r="Z8" s="30" t="str"/>
       <x:c r="AA8" s="30" t="str"/>
-      <x:c r="AB8" s="30" t="str">
+      <x:c r="AB8" s="30" t="str"/>
+      <x:c r="AC8" s="30" t="str">
         <x:v>restrada@poli-film.net:1</x:v>
       </x:c>
-      <x:c r="AC8" s="30" t="str"/>
-      <x:c r="AD8" s="30" t="str">
+      <x:c r="AD8" s="30" t="str"/>
+      <x:c r="AE8" s="30" t="str">
         <x:v>tin; polyethylene; masking film; poly ethylene; po le; cat; ion; rolls</x:v>
       </x:c>
-      <x:c r="AE8" s="30" t="str">
+      <x:c r="AF8" s="30" t="str">
         <x:v>POLYETHYLENE MASKING FILM - ROLLS OF POLY ETHYLENE MASKING FILM(..)PACK ED ONTO PALLETS REF# ,W-- PO #PO LEG// =CONSIGNEE &amp; NOTIFY CONTINUE: TEL:+- TAX IDEN TIFICATION NUMBE R:PME--T&lt;br/&gt;</x:v>
       </x:c>
-      <x:c r="AF8" s="30" t="str"/>
       <x:c r="AG8" s="30" t="str"/>
       <x:c r="AH8" s="30" t="str"/>
-      <x:c r="AI8" s="30" t="str">
+      <x:c r="AI8" s="30" t="str"/>
+      <x:c r="AJ8" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ8" s="30" t="str">
+      <x:c r="AK8" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK8" s="30" t="str">
+      <x:c r="AL8" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL8" s="30" t="str"/>
       <x:c r="AM8" s="30" t="str"/>
-      <x:c r="AN8" s="34" t="n">
+      <x:c r="AN8" s="30" t="str"/>
+      <x:c r="AO8" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -1038,23 +1075,21 @@
         <x:v>US</x:v>
       </x:c>
       <x:c r="G9" s="30" t="str">
-        <x:f>IF(V9&lt;&gt;"",V9,U9)</x:f>
         <x:v>jtaub@pacoa.com</x:v>
       </x:c>
       <x:c r="H9" s="30" t="str">
-        <x:f>IF(V9&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB9)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC9)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC9)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC9)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC9)),"判定无效",IF(V9&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>验证不确定</x:v>
       </x:c>
       <x:c r="I9" s="30" t="str">
-        <x:f>IF(X9&lt;&gt;"",X9,W9)</x:f>
-        <x:v>888.284.3000; 516.284.3000</x:v>
+        <x:v>516.284.3000</x:v>
       </x:c>
       <x:c r="J9" s="30" t="str">
         <x:v>www.pacoa.com</x:v>
       </x:c>
       <x:c r="K9" s="35" t="n">
-        <x:f>ROUND((IF(G9&lt;&gt;"",40,0)+IF(I9&lt;&gt;"",25,0)+IF(J9&lt;&gt;"",20,0)+IF(Z9&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.85</x:v>
+        <x:f>ROUND((IF(H9="已验证有效",40,IF(V9&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y9)),25,0)+IF(J9&lt;&gt;"",20,0)+IF(AA9&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="L9" s="30" t="str">
         <x:v>待联系</x:v>
@@ -1082,7 +1117,7 @@
         <x:v>46146.666666666664</x:v>
       </x:c>
       <x:c r="U9" s="30" t="str">
-        <x:v>jtaub@pacoa.com</x:v>
+        <x:v>jtaub@pacoa.com; joe1199@live.com</x:v>
       </x:c>
       <x:c r="V9" s="30" t="str"/>
       <x:c r="W9" s="30" t="str">
@@ -1091,40 +1126,45 @@
       <x:c r="X9" s="30" t="str">
         <x:v>888.284.3000; 516.284.3000</x:v>
       </x:c>
-      <x:c r="Y9" s="30" t="str"/>
+      <x:c r="Y9" s="30" t="str">
+        <x:v>+1 516-284-3000:状态1/类型3/WhatsApp2; 888.284.3000:状态3/类型0/WhatsApp0; 516.284.3000:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z9" s="30" t="str"/>
       <x:c r="AA9" s="30" t="str">
+        <x:v>https://www.linkedin.com/in/joseph-scherrer-0230a11b</x:v>
+      </x:c>
+      <x:c r="AB9" s="30" t="str">
         <x:v>Website inquiry form</x:v>
       </x:c>
-      <x:c r="AB9" s="30" t="str">
-        <x:v>jtaub@pacoa.com:0</x:v>
-      </x:c>
-      <x:c r="AC9" s="30" t="str"/>
-      <x:c r="AD9" s="30" t="str">
+      <x:c r="AC9" s="30" t="str">
+        <x:v>jtaub@pacoa.com:3; joe1199@live.com:2</x:v>
+      </x:c>
+      <x:c r="AD9" s="30" t="str"/>
+      <x:c r="AE9" s="30" t="str">
         <x:v>wood; plastic drop cloth; ipm; caution tape; sol; masking film; packing material; hat; xxxxx</x:v>
       </x:c>
-      <x:c r="AE9" s="30" t="str">
+      <x:c r="AF9" s="30" t="str">
         <x:v>2,886 CTNS OF PLASTIC DROP CLOTH, MASKING FILM AND CAUTION TAPE P.O. NO.: XXXXXX WE CERT IFY THAT THIS SHIPMENT CONTAINS NO SOLID WOODPACKING MATERIALS.&lt;br/&gt;</x:v>
       </x:c>
-      <x:c r="AF9" s="30" t="str"/>
       <x:c r="AG9" s="30" t="str"/>
       <x:c r="AH9" s="30" t="str"/>
-      <x:c r="AI9" s="30" t="str">
+      <x:c r="AI9" s="30" t="str"/>
+      <x:c r="AJ9" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ9" s="30" t="str">
+      <x:c r="AK9" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK9" s="30" t="str">
-        <x:v>UpKuajing customs company contact API</x:v>
-      </x:c>
       <x:c r="AL9" s="30" t="str">
+        <x:v>UpKuajing customs company contact API; UpKuajing reviewed person contact API</x:v>
+      </x:c>
+      <x:c r="AM9" s="30" t="str">
         <x:v>https://www.pacoa.com/contactus</x:v>
       </x:c>
-      <x:c r="AM9" s="30" t="str">
-        <x:v>Official contact page confirmed address, phone numbers and inquiry form; API email was not displayed on the page.</x:v>
-      </x:c>
-      <x:c r="AN9" s="34" t="n">
+      <x:c r="AN9" s="30" t="str">
+        <x:v>Official contact page confirmed address, phone numbers and inquiry form; API email was not displayed on the page.; 人物补充：Joseph Scherrer（Assistant Buyer）；采购岗位，且公司精确匹配 PACOA。</x:v>
+      </x:c>
+      <x:c r="AO9" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -1148,23 +1188,21 @@
         <x:v>US</x:v>
       </x:c>
       <x:c r="G10" s="30" t="str">
-        <x:f>IF(V10&lt;&gt;"",V10,U10)</x:f>
         <x:v>support@frostking.com</x:v>
       </x:c>
       <x:c r="H10" s="30" t="str">
-        <x:f>IF(V10&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB10)),"API已验证","未验证"))</x:f>
-        <x:v>官网已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC10)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC10)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC10)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC10)),"判定无效",IF(V10&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>验证不确定</x:v>
       </x:c>
       <x:c r="I10" s="30" t="str">
-        <x:f>IF(X10&lt;&gt;"",X10,W10)</x:f>
-        <x:v>201-684-4400; 775-331-5291</x:v>
+        <x:v>+1 201-684-4400</x:v>
       </x:c>
       <x:c r="J10" s="30" t="str">
         <x:v>http://www.frostking.com/</x:v>
       </x:c>
       <x:c r="K10" s="35" t="n">
-        <x:f>ROUND((IF(G10&lt;&gt;"",40,0)+IF(I10&lt;&gt;"",25,0)+IF(J10&lt;&gt;"",20,0)+IF(Z10&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.85</x:v>
+        <x:f>ROUND((IF(H10="已验证有效",40,IF(V10&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y10)),25,0)+IF(J10&lt;&gt;"",20,0)+IF(AA10&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>0.65</x:v>
       </x:c>
       <x:c r="L10" s="30" t="str">
         <x:v>待联系</x:v>
@@ -1203,40 +1241,43 @@
       <x:c r="X10" s="30" t="str">
         <x:v>201-684-4400; 775-331-5291</x:v>
       </x:c>
-      <x:c r="Y10" s="30" t="str"/>
+      <x:c r="Y10" s="30" t="str">
+        <x:v>+1 201-684-4400:状态1/类型2/WhatsApp2; 201-684-4400:状态2/类型3/WhatsApp2; 775-331-5291:状态3/类型0/WhatsApp0</x:v>
+      </x:c>
       <x:c r="Z10" s="30" t="str"/>
-      <x:c r="AA10" s="30" t="str">
+      <x:c r="AA10" s="30" t="str"/>
+      <x:c r="AB10" s="30" t="str">
         <x:v>Official email and website inquiry form</x:v>
       </x:c>
-      <x:c r="AB10" s="30" t="str">
-        <x:v>support@frostking.com:0</x:v>
-      </x:c>
-      <x:c r="AC10" s="30" t="str"/>
-      <x:c r="AD10" s="30" t="str">
+      <x:c r="AC10" s="30" t="str">
+        <x:v>support@frostking.com:3</x:v>
+      </x:c>
+      <x:c r="AD10" s="30" t="str"/>
+      <x:c r="AE10" s="30" t="str">
         <x:v>plastic masking film</x:v>
       </x:c>
-      <x:c r="AE10" s="30" t="str">
+      <x:c r="AF10" s="30" t="str">
         <x:v>PLASTIC MASKING FILM,HS:392010&lt;br/&gt;</x:v>
       </x:c>
-      <x:c r="AF10" s="30" t="str"/>
       <x:c r="AG10" s="30" t="str"/>
       <x:c r="AH10" s="30" t="str"/>
-      <x:c r="AI10" s="30" t="str">
+      <x:c r="AI10" s="30" t="str"/>
+      <x:c r="AJ10" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ10" s="30" t="str">
+      <x:c r="AK10" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK10" s="30" t="str">
+      <x:c r="AL10" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL10" s="30" t="str">
+      <x:c r="AM10" s="30" t="str">
         <x:v>https://www.frostking.com/contact; https://www.frostking.com/accessibility-statement</x:v>
       </x:c>
-      <x:c r="AM10" s="30" t="str">
+      <x:c r="AN10" s="30" t="str">
         <x:v>Official accessibility page confirms support@frostking.com, matching the API email.</x:v>
       </x:c>
-      <x:c r="AN10" s="34" t="n">
+      <x:c r="AO10" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -1260,21 +1301,19 @@
         <x:v>US</x:v>
       </x:c>
       <x:c r="G11" s="30" t="str">
-        <x:f>IF(V11&lt;&gt;"",V11,U11)</x:f>
-        <x:v>csr1@tplogix.com; csr5@tplogix.com</x:v>
+        <x:v>csr1@tplogix.com</x:v>
       </x:c>
       <x:c r="H11" s="30" t="str">
-        <x:f>IF(V11&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB11)),"API已验证","未验证"))</x:f>
-        <x:v>官网已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC11)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC11)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC11)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC11)),"判定无效",IF(V11&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>验证不确定</x:v>
       </x:c>
       <x:c r="I11" s="30" t="str">
-        <x:f>IF(X11&lt;&gt;"",X11,W11)</x:f>
-        <x:v>562-474-8460</x:v>
+        <x:v>+1 562-474-8460</x:v>
       </x:c>
       <x:c r="J11" s="30" t="str"/>
       <x:c r="K11" s="35" t="n">
-        <x:f>ROUND((IF(G11&lt;&gt;"",40,0)+IF(I11&lt;&gt;"",25,0)+IF(J11&lt;&gt;"",20,0)+IF(Z11&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.65</x:v>
+        <x:f>ROUND((IF(H11="已验证有效",40,IF(V11&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y11)),25,0)+IF(J11&lt;&gt;"",20,0)+IF(AA11&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="L11" s="30" t="str">
         <x:v>待联系</x:v>
@@ -1311,38 +1350,41 @@
       <x:c r="X11" s="30" t="str">
         <x:v>562-474-8460</x:v>
       </x:c>
-      <x:c r="Y11" s="30" t="str"/>
+      <x:c r="Y11" s="30" t="str">
+        <x:v>+1 562-474-8460:状态1/类型3/WhatsApp2; 5624748460:状态3/类型0/WhatsApp0; 562-474-8460:状态2/类型3/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z11" s="30" t="str"/>
-      <x:c r="AA11" s="30" t="str">
+      <x:c r="AA11" s="30" t="str"/>
+      <x:c r="AB11" s="30" t="str">
         <x:v>Official customer-service emails, phone and inquiry form</x:v>
       </x:c>
-      <x:c r="AB11" s="30" t="str">
-        <x:v>r1@tplogix.com:0</x:v>
-      </x:c>
-      <x:c r="AC11" s="30" t="str"/>
+      <x:c r="AC11" s="30" t="str">
+        <x:v>r1@tplogix.com:2; csr1@tplogix.com:3; csr5@tplogix.com:3</x:v>
+      </x:c>
       <x:c r="AD11" s="30" t="str"/>
-      <x:c r="AE11" s="30" t="str">
+      <x:c r="AE11" s="30" t="str"/>
+      <x:c r="AF11" s="30" t="str">
         <x:v>MASKING FILM HBL BCOLO SCAC CODE BCPI ACI CODE W</x:v>
       </x:c>
-      <x:c r="AF11" s="30" t="str"/>
       <x:c r="AG11" s="30" t="str"/>
       <x:c r="AH11" s="30" t="str"/>
-      <x:c r="AI11" s="30" t="str">
+      <x:c r="AI11" s="30" t="str"/>
+      <x:c r="AJ11" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ11" s="30" t="str">
+      <x:c r="AK11" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK11" s="30" t="str">
+      <x:c r="AL11" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL11" s="30" t="str">
+      <x:c r="AM11" s="30" t="str">
         <x:v>https://tplogix.com/contact-us/</x:v>
       </x:c>
-      <x:c r="AM11" s="30" t="str">
+      <x:c r="AN11" s="30" t="str">
         <x:v>Official contact page provides two customer-service emails; use these ahead of the unverified API email.</x:v>
       </x:c>
-      <x:c r="AN11" s="34" t="n">
+      <x:c r="AO11" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -1366,22 +1408,20 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G12" s="30" t="str">
-        <x:f>IF(V12&lt;&gt;"",V12,U12)</x:f>
         <x:v>investorrelations@dixoninfo.com</x:v>
       </x:c>
       <x:c r="H12" s="30" t="str">
-        <x:f>IF(V12&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB12)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC12)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC12)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC12)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC12)),"判定无效",IF(V12&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I12" s="30" t="str">
-        <x:f>IF(X12&lt;&gt;"",X12,W12)</x:f>
         <x:v>+91 120 473 7200</x:v>
       </x:c>
       <x:c r="J12" s="30" t="str">
         <x:v>www.dixoninfo.com</x:v>
       </x:c>
       <x:c r="K12" s="35" t="n">
-        <x:f>ROUND((IF(G12&lt;&gt;"",40,0)+IF(I12&lt;&gt;"",25,0)+IF(J12&lt;&gt;"",20,0)+IF(Z12&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H12="已验证有效",40,IF(V12&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y12)),25,0)+IF(J12&lt;&gt;"",20,0)+IF(AA12&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="L12" s="30" t="str">
@@ -1413,44 +1453,47 @@
         <x:v>+91 120 473 7200</x:v>
       </x:c>
       <x:c r="X12" s="30" t="str"/>
-      <x:c r="Y12" s="30" t="str"/>
-      <x:c r="Z12" s="30" t="str">
+      <x:c r="Y12" s="30" t="str">
+        <x:v>+91 120 473 7200:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
+      <x:c r="Z12" s="30" t="str"/>
+      <x:c r="AA12" s="30" t="str">
         <x:v>https://www.linkedin.com/in/dixon-technologies-india-limited-625197186</x:v>
       </x:c>
-      <x:c r="AA12" s="30" t="str"/>
-      <x:c r="AB12" s="30" t="str">
+      <x:c r="AB12" s="30" t="str"/>
+      <x:c r="AC12" s="30" t="str">
         <x:v>investorrelations@dixoninfo.com:1</x:v>
       </x:c>
-      <x:c r="AC12" s="30" t="str">
+      <x:c r="AD12" s="30" t="str">
         <x:v>Rubber Tape; Parts for LED TV</x:v>
       </x:c>
-      <x:c r="AD12" s="30" t="str">
+      <x:c r="AE12" s="30" t="str">
         <x:v>Rubber; Tape; TPE; LED TV; Parts</x:v>
       </x:c>
-      <x:c r="AE12" s="30" t="str">
+      <x:c r="AF12" s="30" t="str">
         <x:v>RUBBER,TAPE,TPE,300X4.5X2,32,43,55DOTBL-0609-0000019-10-PARTS FOR LED TV-FOCPARTS FOR LED TV</x:v>
       </x:c>
-      <x:c r="AF12" s="30" t="str">
+      <x:c r="AG12" s="30" t="str">
         <x:v>Rubber Adhesive Tape; LED TV Accessories; TPE Tape; TV Parts; Rubber Strip</x:v>
       </x:c>
-      <x:c r="AG12" s="30" t="str">
+      <x:c r="AH12" s="30" t="str">
         <x:v>Rubber Resin; TPE Polymer; Plastic; Metal; Electronic Components</x:v>
       </x:c>
-      <x:c r="AH12" s="30" t="str">
+      <x:c r="AI12" s="30" t="str">
         <x:v>LED TVs; Monitor; Display Devices; Home Appliances; Consumer Electronics</x:v>
       </x:c>
-      <x:c r="AI12" s="30" t="str">
+      <x:c r="AJ12" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ12" s="30" t="str">
+      <x:c r="AK12" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK12" s="30" t="str">
+      <x:c r="AL12" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL12" s="30" t="str"/>
       <x:c r="AM12" s="30" t="str"/>
-      <x:c r="AN12" s="34" t="n">
+      <x:c r="AN12" s="30" t="str"/>
+      <x:c r="AO12" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -1474,22 +1517,20 @@
         <x:v>EC</x:v>
       </x:c>
       <x:c r="G13" s="30" t="str">
-        <x:f>IF(V13&lt;&gt;"",V13,U13)</x:f>
         <x:v>ccoque@grupolaar.com</x:v>
       </x:c>
       <x:c r="H13" s="30" t="str">
-        <x:f>IF(V13&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB13)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC13)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC13)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC13)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC13)),"判定无效",IF(V13&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I13" s="30" t="str">
-        <x:f>IF(X13&lt;&gt;"",X13,W13)</x:f>
         <x:v>+593 2-396-0000</x:v>
       </x:c>
       <x:c r="J13" s="30" t="str">
         <x:v>www.laarcourier.com</x:v>
       </x:c>
       <x:c r="K13" s="35" t="n">
-        <x:f>ROUND((IF(G13&lt;&gt;"",40,0)+IF(I13&lt;&gt;"",25,0)+IF(J13&lt;&gt;"",20,0)+IF(Z13&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H13="已验证有效",40,IF(V13&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y13)),25,0)+IF(J13&lt;&gt;"",20,0)+IF(AA13&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="L13" s="30" t="str">
@@ -1521,40 +1562,43 @@
         <x:v>+593 2-396-0000</x:v>
       </x:c>
       <x:c r="X13" s="30" t="str"/>
-      <x:c r="Y13" s="30" t="str"/>
+      <x:c r="Y13" s="30" t="str">
+        <x:v>+593 2-396-0000:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z13" s="30" t="str"/>
       <x:c r="AA13" s="30" t="str"/>
-      <x:c r="AB13" s="30" t="str">
+      <x:c r="AB13" s="30" t="str"/>
+      <x:c r="AC13" s="30" t="str">
         <x:v>ccoque@grupolaar.com:1</x:v>
       </x:c>
-      <x:c r="AC13" s="30" t="str"/>
-      <x:c r="AD13" s="30" t="str">
+      <x:c r="AD13" s="30" t="str"/>
+      <x:c r="AE13" s="30" t="str">
         <x:v>coffee maker; glove; bedspread; pressure transmitter</x:v>
       </x:c>
-      <x:c r="AE13" s="30" t="str">
+      <x:c r="AF13" s="30" t="str">
         <x:v>TWO-PIECE SWIMSUIT 35911615558 SOMBRERO DE COPA VACIO 10712856281 VESTIDO 9850584530 SOMBRERO DE COPA VACIO 89050573348 TWO-PIECE SWIMSUIT 4804392116 REPAIR TAPE 44363863818 LONG SLEEVE CREW NECK FOR</x:v>
       </x:c>
-      <x:c r="AF13" s="30" t="str"/>
       <x:c r="AG13" s="30" t="str"/>
       <x:c r="AH13" s="30" t="str"/>
-      <x:c r="AI13" s="30" t="str">
+      <x:c r="AI13" s="30" t="str"/>
+      <x:c r="AJ13" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ13" s="30" t="str">
+      <x:c r="AK13" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK13" s="30" t="str">
+      <x:c r="AL13" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL13" s="30" t="str"/>
       <x:c r="AM13" s="30" t="str"/>
-      <x:c r="AN13" s="34" t="n">
+      <x:c r="AN13" s="30" t="str"/>
+      <x:c r="AO13" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="44" customHeight="1">
       <x:c r="A14" s="30" t="str">
-        <x:v>API联系方式已获取</x:v>
+        <x:v>已补充有效决策人邮箱</x:v>
       </x:c>
       <x:c r="B14" s="30" t="str">
         <x:v>常规-全球</x:v>
@@ -1572,23 +1616,21 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G14" s="30" t="str">
-        <x:f>IF(V14&lt;&gt;"",V14,U14)</x:f>
-        <x:v>komal.neb@samsung.com</x:v>
+        <x:v>kiran.shindemumbai@gmail.com</x:v>
       </x:c>
       <x:c r="H14" s="30" t="str">
-        <x:f>IF(V14&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB14)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC14)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC14)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC14)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC14)),"判定无效",IF(V14&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I14" s="30" t="str">
-        <x:f>IF(X14&lt;&gt;"",X14,W14)</x:f>
         <x:v>+91 124 488 1234</x:v>
       </x:c>
       <x:c r="J14" s="30" t="str">
         <x:v>www.samsung.com/in</x:v>
       </x:c>
       <x:c r="K14" s="35" t="n">
-        <x:f>ROUND((IF(G14&lt;&gt;"",40,0)+IF(I14&lt;&gt;"",25,0)+IF(J14&lt;&gt;"",20,0)+IF(Z14&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.85</x:v>
+        <x:f>ROUND((IF(H14="已验证有效",40,IF(V14&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y14)),25,0)+IF(J14&lt;&gt;"",20,0)+IF(AA14&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L14" s="30" t="str">
         <x:v>待联系</x:v>
@@ -1614,39 +1656,46 @@
         <x:v>45868.666666666664</x:v>
       </x:c>
       <x:c r="U14" s="30" t="str">
-        <x:v>komal.neb@samsung.com</x:v>
+        <x:v>komal.neb@samsung.com; kiran.shindemumbai@gmail.com; kiranshindemumbai@gmail.com</x:v>
       </x:c>
       <x:c r="V14" s="30" t="str"/>
       <x:c r="W14" s="30" t="str">
         <x:v>+91 124 488 1234</x:v>
       </x:c>
       <x:c r="X14" s="30" t="str"/>
-      <x:c r="Y14" s="30" t="str"/>
+      <x:c r="Y14" s="30" t="str">
+        <x:v>+91 124 488 1234:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z14" s="30" t="str"/>
-      <x:c r="AA14" s="30" t="str"/>
-      <x:c r="AB14" s="30" t="str">
-        <x:v>komal.neb@samsung.com:0</x:v>
-      </x:c>
-      <x:c r="AC14" s="30" t="str"/>
+      <x:c r="AA14" s="30" t="str">
+        <x:v>https://www.linkedin.com/in/kiran-shinde-3a05091a</x:v>
+      </x:c>
+      <x:c r="AB14" s="30" t="str"/>
+      <x:c r="AC14" s="30" t="str">
+        <x:v>komal.neb@samsung.com:2; kiran.shindemumbai@gmail.com:1; kiranshindemumbai@gmail.com:1</x:v>
+      </x:c>
       <x:c r="AD14" s="30" t="str"/>
-      <x:c r="AE14" s="30" t="str">
+      <x:c r="AE14" s="30" t="str"/>
+      <x:c r="AF14" s="30" t="str">
         <x:v>TAPE-SINGLE FACE PAPER,T0.14,W75,L400M,B (0203-007500)(CEPANO:C020-25-0017622)TAPE-SINGLE FACE PAPER,T0.14,W75,L400M,B (0203-007500)(CEPA</x:v>
       </x:c>
-      <x:c r="AF14" s="30" t="str"/>
       <x:c r="AG14" s="30" t="str"/>
       <x:c r="AH14" s="30" t="str"/>
-      <x:c r="AI14" s="30" t="str">
+      <x:c r="AI14" s="30" t="str"/>
+      <x:c r="AJ14" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ14" s="30" t="str">
+      <x:c r="AK14" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK14" s="30" t="str">
-        <x:v>UpKuajing customs company contact API</x:v>
-      </x:c>
-      <x:c r="AL14" s="30" t="str"/>
+      <x:c r="AL14" s="30" t="str">
+        <x:v>UpKuajing customs company contact API; UpKuajing reviewed person contact API</x:v>
+      </x:c>
       <x:c r="AM14" s="30" t="str"/>
-      <x:c r="AN14" s="34" t="n">
+      <x:c r="AN14" s="30" t="str">
+        <x:v>人物补充：Kiran Shinde（Regional Distribution Manager）；供应链相关岗位，且公司匹配 Samsung India。</x:v>
+      </x:c>
+      <x:c r="AO14" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -1670,22 +1719,20 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G15" s="30" t="str">
-        <x:f>IF(V15&lt;&gt;"",V15,U15)</x:f>
-        <x:v>support.in@vivo.com; vcare@vivo.com</x:v>
+        <x:v>support.in@vivo.com</x:v>
       </x:c>
       <x:c r="H15" s="30" t="str">
-        <x:f>IF(V15&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB15)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC15)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC15)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC15)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC15)),"判定无效",IF(V15&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I15" s="30" t="str">
-        <x:f>IF(X15&lt;&gt;"",X15,W15)</x:f>
-        <x:v>01206283388; 18001023388; 18002083388; 18002084488; +91 120 628 3388</x:v>
+        <x:v>18002083388</x:v>
       </x:c>
       <x:c r="J15" s="30" t="str">
         <x:v>www.vivo.co.in</x:v>
       </x:c>
       <x:c r="K15" s="35" t="n">
-        <x:f>ROUND((IF(G15&lt;&gt;"",40,0)+IF(I15&lt;&gt;"",25,0)+IF(J15&lt;&gt;"",20,0)+IF(Z15&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H15="已验证有效",40,IF(V15&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y15)),25,0)+IF(J15&lt;&gt;"",20,0)+IF(AA15&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="L15" s="30" t="str">
@@ -1719,34 +1766,37 @@
         <x:v>01206283388; 18001023388; 18002083388; 18002084488; +91 120 628 3388</x:v>
       </x:c>
       <x:c r="X15" s="30" t="str"/>
-      <x:c r="Y15" s="30" t="str"/>
-      <x:c r="Z15" s="30" t="str">
+      <x:c r="Y15" s="30" t="str">
+        <x:v>01206283388:状态2/类型1/WhatsApp2; 18001023388:状态2/类型0/WhatsApp2; 18002083388:状态1/类型3/WhatsApp2; 18002084488:状态2/类型0/WhatsApp2; +91 120 628 3388:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
+      <x:c r="Z15" s="30" t="str"/>
+      <x:c r="AA15" s="30" t="str">
         <x:v>https://www.facebook.com/vivoIndia; https://www.instagram.com/accounts/login; https://www.linkedin.com/company/vivo-india; https://twitter.com/Vivo_India; https://www.youtube.com/c/VivoIndiaofficial</x:v>
       </x:c>
-      <x:c r="AA15" s="30" t="str"/>
-      <x:c r="AB15" s="30" t="str">
+      <x:c r="AB15" s="30" t="str"/>
+      <x:c r="AC15" s="30" t="str">
         <x:v>support.in@vivo.com:1; vcare@vivo.com:1</x:v>
       </x:c>
-      <x:c r="AC15" s="30" t="str"/>
       <x:c r="AD15" s="30" t="str"/>
-      <x:c r="AE15" s="30" t="str">
+      <x:c r="AE15" s="30" t="str"/>
+      <x:c r="AF15" s="30" t="str">
         <x:v>5181720 WATER CONTACT INDICATOR TAPE (PAPER) (PARTS FOR MFG.OF MOBILE PHONE)5181720 WATER CONTACT INDICATOR TAPE (PAPER) (PARTS FOR MFG.</x:v>
       </x:c>
-      <x:c r="AF15" s="30" t="str"/>
       <x:c r="AG15" s="30" t="str"/>
       <x:c r="AH15" s="30" t="str"/>
-      <x:c r="AI15" s="30" t="str">
+      <x:c r="AI15" s="30" t="str"/>
+      <x:c r="AJ15" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ15" s="30" t="str">
+      <x:c r="AK15" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK15" s="30" t="str">
+      <x:c r="AL15" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL15" s="30" t="str"/>
       <x:c r="AM15" s="30" t="str"/>
-      <x:c r="AN15" s="34" t="n">
+      <x:c r="AN15" s="30" t="str"/>
+      <x:c r="AO15" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -1770,21 +1820,18 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G16" s="30" t="str">
-        <x:f>IF(V16&lt;&gt;"",V16,U16)</x:f>
         <x:v>info@brandix.com</x:v>
       </x:c>
       <x:c r="H16" s="30" t="str">
-        <x:f>IF(V16&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB16)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
-      </x:c>
-      <x:c r="I16" s="30" t="str">
-        <x:f>IF(X16&lt;&gt;"",X16,W16)</x:f>
-      </x:c>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC16)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC16)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC16)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC16)),"判定无效",IF(V16&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
+      </x:c>
+      <x:c r="I16" s="30" t="str"/>
       <x:c r="J16" s="30" t="str">
         <x:v>www.brandix.com</x:v>
       </x:c>
       <x:c r="K16" s="35" t="n">
-        <x:f>ROUND((IF(G16&lt;&gt;"",40,0)+IF(I16&lt;&gt;"",25,0)+IF(J16&lt;&gt;"",20,0)+IF(Z16&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H16="已验证有效",40,IF(V16&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y16)),25,0)+IF(J16&lt;&gt;"",20,0)+IF(AA16&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="L16" s="30" t="str">
@@ -1819,31 +1866,32 @@
       <x:c r="Y16" s="30" t="str"/>
       <x:c r="Z16" s="30" t="str"/>
       <x:c r="AA16" s="30" t="str"/>
-      <x:c r="AB16" s="30" t="str">
+      <x:c r="AB16" s="30" t="str"/>
+      <x:c r="AC16" s="30" t="str">
         <x:v>info@brandix.com:1</x:v>
       </x:c>
-      <x:c r="AC16" s="30" t="str"/>
-      <x:c r="AD16" s="30" t="str">
+      <x:c r="AD16" s="30" t="str"/>
+      <x:c r="AE16" s="30" t="str">
         <x:v>fabric elastic; tape; narrow woven</x:v>
       </x:c>
-      <x:c r="AE16" s="30" t="str">
+      <x:c r="AF16" s="30" t="str">
         <x:v>NARROW WOVEN FABRIC ELASTIC TAPE 7000 MTRS BEL 8588023</x:v>
       </x:c>
-      <x:c r="AF16" s="30" t="str"/>
       <x:c r="AG16" s="30" t="str"/>
       <x:c r="AH16" s="30" t="str"/>
-      <x:c r="AI16" s="30" t="str">
+      <x:c r="AI16" s="30" t="str"/>
+      <x:c r="AJ16" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ16" s="30" t="str">
+      <x:c r="AK16" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK16" s="30" t="str">
+      <x:c r="AL16" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL16" s="30" t="str"/>
       <x:c r="AM16" s="30" t="str"/>
-      <x:c r="AN16" s="34" t="n">
+      <x:c r="AN16" s="30" t="str"/>
+      <x:c r="AO16" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -1867,20 +1915,19 @@
         <x:v>VN</x:v>
       </x:c>
       <x:c r="G17" s="30" t="str">
-        <x:f>IF(V17&lt;&gt;"",V17,U17)</x:f>
-        <x:v>hue.dt@honestcom.vn</x:v>
+        <x:v>hue.dt@honestvietnam.com.vn</x:v>
       </x:c>
       <x:c r="H17" s="30" t="str">
-        <x:f>IF(V17&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB17)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC17)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC17)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC17)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC17)),"判定无效",IF(V17&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>验证不确定</x:v>
       </x:c>
       <x:c r="I17" s="30" t="str">
-        <x:f>IF(X17&lt;&gt;"",X17,W17)</x:f>
+        <x:v>+84 24 3582 2456</x:v>
       </x:c>
       <x:c r="J17" s="30" t="str"/>
       <x:c r="K17" s="35" t="n">
-        <x:f>ROUND((IF(G17&lt;&gt;"",40,0)+IF(I17&lt;&gt;"",25,0)+IF(J17&lt;&gt;"",20,0)+IF(Z17&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.4</x:v>
+        <x:f>ROUND((IF(H17="已验证有效",40,IF(V17&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y17)),25,0)+IF(J17&lt;&gt;"",20,0)+IF(AA17&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="L17" s="30" t="str">
         <x:v>待联系</x:v>
@@ -1908,37 +1955,48 @@
       <x:c r="U17" s="30" t="str">
         <x:v>hue.dt@honestcom.vn</x:v>
       </x:c>
-      <x:c r="V17" s="30" t="str"/>
+      <x:c r="V17" s="30" t="str">
+        <x:v>hue.dt@honestvietnam.com.vn</x:v>
+      </x:c>
       <x:c r="W17" s="30" t="str"/>
-      <x:c r="X17" s="30" t="str"/>
-      <x:c r="Y17" s="30" t="str"/>
+      <x:c r="X17" s="30" t="str">
+        <x:v>+84 24 3582 2456</x:v>
+      </x:c>
+      <x:c r="Y17" s="30" t="str">
+        <x:v>+84 24 3582 2456:状态1/类型1/WhatsApp0</x:v>
+      </x:c>
       <x:c r="Z17" s="30" t="str"/>
       <x:c r="AA17" s="30" t="str"/>
-      <x:c r="AB17" s="30" t="str">
-        <x:v>hue.dt@honestcom.vn:0</x:v>
-      </x:c>
-      <x:c r="AC17" s="30" t="str"/>
-      <x:c r="AD17" s="30" t="str">
+      <x:c r="AB17" s="30" t="str"/>
+      <x:c r="AC17" s="30" t="str">
+        <x:v>hue.dt@honestcom.vn:2; hue.dt@honestvietnam.com.vn:3</x:v>
+      </x:c>
+      <x:c r="AD17" s="30" t="str"/>
+      <x:c r="AE17" s="30" t="str">
         <x:v>camshaft; adhesive tape</x:v>
       </x:c>
-      <x:c r="AE17" s="30" t="str">
+      <x:c r="AF17" s="30" t="str">
         <x:v>PS-1#&amp;Trục bằng thép</x:v>
       </x:c>
-      <x:c r="AF17" s="30" t="str"/>
       <x:c r="AG17" s="30" t="str"/>
       <x:c r="AH17" s="30" t="str"/>
-      <x:c r="AI17" s="30" t="str">
+      <x:c r="AI17" s="30" t="str"/>
+      <x:c r="AJ17" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ17" s="30" t="str">
+      <x:c r="AK17" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK17" s="30" t="str">
+      <x:c r="AL17" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL17" s="30" t="str"/>
-      <x:c r="AM17" s="30" t="str"/>
-      <x:c r="AN17" s="34" t="n">
+      <x:c r="AM17" s="30" t="str">
+        <x:v>https://www.hhtp.gov.vn/media/thong-bao-tuyen-dung/2025_07/2bao-cao-de-xuat-cap-lai-gpmt_compressed-1-389.pdf</x:v>
+      </x:c>
+      <x:c r="AN17" s="30" t="str">
+        <x:v>政府公开文件；2025 年企业环境许可文件列出的副总经理邮箱和公司电话 024 35822456。 验证状态=3。</x:v>
+      </x:c>
+      <x:c r="AO17" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -1962,22 +2020,20 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G18" s="30" t="str">
-        <x:f>IF(V18&lt;&gt;"",V18,U18)</x:f>
-        <x:v>info@genuselectrotech.com; sales@divicon.com</x:v>
+        <x:v>info@genuselectrotech.com</x:v>
       </x:c>
       <x:c r="H18" s="30" t="str">
-        <x:f>IF(V18&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB18)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC18)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC18)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC18)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC18)),"判定无效",IF(V18&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I18" s="30" t="str">
-        <x:f>IF(X18&lt;&gt;"",X18,W18)</x:f>
-        <x:v>+91 2836 240 872; +91 99789 59714; +91 99789 59735</x:v>
+        <x:v>+91 2836 240 872</x:v>
       </x:c>
       <x:c r="J18" s="30" t="str">
         <x:v>www.genuselectrotech.co.in</x:v>
       </x:c>
       <x:c r="K18" s="35" t="n">
-        <x:f>ROUND((IF(G18&lt;&gt;"",40,0)+IF(I18&lt;&gt;"",25,0)+IF(J18&lt;&gt;"",20,0)+IF(Z18&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H18="已验证有效",40,IF(V18&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y18)),25,0)+IF(J18&lt;&gt;"",20,0)+IF(AA18&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="L18" s="30" t="str">
@@ -2012,37 +2068,40 @@
       </x:c>
       <x:c r="X18" s="30" t="str"/>
       <x:c r="Y18" s="30" t="str">
+        <x:v>+91 2836 240 872:状态1/类型1/WhatsApp2; +91 99789 59714:状态1/类型2/WhatsApp1; +91 99789 59735:状态1/类型2/WhatsApp1</x:v>
+      </x:c>
+      <x:c r="Z18" s="30" t="str">
         <x:v>+91 99789 59714; +91 99789 59735</x:v>
       </x:c>
-      <x:c r="Z18" s="30" t="str">
+      <x:c r="AA18" s="30" t="str">
         <x:v>https://www.facebook.com/genuselectrotech10; https://www.instagram.com/genuselectrotechlimited; https://www.linkedin.com/company/genuselectrotechltd</x:v>
       </x:c>
-      <x:c r="AA18" s="30" t="str"/>
-      <x:c r="AB18" s="30" t="str">
-        <x:v>info@genuselectrotech.com:1; sales@divicon.com:0</x:v>
-      </x:c>
-      <x:c r="AC18" s="30" t="str"/>
-      <x:c r="AD18" s="30" t="str">
+      <x:c r="AB18" s="30" t="str"/>
+      <x:c r="AC18" s="30" t="str">
+        <x:v>info@genuselectrotech.com:1; sales@divicon.com:2</x:v>
+      </x:c>
+      <x:c r="AD18" s="30" t="str"/>
+      <x:c r="AE18" s="30" t="str">
         <x:v>fixture; ail; vhb tape</x:v>
       </x:c>
-      <x:c r="AE18" s="30" t="str">
+      <x:c r="AF18" s="30" t="str">
         <x:v>VHB TAPE PRESSURE HOLDING FIXTURE REST DETAILS AS PER INV &amp;PL VHB TAPE PRESSURE HOLDING FIXTURE REST DETAILS AS PER INV &amp;</x:v>
       </x:c>
-      <x:c r="AF18" s="30" t="str"/>
       <x:c r="AG18" s="30" t="str"/>
       <x:c r="AH18" s="30" t="str"/>
-      <x:c r="AI18" s="30" t="str">
+      <x:c r="AI18" s="30" t="str"/>
+      <x:c r="AJ18" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ18" s="30" t="str">
+      <x:c r="AK18" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK18" s="30" t="str">
+      <x:c r="AL18" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL18" s="30" t="str"/>
       <x:c r="AM18" s="30" t="str"/>
-      <x:c r="AN18" s="34" t="n">
+      <x:c r="AN18" s="30" t="str"/>
+      <x:c r="AO18" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -2066,21 +2125,19 @@
         <x:v>KR</x:v>
       </x:c>
       <x:c r="G19" s="30" t="str">
-        <x:f>IF(V19&lt;&gt;"",V19,U19)</x:f>
         <x:v>sim291@hanmail.net</x:v>
       </x:c>
       <x:c r="H19" s="30" t="str">
-        <x:f>IF(V19&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB19)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC19)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC19)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC19)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC19)),"判定无效",IF(V19&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>判定无效</x:v>
       </x:c>
       <x:c r="I19" s="30" t="str">
-        <x:f>IF(X19&lt;&gt;"",X19,W19)</x:f>
         <x:v>+82 51-266-7110</x:v>
       </x:c>
       <x:c r="J19" s="30" t="str"/>
       <x:c r="K19" s="35" t="n">
-        <x:f>ROUND((IF(G19&lt;&gt;"",40,0)+IF(I19&lt;&gt;"",25,0)+IF(J19&lt;&gt;"",20,0)+IF(Z19&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.65</x:v>
+        <x:f>ROUND((IF(H19="已验证有效",40,IF(V19&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y19)),25,0)+IF(J19&lt;&gt;"",20,0)+IF(AA19&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="L19" s="30" t="str">
         <x:v>待联系</x:v>
@@ -2113,34 +2170,37 @@
         <x:v>+82 51-266-7110</x:v>
       </x:c>
       <x:c r="X19" s="30" t="str"/>
-      <x:c r="Y19" s="30" t="str"/>
+      <x:c r="Y19" s="30" t="str">
+        <x:v>+82 51-266-7110:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z19" s="30" t="str"/>
       <x:c r="AA19" s="30" t="str"/>
-      <x:c r="AB19" s="30" t="str">
-        <x:v>sim291@hanmail.net:0</x:v>
-      </x:c>
-      <x:c r="AC19" s="30" t="str"/>
-      <x:c r="AD19" s="30" t="str">
+      <x:c r="AB19" s="30" t="str"/>
+      <x:c r="AC19" s="30" t="str">
+        <x:v>sim291@hanmail.net:2</x:v>
+      </x:c>
+      <x:c r="AD19" s="30" t="str"/>
+      <x:c r="AE19" s="30" t="str">
         <x:v>textile insulation tape</x:v>
       </x:c>
-      <x:c r="AE19" s="30" t="str">
+      <x:c r="AF19" s="30" t="str">
         <x:v>CLT-26-2037#&amp;Vải dệt đã cao su hóa 200MIC X 50MM X 25M #&amp;VN</x:v>
       </x:c>
-      <x:c r="AF19" s="30" t="str"/>
       <x:c r="AG19" s="30" t="str"/>
       <x:c r="AH19" s="30" t="str"/>
-      <x:c r="AI19" s="30" t="str">
+      <x:c r="AI19" s="30" t="str"/>
+      <x:c r="AJ19" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ19" s="30" t="str">
+      <x:c r="AK19" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK19" s="30" t="str">
+      <x:c r="AL19" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL19" s="30" t="str"/>
       <x:c r="AM19" s="30" t="str"/>
-      <x:c r="AN19" s="34" t="n">
+      <x:c r="AN19" s="30" t="str"/>
+      <x:c r="AO19" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -2164,20 +2224,18 @@
         <x:v>KR</x:v>
       </x:c>
       <x:c r="G20" s="30" t="str">
-        <x:f>IF(V20&lt;&gt;"",V20,U20)</x:f>
         <x:v>jworld@jworld21.com</x:v>
       </x:c>
       <x:c r="H20" s="30" t="str">
-        <x:f>IF(V20&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB20)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC20)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC20)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC20)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC20)),"判定无效",IF(V20&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I20" s="30" t="str">
-        <x:f>IF(X20&lt;&gt;"",X20,W20)</x:f>
         <x:v>+82 31-456-8001</x:v>
       </x:c>
       <x:c r="J20" s="30" t="str"/>
       <x:c r="K20" s="35" t="n">
-        <x:f>ROUND((IF(G20&lt;&gt;"",40,0)+IF(I20&lt;&gt;"",25,0)+IF(J20&lt;&gt;"",20,0)+IF(Z20&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H20="已验证有效",40,IF(V20&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y20)),25,0)+IF(J20&lt;&gt;"",20,0)+IF(AA20&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.65</x:v>
       </x:c>
       <x:c r="L20" s="30" t="str">
@@ -2211,34 +2269,37 @@
         <x:v>+82 31-456-8001</x:v>
       </x:c>
       <x:c r="X20" s="30" t="str"/>
-      <x:c r="Y20" s="30" t="str"/>
+      <x:c r="Y20" s="30" t="str">
+        <x:v>+82 31-456-8001:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z20" s="30" t="str"/>
       <x:c r="AA20" s="30" t="str"/>
-      <x:c r="AB20" s="30" t="str">
+      <x:c r="AB20" s="30" t="str"/>
+      <x:c r="AC20" s="30" t="str">
         <x:v>jworld@jworld21.com:1</x:v>
       </x:c>
-      <x:c r="AC20" s="30" t="str"/>
-      <x:c r="AD20" s="30" t="str">
+      <x:c r="AD20" s="30" t="str"/>
+      <x:c r="AE20" s="30" t="str">
         <x:v>deco film</x:v>
       </x:c>
-      <x:c r="AE20" s="30" t="str">
+      <x:c r="AF20" s="30" t="str">
         <x:v>RNDT09754#&amp;Băng dính dùng cho điện thoại di động TAPE WP SUB UB 3SIDE VH301_0219 kích thước 78.73*71.37 mm*mm#&amp;VN</x:v>
       </x:c>
-      <x:c r="AF20" s="30" t="str"/>
       <x:c r="AG20" s="30" t="str"/>
       <x:c r="AH20" s="30" t="str"/>
-      <x:c r="AI20" s="30" t="str">
+      <x:c r="AI20" s="30" t="str"/>
+      <x:c r="AJ20" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ20" s="30" t="str">
+      <x:c r="AK20" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK20" s="30" t="str">
+      <x:c r="AL20" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL20" s="30" t="str"/>
       <x:c r="AM20" s="30" t="str"/>
-      <x:c r="AN20" s="34" t="n">
+      <x:c r="AN20" s="30" t="str"/>
+      <x:c r="AO20" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -2262,23 +2323,21 @@
         <x:v>MX</x:v>
       </x:c>
       <x:c r="G21" s="30" t="str">
-        <x:f>IF(V21&lt;&gt;"",V21,U21)</x:f>
         <x:v>privacidad@suzuki.com.mx</x:v>
       </x:c>
       <x:c r="H21" s="30" t="str">
-        <x:f>IF(V21&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB21)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC21)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC21)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC21)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC21)),"判定无效",IF(V21&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>判定无效</x:v>
       </x:c>
       <x:c r="I21" s="30" t="str">
-        <x:f>IF(X21&lt;&gt;"",X21,W21)</x:f>
         <x:v>+52 55 5365 2626</x:v>
       </x:c>
       <x:c r="J21" s="30" t="str">
         <x:v>http://www.suzuki.com.mx/</x:v>
       </x:c>
       <x:c r="K21" s="35" t="n">
-        <x:f>ROUND((IF(G21&lt;&gt;"",40,0)+IF(I21&lt;&gt;"",25,0)+IF(J21&lt;&gt;"",20,0)+IF(Z21&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.85</x:v>
+        <x:f>ROUND((IF(H21="已验证有效",40,IF(V21&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y21)),25,0)+IF(J21&lt;&gt;"",20,0)+IF(AA21&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="L21" s="30" t="str">
         <x:v>待联系</x:v>
@@ -2311,40 +2370,43 @@
         <x:v>+52 55 5365 2626</x:v>
       </x:c>
       <x:c r="X21" s="30" t="str"/>
-      <x:c r="Y21" s="30" t="str"/>
+      <x:c r="Y21" s="30" t="str">
+        <x:v>+52 55 5365 2626:状态1/类型3/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z21" s="30" t="str"/>
       <x:c r="AA21" s="30" t="str"/>
-      <x:c r="AB21" s="30" t="str">
-        <x:v>privacidad@suzuki.com.mx:0</x:v>
-      </x:c>
-      <x:c r="AC21" s="30" t="str"/>
-      <x:c r="AD21" s="30" t="str">
+      <x:c r="AB21" s="30" t="str"/>
+      <x:c r="AC21" s="30" t="str">
+        <x:v>privacidad@suzuki.com.mx:2</x:v>
+      </x:c>
+      <x:c r="AD21" s="30" t="str"/>
+      <x:c r="AE21" s="30" t="str">
         <x:v>green tape; yellow ribbon</x:v>
       </x:c>
-      <x:c r="AE21" s="30" t="str">
+      <x:c r="AF21" s="30" t="str">
         <x:v>CINTA COD 83926 54P10 0CE</x:v>
       </x:c>
-      <x:c r="AF21" s="30" t="str"/>
       <x:c r="AG21" s="30" t="str"/>
       <x:c r="AH21" s="30" t="str"/>
-      <x:c r="AI21" s="30" t="str">
+      <x:c r="AI21" s="30" t="str"/>
+      <x:c r="AJ21" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ21" s="30" t="str">
+      <x:c r="AK21" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK21" s="30" t="str">
+      <x:c r="AL21" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL21" s="30" t="str"/>
       <x:c r="AM21" s="30" t="str"/>
-      <x:c r="AN21" s="34" t="n">
+      <x:c r="AN21" s="30" t="str"/>
+      <x:c r="AO21" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="44" customHeight="1">
       <x:c r="A22" s="30" t="str">
-        <x:v>API联系方式已获取</x:v>
+        <x:v>已补充有效决策人邮箱</x:v>
       </x:c>
       <x:c r="B22" s="30" t="str">
         <x:v>常规-全球</x:v>
@@ -2362,22 +2424,21 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G22" s="30" t="str">
-        <x:f>IF(V22&lt;&gt;"",V22,U22)</x:f>
-        <x:v>info@haierindia.com</x:v>
+        <x:v>chuktiii@gmail.com</x:v>
       </x:c>
       <x:c r="H22" s="30" t="str">
-        <x:f>IF(V22&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB22)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC22)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC22)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC22)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC22)),"判定无效",IF(V22&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I22" s="30" t="str">
-        <x:f>IF(X22&lt;&gt;"",X22,W22)</x:f>
+        <x:v>+91 1800 419 9999</x:v>
       </x:c>
       <x:c r="J22" s="30" t="str">
         <x:v>www.haier.com</x:v>
       </x:c>
       <x:c r="K22" s="35" t="n">
-        <x:f>ROUND((IF(G22&lt;&gt;"",40,0)+IF(I22&lt;&gt;"",25,0)+IF(J22&lt;&gt;"",20,0)+IF(Z22&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.6</x:v>
+        <x:f>ROUND((IF(H22="已验证有效",40,IF(V22&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y22)),25,0)+IF(J22&lt;&gt;"",20,0)+IF(AA22&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L22" s="30" t="str">
         <x:v>待联系</x:v>
@@ -2403,39 +2464,54 @@
         <x:v>45655.666666666664</x:v>
       </x:c>
       <x:c r="U22" s="30" t="str">
-        <x:v>info@haierindia.com</x:v>
-      </x:c>
-      <x:c r="V22" s="30" t="str"/>
+        <x:v>info@haierindia.com; chuktiii@gmail.com</x:v>
+      </x:c>
+      <x:c r="V22" s="30" t="str">
+        <x:v>customercare@haierindia.com</x:v>
+      </x:c>
       <x:c r="W22" s="30" t="str"/>
-      <x:c r="X22" s="30" t="str"/>
-      <x:c r="Y22" s="30" t="str"/>
-      <x:c r="Z22" s="30" t="str"/>
-      <x:c r="AA22" s="30" t="str"/>
-      <x:c r="AB22" s="30" t="str">
-        <x:v>info@haierindia.com:0</x:v>
-      </x:c>
-      <x:c r="AC22" s="30" t="str"/>
-      <x:c r="AD22" s="30" t="str">
+      <x:c r="X22" s="30" t="str">
+        <x:v>+91 1800 419 9999; +91 1800 102 9999</x:v>
+      </x:c>
+      <x:c r="Y22" s="30" t="str">
+        <x:v>+91 1800 419 9999:状态1/类型3/WhatsApp2; +91 1800 102 9999:状态3/类型0/WhatsApp0</x:v>
+      </x:c>
+      <x:c r="Z22" s="30" t="str">
+        <x:v>+91 85530 49999</x:v>
+      </x:c>
+      <x:c r="AA22" s="30" t="str">
+        <x:v>https://www.linkedin.com/in/madhumay-panigrahi-528ab842; https://www.facebook.com/madhumay.panigrahi</x:v>
+      </x:c>
+      <x:c r="AB22" s="30" t="str"/>
+      <x:c r="AC22" s="30" t="str">
+        <x:v>info@haierindia.com:3; chuktiii@gmail.com:1; customercare@haierindia.com:3</x:v>
+      </x:c>
+      <x:c r="AD22" s="30" t="str"/>
+      <x:c r="AE22" s="30" t="str">
         <x:v>packing tap; t code; e 80; x7; model; assembly component</x:v>
       </x:c>
-      <x:c r="AE22" s="30" t="str">
+      <x:c r="AF22" s="30" t="str">
         <x:v>PACKING TAPE 800MX72X0.045MM 50P7GT-P PART CODE: 0090303389MODEL NO 50P7GT-P (ASSEMBLY COMPONENT)PACKING TAPE 800MX72X0.045MM 50P7GT-P PART CODE: 0090303389</x:v>
       </x:c>
-      <x:c r="AF22" s="30" t="str"/>
       <x:c r="AG22" s="30" t="str"/>
       <x:c r="AH22" s="30" t="str"/>
-      <x:c r="AI22" s="30" t="str">
+      <x:c r="AI22" s="30" t="str"/>
+      <x:c r="AJ22" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ22" s="30" t="str">
+      <x:c r="AK22" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK22" s="30" t="str">
-        <x:v>UpKuajing customs company contact API</x:v>
-      </x:c>
-      <x:c r="AL22" s="30" t="str"/>
-      <x:c r="AM22" s="30" t="str"/>
-      <x:c r="AN22" s="34" t="n">
+      <x:c r="AL22" s="30" t="str">
+        <x:v>UpKuajing customs company contact API; UpKuajing reviewed person contact API</x:v>
+      </x:c>
+      <x:c r="AM22" s="30" t="str">
+        <x:v>https://www.haier.com/in/blogs/hassle-free-installation-and-service-support-for-haier-led-tvs-in-india.shtml</x:v>
+      </x:c>
+      <x:c r="AN22" s="30" t="str">
+        <x:v>企业官网；Haier India 官网公布的客服邮箱；同时公布电话 1800-419-9999、1800-102-9999 和 WhatsApp 8553049999。 验证状态=3。; 人物补充：Madhumay Panigrahi（Branch Logistics Manager）；物流岗位，且公司精确匹配 Haier India。 排除 madhumay.panigrahi@havells.com：邮箱域名属于 Havells，与当前 Haier 实体不一致</x:v>
+      </x:c>
+      <x:c r="AO22" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -2459,21 +2535,18 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G23" s="30" t="str">
-        <x:f>IF(V23&lt;&gt;"",V23,U23)</x:f>
         <x:v>murugan.selvaraj@triumph.com</x:v>
       </x:c>
       <x:c r="H23" s="30" t="str">
-        <x:f>IF(V23&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB23)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
-      </x:c>
-      <x:c r="I23" s="30" t="str">
-        <x:f>IF(X23&lt;&gt;"",X23,W23)</x:f>
-      </x:c>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC23)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC23)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC23)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC23)),"判定无效",IF(V23&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
+      </x:c>
+      <x:c r="I23" s="30" t="str"/>
       <x:c r="J23" s="30" t="str">
         <x:v>www.triumph.com</x:v>
       </x:c>
       <x:c r="K23" s="35" t="n">
-        <x:f>ROUND((IF(G23&lt;&gt;"",40,0)+IF(I23&lt;&gt;"",25,0)+IF(J23&lt;&gt;"",20,0)+IF(Z23&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H23="已验证有效",40,IF(V23&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y23)),25,0)+IF(J23&lt;&gt;"",20,0)+IF(AA23&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="L23" s="30" t="str">
@@ -2508,29 +2581,30 @@
       <x:c r="Y23" s="30" t="str"/>
       <x:c r="Z23" s="30" t="str"/>
       <x:c r="AA23" s="30" t="str"/>
-      <x:c r="AB23" s="30" t="str">
+      <x:c r="AB23" s="30" t="str"/>
+      <x:c r="AC23" s="30" t="str">
         <x:v>murugan.selvaraj@triumph.com:1</x:v>
       </x:c>
-      <x:c r="AC23" s="30" t="str"/>
       <x:c r="AD23" s="30" t="str"/>
-      <x:c r="AE23" s="30" t="str">
+      <x:c r="AE23" s="30" t="str"/>
+      <x:c r="AF23" s="30" t="str">
         <x:v>ITEM 3329/22 COLOR OP3701-ELASTIC TAPE ITEM 3329/22 COLOR OP3701</x:v>
       </x:c>
-      <x:c r="AF23" s="30" t="str"/>
       <x:c r="AG23" s="30" t="str"/>
       <x:c r="AH23" s="30" t="str"/>
-      <x:c r="AI23" s="30" t="str">
+      <x:c r="AI23" s="30" t="str"/>
+      <x:c r="AJ23" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ23" s="30" t="str">
+      <x:c r="AK23" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK23" s="30" t="str">
+      <x:c r="AL23" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL23" s="30" t="str"/>
       <x:c r="AM23" s="30" t="str"/>
-      <x:c r="AN23" s="34" t="n">
+      <x:c r="AN23" s="30" t="str"/>
+      <x:c r="AO23" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -2554,22 +2628,20 @@
         <x:v>VN</x:v>
       </x:c>
       <x:c r="G24" s="30" t="str">
-        <x:f>IF(V24&lt;&gt;"",V24,U24)</x:f>
-        <x:v>admin@asti.com.vn; info@asti.com</x:v>
+        <x:v>admin@asti.com.vn</x:v>
       </x:c>
       <x:c r="H24" s="30" t="str">
-        <x:f>IF(V24&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB24)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC24)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC24)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC24)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC24)),"判定无效",IF(V24&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I24" s="30" t="str">
-        <x:f>IF(X24&lt;&gt;"",X24,W24)</x:f>
-        <x:v>+84 274 2742 464; +84 274 3742 464; +84 274 3742 594; 84274742464</x:v>
+        <x:v>+84 274 2742 464</x:v>
       </x:c>
       <x:c r="J24" s="30" t="str">
         <x:v>www.asti.com.vn</x:v>
       </x:c>
       <x:c r="K24" s="35" t="n">
-        <x:f>ROUND((IF(G24&lt;&gt;"",40,0)+IF(I24&lt;&gt;"",25,0)+IF(J24&lt;&gt;"",20,0)+IF(Z24&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H24="已验证有效",40,IF(V24&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y24)),25,0)+IF(J24&lt;&gt;"",20,0)+IF(AA24&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="L24" s="30" t="str">
@@ -2601,32 +2673,35 @@
         <x:v>+84 274 2742 464; +84 274 3742 464; +84 274 3742 594; 84274742464</x:v>
       </x:c>
       <x:c r="X24" s="30" t="str"/>
-      <x:c r="Y24" s="30" t="str"/>
+      <x:c r="Y24" s="30" t="str">
+        <x:v>+84 274 2742 464:状态1/类型1/WhatsApp2; +84 274 3742 464:状态1/类型1/WhatsApp2; +84 274 3742 594:状态1/类型1/WhatsApp2; 84274742464:状态2/类型3/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z24" s="30" t="str"/>
       <x:c r="AA24" s="30" t="str"/>
-      <x:c r="AB24" s="30" t="str">
+      <x:c r="AB24" s="30" t="str"/>
+      <x:c r="AC24" s="30" t="str">
         <x:v>admin@asti.com.vn:1; info@asti.com:1</x:v>
       </x:c>
-      <x:c r="AC24" s="30" t="str"/>
       <x:c r="AD24" s="30" t="str"/>
-      <x:c r="AE24" s="30" t="str">
+      <x:c r="AE24" s="30" t="str"/>
+      <x:c r="AF24" s="30" t="str">
         <x:v>A003BK#&amp;amp;Tape glue for cluster conductor electric motorcycle (Tape) 0.1X19X25:BLACK, 100% brand new</x:v>
       </x:c>
-      <x:c r="AF24" s="30" t="str"/>
       <x:c r="AG24" s="30" t="str"/>
       <x:c r="AH24" s="30" t="str"/>
-      <x:c r="AI24" s="30" t="str">
+      <x:c r="AI24" s="30" t="str"/>
+      <x:c r="AJ24" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ24" s="30" t="str">
+      <x:c r="AK24" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK24" s="30" t="str">
+      <x:c r="AL24" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL24" s="30" t="str"/>
       <x:c r="AM24" s="30" t="str"/>
-      <x:c r="AN24" s="34" t="n">
+      <x:c r="AN24" s="30" t="str"/>
+      <x:c r="AO24" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -2650,22 +2725,20 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G25" s="30" t="str">
-        <x:f>IF(V25&lt;&gt;"",V25,U25)</x:f>
         <x:v>info.india@triumph.com</x:v>
       </x:c>
       <x:c r="H25" s="30" t="str">
-        <x:f>IF(V25&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB25)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC25)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC25)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC25)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC25)),"判定无效",IF(V25&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I25" s="30" t="str">
-        <x:f>IF(X25&lt;&gt;"",X25,W25)</x:f>
         <x:v>+91 44 2842 0743</x:v>
       </x:c>
       <x:c r="J25" s="30" t="str">
         <x:v>http://www.triumph.com</x:v>
       </x:c>
       <x:c r="K25" s="35" t="n">
-        <x:f>ROUND((IF(G25&lt;&gt;"",40,0)+IF(I25&lt;&gt;"",25,0)+IF(J25&lt;&gt;"",20,0)+IF(Z25&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H25="已验证有效",40,IF(V25&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y25)),25,0)+IF(J25&lt;&gt;"",20,0)+IF(AA25&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="L25" s="30" t="str">
@@ -2699,34 +2772,37 @@
         <x:v>+91 44 2842 0743</x:v>
       </x:c>
       <x:c r="X25" s="30" t="str"/>
-      <x:c r="Y25" s="30" t="str"/>
+      <x:c r="Y25" s="30" t="str">
+        <x:v>+91 44 2842 0743:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z25" s="30" t="str"/>
       <x:c r="AA25" s="30" t="str"/>
-      <x:c r="AB25" s="30" t="str">
+      <x:c r="AB25" s="30" t="str"/>
+      <x:c r="AC25" s="30" t="str">
         <x:v>info.india@triumph.com:1</x:v>
       </x:c>
-      <x:c r="AC25" s="30" t="str"/>
-      <x:c r="AD25" s="30" t="str">
+      <x:c r="AD25" s="30" t="str"/>
+      <x:c r="AE25" s="30" t="str">
         <x:v>eye tape; pearl</x:v>
       </x:c>
-      <x:c r="AE25" s="30" t="str">
+      <x:c r="AF25" s="30" t="str">
         <x:v>PRECUT EYE TAPE 000 S0182S 38MM A PEARL GR 38198 PO 4512863360 12863362PRECUT EYE TAPE</x:v>
       </x:c>
-      <x:c r="AF25" s="30" t="str"/>
       <x:c r="AG25" s="30" t="str"/>
       <x:c r="AH25" s="30" t="str"/>
-      <x:c r="AI25" s="30" t="str">
+      <x:c r="AI25" s="30" t="str"/>
+      <x:c r="AJ25" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ25" s="30" t="str">
+      <x:c r="AK25" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK25" s="30" t="str">
+      <x:c r="AL25" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL25" s="30" t="str"/>
       <x:c r="AM25" s="30" t="str"/>
-      <x:c r="AN25" s="34" t="n">
+      <x:c r="AN25" s="30" t="str"/>
+      <x:c r="AO25" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -2750,21 +2826,19 @@
         <x:v>KR</x:v>
       </x:c>
       <x:c r="G26" s="30" t="str">
-        <x:f>IF(V26&lt;&gt;"",V26,U26)</x:f>
         <x:v>cosmotech@korea.com</x:v>
       </x:c>
       <x:c r="H26" s="30" t="str">
-        <x:f>IF(V26&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB26)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC26)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC26)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC26)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC26)),"判定无效",IF(V26&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>验证不确定</x:v>
       </x:c>
       <x:c r="I26" s="30" t="str">
-        <x:f>IF(X26&lt;&gt;"",X26,W26)</x:f>
         <x:v>+82 32-817-6552</x:v>
       </x:c>
       <x:c r="J26" s="30" t="str"/>
       <x:c r="K26" s="35" t="n">
-        <x:f>ROUND((IF(G26&lt;&gt;"",40,0)+IF(I26&lt;&gt;"",25,0)+IF(J26&lt;&gt;"",20,0)+IF(Z26&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.65</x:v>
+        <x:f>ROUND((IF(H26="已验证有效",40,IF(V26&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y26)),25,0)+IF(J26&lt;&gt;"",20,0)+IF(AA26&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="L26" s="30" t="str">
         <x:v>待联系</x:v>
@@ -2797,42 +2871,45 @@
         <x:v>+82 32-817-6552</x:v>
       </x:c>
       <x:c r="X26" s="30" t="str"/>
-      <x:c r="Y26" s="30" t="str"/>
+      <x:c r="Y26" s="30" t="str">
+        <x:v>+82 32-817-6552:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z26" s="30" t="str"/>
       <x:c r="AA26" s="30" t="str"/>
-      <x:c r="AB26" s="30" t="str">
-        <x:v>cosmotech@korea.com:0</x:v>
-      </x:c>
+      <x:c r="AB26" s="30" t="str"/>
       <x:c r="AC26" s="30" t="str">
+        <x:v>cosmotech@korea.com:3</x:v>
+      </x:c>
+      <x:c r="AD26" s="30" t="str">
         <x:v>TAPE-1 P1 DUO</x:v>
       </x:c>
-      <x:c r="AD26" s="30" t="str">
+      <x:c r="AE26" s="30" t="str">
         <x:v>tape; plastic; self - adhesive; recycled</x:v>
       </x:c>
-      <x:c r="AE26" s="30" t="str">
+      <x:c r="AF26" s="30" t="str">
         <x:v>TAPE-1 P1 DUO#&amp;Miếng plastic tự dán TAPE-1 P1 DUO (TOP TAPE TESA61885), kt 120.08*12.50mm, hàng mới 100% tái xuất mục 44 TK 107230146220#&amp;KR</x:v>
       </x:c>
-      <x:c r="AF26" s="30" t="str">
+      <x:c r="AG26" s="30" t="str">
         <x:v>Adhesive tape; Self - sticking tape; Plastic tape; Duo tape; TESA tape</x:v>
       </x:c>
-      <x:c r="AG26" s="30" t="str">
+      <x:c r="AH26" s="30" t="str">
         <x:v>Plastic resin; Adhesive; Polymer; Additives; Recycled plastic</x:v>
       </x:c>
-      <x:c r="AH26" s="30" t="str">
+      <x:c r="AI26" s="30" t="str">
         <x:v>Packaging; Labeling; Crafts; Electronics assembly; Office use</x:v>
       </x:c>
-      <x:c r="AI26" s="30" t="str">
+      <x:c r="AJ26" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ26" s="30" t="str">
+      <x:c r="AK26" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK26" s="30" t="str">
+      <x:c r="AL26" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL26" s="30" t="str"/>
       <x:c r="AM26" s="30" t="str"/>
-      <x:c r="AN26" s="34" t="n">
+      <x:c r="AN26" s="30" t="str"/>
+      <x:c r="AO26" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -2856,22 +2933,20 @@
         <x:v>KR</x:v>
       </x:c>
       <x:c r="G27" s="30" t="str">
-        <x:f>IF(V27&lt;&gt;"",V27,U27)</x:f>
         <x:v>annapark@hansoll.com</x:v>
       </x:c>
       <x:c r="H27" s="30" t="str">
-        <x:f>IF(V27&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB27)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC27)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC27)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC27)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC27)),"判定无效",IF(V27&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I27" s="30" t="str">
-        <x:f>IF(X27&lt;&gt;"",X27,W27)</x:f>
         <x:v>+1 212-764-4270</x:v>
       </x:c>
       <x:c r="J27" s="30" t="str">
         <x:v>http://www.hansoll.com/</x:v>
       </x:c>
       <x:c r="K27" s="35" t="n">
-        <x:f>ROUND((IF(G27&lt;&gt;"",40,0)+IF(I27&lt;&gt;"",25,0)+IF(J27&lt;&gt;"",20,0)+IF(Z27&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H27="已验证有效",40,IF(V27&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y27)),25,0)+IF(J27&lt;&gt;"",20,0)+IF(AA27&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="L27" s="30" t="str">
@@ -2905,34 +2980,37 @@
         <x:v>+1 212-764-4270</x:v>
       </x:c>
       <x:c r="X27" s="30" t="str"/>
-      <x:c r="Y27" s="30" t="str"/>
+      <x:c r="Y27" s="30" t="str">
+        <x:v>+1 212-764-4270:状态1/类型3/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z27" s="30" t="str"/>
       <x:c r="AA27" s="30" t="str"/>
-      <x:c r="AB27" s="30" t="str">
+      <x:c r="AB27" s="30" t="str"/>
+      <x:c r="AC27" s="30" t="str">
         <x:v>annapark@hansoll.com:1</x:v>
       </x:c>
-      <x:c r="AC27" s="30" t="str"/>
-      <x:c r="AD27" s="30" t="str">
+      <x:c r="AD27" s="30" t="str"/>
+      <x:c r="AE27" s="30" t="str">
         <x:v>accessories of plastics</x:v>
       </x:c>
-      <x:c r="AE27" s="30" t="str">
+      <x:c r="AF27" s="30" t="str">
         <x:v>DÂY CHỐNG DÃN 0608 (MOBILON TAPE SHL-0608; DÂY VIỀN 0608; Kích thước: 6 MM x 0.08 MM; 826,491.41 MÉT; SỬ DỤNG TRONG MAY MẶC; CHẤT LIỆU: POLYURE THANE; HÀNG MỚI 100%)#&amp;KR</x:v>
       </x:c>
-      <x:c r="AF27" s="30" t="str"/>
       <x:c r="AG27" s="30" t="str"/>
       <x:c r="AH27" s="30" t="str"/>
-      <x:c r="AI27" s="30" t="str">
+      <x:c r="AI27" s="30" t="str"/>
+      <x:c r="AJ27" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ27" s="30" t="str">
+      <x:c r="AK27" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK27" s="30" t="str">
+      <x:c r="AL27" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL27" s="30" t="str"/>
       <x:c r="AM27" s="30" t="str"/>
-      <x:c r="AN27" s="34" t="n">
+      <x:c r="AN27" s="30" t="str"/>
+      <x:c r="AO27" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -2956,22 +3034,20 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G28" s="30" t="str">
-        <x:f>IF(V28&lt;&gt;"",V28,U28)</x:f>
-        <x:v>marketing@ajitindustries.com; suneet@ajitindustries.com</x:v>
+        <x:v>marketing@ajitindustries.com</x:v>
       </x:c>
       <x:c r="H28" s="30" t="str">
-        <x:f>IF(V28&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB28)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC28)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC28)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC28)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC28)),"判定无效",IF(V28&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I28" s="30" t="str">
-        <x:f>IF(X28&lt;&gt;"",X28,W28)</x:f>
-        <x:v>01149010101; +91 80 6882 0110; +91 82879 48064; +91 95996 77993</x:v>
+        <x:v>+91 80 6882 0110</x:v>
       </x:c>
       <x:c r="J28" s="30" t="str">
         <x:v>www.ajitindustries.com</x:v>
       </x:c>
       <x:c r="K28" s="35" t="n">
-        <x:f>ROUND((IF(G28&lt;&gt;"",40,0)+IF(I28&lt;&gt;"",25,0)+IF(J28&lt;&gt;"",20,0)+IF(Z28&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H28="已验证有效",40,IF(V28&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y28)),25,0)+IF(J28&lt;&gt;"",20,0)+IF(AA28&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="L28" s="30" t="str">
@@ -3004,51 +3080,54 @@
       </x:c>
       <x:c r="X28" s="30" t="str"/>
       <x:c r="Y28" s="30" t="str">
+        <x:v>01149010101:状态2/类型0/WhatsApp0; +91 80 6882 0110:状态1/类型1/WhatsApp2; +91 82879 48064:状态1/类型2/WhatsApp1; +91 95996 77993:状态1/类型2/WhatsApp1</x:v>
+      </x:c>
+      <x:c r="Z28" s="30" t="str">
         <x:v>+91 82879 48064; +91 95996 77993</x:v>
       </x:c>
-      <x:c r="Z28" s="30" t="str">
+      <x:c r="AA28" s="30" t="str">
         <x:v>https://www.youtube.com/watch?v=TUJvH6kYIWE</x:v>
       </x:c>
-      <x:c r="AA28" s="30" t="str"/>
-      <x:c r="AB28" s="30" t="str">
+      <x:c r="AB28" s="30" t="str"/>
+      <x:c r="AC28" s="30" t="str">
         <x:v>marketing@ajitindustries.com:1; suneet@ajitindustries.com:1</x:v>
       </x:c>
-      <x:c r="AC28" s="30" t="str">
+      <x:c r="AD28" s="30" t="str">
         <x:v>PE Masking Film</x:v>
       </x:c>
-      <x:c r="AD28" s="30" t="str">
+      <x:c r="AE28" s="30" t="str">
         <x:v>PE; Masking film; Industrial use</x:v>
       </x:c>
-      <x:c r="AE28" s="30" t="str">
+      <x:c r="AF28" s="30" t="str">
         <x:v>MASKING TAPE (IN JUMBO ROLLS)PRODUCT CODE:770UU;COLOR:BEIGE;SIZE:1570mm x 2000m (RLS:53)(PIMS NO:ORIGINAL DPIIT-PPR-2025MASKING TAPE (IN JUMBO ROLLS)PRODUCT CODE:770UU;COLOR:BEIGE;; PE MASKING FILM IN LARGE ROLL SIZE: 2700MM*1600M (ROLL 600)(FOR INDUSTRIAL USE)PE MASKING FILM IN</x:v>
       </x:c>
-      <x:c r="AF28" s="30" t="str">
+      <x:c r="AG28" s="30" t="str">
         <x:v>PE protective film; PE masking tape; Polyethylene masking film; Industrial masking film; PE covering film</x:v>
       </x:c>
-      <x:c r="AG28" s="30" t="str">
+      <x:c r="AH28" s="30" t="str">
         <x:v>Polyethylene resin; Plastic additives; Petroleum; Ethylene; Catalyst</x:v>
       </x:c>
-      <x:c r="AH28" s="30" t="str">
+      <x:c r="AI28" s="30" t="str">
         <x:v>Automotive painting; Electronics manufacturing; Furniture production; Construction; Metal processing</x:v>
       </x:c>
-      <x:c r="AI28" s="30" t="str">
+      <x:c r="AJ28" s="30" t="str">
         <x:v>tape; masking film</x:v>
       </x:c>
-      <x:c r="AJ28" s="30" t="str">
+      <x:c r="AK28" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search; masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK28" s="30" t="str">
+      <x:c r="AL28" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL28" s="30" t="str"/>
       <x:c r="AM28" s="30" t="str"/>
-      <x:c r="AN28" s="34" t="n">
+      <x:c r="AN28" s="30" t="str"/>
+      <x:c r="AO28" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="44" customHeight="1">
       <x:c r="A29" s="30" t="str">
-        <x:v>API联系方式已获取</x:v>
+        <x:v>同法人实体已去重-复用有效邮箱</x:v>
       </x:c>
       <x:c r="B29" s="30" t="str">
         <x:v>常规-全球</x:v>
@@ -3066,19 +3145,16 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G29" s="30" t="str">
-        <x:f>IF(V29&lt;&gt;"",V29,U29)</x:f>
-        <x:v>aruna.sharma@vivoglobal.com</x:v>
+        <x:v>support.in@vivo.com</x:v>
       </x:c>
       <x:c r="H29" s="30" t="str">
-        <x:f>IF(V29&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB29)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
-      </x:c>
-      <x:c r="I29" s="30" t="str">
-        <x:f>IF(X29&lt;&gt;"",X29,W29)</x:f>
-      </x:c>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC29)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC29)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC29)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC29)),"判定无效",IF(V29&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
+      </x:c>
+      <x:c r="I29" s="30" t="str"/>
       <x:c r="J29" s="30" t="str"/>
       <x:c r="K29" s="35" t="n">
-        <x:f>ROUND((IF(G29&lt;&gt;"",40,0)+IF(I29&lt;&gt;"",25,0)+IF(J29&lt;&gt;"",20,0)+IF(Z29&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H29="已验证有效",40,IF(V29&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y29)),25,0)+IF(J29&lt;&gt;"",20,0)+IF(AA29&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="L29" s="30" t="str">
@@ -3107,37 +3183,44 @@
       <x:c r="U29" s="30" t="str">
         <x:v>aruna.sharma@vivoglobal.com</x:v>
       </x:c>
-      <x:c r="V29" s="30" t="str"/>
+      <x:c r="V29" s="30" t="str">
+        <x:v>support.in@vivo.com; vcare@vivo.com</x:v>
+      </x:c>
       <x:c r="W29" s="30" t="str"/>
       <x:c r="X29" s="30" t="str"/>
       <x:c r="Y29" s="30" t="str"/>
       <x:c r="Z29" s="30" t="str"/>
       <x:c r="AA29" s="30" t="str"/>
-      <x:c r="AB29" s="30" t="str">
-        <x:v>aruna.sharma@vivoglobal.com:0</x:v>
-      </x:c>
-      <x:c r="AC29" s="30" t="str"/>
-      <x:c r="AD29" s="30" t="str">
+      <x:c r="AB29" s="30" t="str"/>
+      <x:c r="AC29" s="30" t="str">
+        <x:v>aruna.sharma@vivoglobal.com:3; support.in@vivo.com:1; vcare@vivo.com:1</x:v>
+      </x:c>
+      <x:c r="AD29" s="30" t="str"/>
+      <x:c r="AE29" s="30" t="str">
         <x:v>paper; arts; water contact indicator tape; mobile phone 5</x:v>
       </x:c>
-      <x:c r="AE29" s="30" t="str">
+      <x:c r="AF29" s="30" t="str">
         <x:v>5181866 WATER CONTACT INDICATOR TAPE PAPER PARTS FOR MFG OF MOBILE PHONE 5181866 WATER CONTACT INDICATOR TAPE PAPER PARTS FOR MFG</x:v>
       </x:c>
-      <x:c r="AF29" s="30" t="str"/>
       <x:c r="AG29" s="30" t="str"/>
       <x:c r="AH29" s="30" t="str"/>
-      <x:c r="AI29" s="30" t="str">
+      <x:c r="AI29" s="30" t="str"/>
+      <x:c r="AJ29" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ29" s="30" t="str">
+      <x:c r="AK29" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK29" s="30" t="str">
+      <x:c r="AL29" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL29" s="30" t="str"/>
-      <x:c r="AM29" s="30" t="str"/>
-      <x:c r="AN29" s="34" t="n">
+      <x:c r="AM29" s="30" t="str">
+        <x:v>同一总表中的同法人实体记录；两个邮箱已由 API 验证为有效</x:v>
+      </x:c>
+      <x:c r="AN29" s="30" t="str">
+        <x:v>公司名称、国家和业务实体一致；避免为重复实体再次购买联系方式。</x:v>
+      </x:c>
+      <x:c r="AO29" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -3161,22 +3244,21 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G30" s="30" t="str">
-        <x:f>IF(V30&lt;&gt;"",V30,U30)</x:f>
-        <x:v>contact.india@tesa.com</x:v>
+        <x:v>marketing.india@tesa.com</x:v>
       </x:c>
       <x:c r="H30" s="30" t="str">
-        <x:f>IF(V30&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB30)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC30)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC30)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC30)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC30)),"判定无效",IF(V30&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>验证不确定</x:v>
       </x:c>
       <x:c r="I30" s="30" t="str">
-        <x:f>IF(X30&lt;&gt;"",X30,W30)</x:f>
+        <x:v>+91 22 4741 9200</x:v>
       </x:c>
       <x:c r="J30" s="30" t="str">
         <x:v>www.tesa.in</x:v>
       </x:c>
       <x:c r="K30" s="35" t="n">
-        <x:f>ROUND((IF(G30&lt;&gt;"",40,0)+IF(I30&lt;&gt;"",25,0)+IF(J30&lt;&gt;"",20,0)+IF(Z30&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.75</x:v>
+        <x:f>ROUND((IF(H30="已验证有效",40,IF(V30&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y30)),25,0)+IF(J30&lt;&gt;"",20,0)+IF(AA30&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="L30" s="30" t="str">
         <x:v>待联系</x:v>
@@ -3202,39 +3284,50 @@
         <x:v>45867.666666666664</x:v>
       </x:c>
       <x:c r="U30" s="30" t="str">
-        <x:v>contact.india@tesa.com</x:v>
-      </x:c>
-      <x:c r="V30" s="30" t="str"/>
+        <x:v>contact.india@tesa.com; arorarajeev2001@yahoo.com</x:v>
+      </x:c>
+      <x:c r="V30" s="30" t="str">
+        <x:v>marketing.india@tesa.com</x:v>
+      </x:c>
       <x:c r="W30" s="30" t="str"/>
-      <x:c r="X30" s="30" t="str"/>
-      <x:c r="Y30" s="30" t="str"/>
-      <x:c r="Z30" s="30" t="str">
-        <x:v>https://www.linkedin.com/company/tesa</x:v>
-      </x:c>
-      <x:c r="AA30" s="30" t="str"/>
-      <x:c r="AB30" s="30" t="str">
-        <x:v>contact.india@tesa.com:0</x:v>
-      </x:c>
-      <x:c r="AC30" s="30" t="str"/>
+      <x:c r="X30" s="30" t="str">
+        <x:v>+91 22 4741 9200</x:v>
+      </x:c>
+      <x:c r="Y30" s="30" t="str">
+        <x:v>+91 22 4741 9200:状态1/类型1/WhatsApp0</x:v>
+      </x:c>
+      <x:c r="Z30" s="30" t="str"/>
+      <x:c r="AA30" s="30" t="str">
+        <x:v>https://www.linkedin.com/company/tesa; https://www.linkedin.com/in/rajeev-arora-a04a3521</x:v>
+      </x:c>
+      <x:c r="AB30" s="30" t="str"/>
+      <x:c r="AC30" s="30" t="str">
+        <x:v>contact.india@tesa.com:2; arorarajeev2001@yahoo.com:0; marketing.india@tesa.com:3</x:v>
+      </x:c>
       <x:c r="AD30" s="30" t="str"/>
-      <x:c r="AE30" s="30" t="str">
+      <x:c r="AE30" s="30" t="str"/>
+      <x:c r="AF30" s="30" t="str">
         <x:v>P/N:60996-60000-43 TS4363TLW050M10800 4363-PV43 TESA D/S ADHESIVE TAPE 1080MMX50MP/N:60996-60000-43 TS4363TLW050M10800 4363-PV43 TESA D/S ADH</x:v>
       </x:c>
-      <x:c r="AF30" s="30" t="str"/>
       <x:c r="AG30" s="30" t="str"/>
       <x:c r="AH30" s="30" t="str"/>
-      <x:c r="AI30" s="30" t="str">
+      <x:c r="AI30" s="30" t="str"/>
+      <x:c r="AJ30" s="30" t="str">
         <x:v>tape</x:v>
       </x:c>
-      <x:c r="AJ30" s="30" t="str">
+      <x:c r="AK30" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
       </x:c>
-      <x:c r="AK30" s="30" t="str">
-        <x:v>UpKuajing customs company contact API</x:v>
-      </x:c>
-      <x:c r="AL30" s="30" t="str"/>
-      <x:c r="AM30" s="30" t="str"/>
-      <x:c r="AN30" s="34" t="n">
+      <x:c r="AL30" s="30" t="str">
+        <x:v>UpKuajing customs company contact API; UpKuajing reviewed person contact API</x:v>
+      </x:c>
+      <x:c r="AM30" s="30" t="str">
+        <x:v>https://www.tesa.com/en-in/industry/lp/automotive/hole-covering-linkedin</x:v>
+      </x:c>
+      <x:c r="AN30" s="30" t="str">
+        <x:v>企业官网；tesa India 官网明确标注的业务联系邮箱和电话 +91 22 4741 9200。 验证状态=3。; 人物补充：Rajeev Arora（Head of Operations）；运营负责人，且公司精确匹配 tesa India。</x:v>
+      </x:c>
+      <x:c r="AO30" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -3258,22 +3351,20 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G31" s="30" t="str">
-        <x:f>IF(V31&lt;&gt;"",V31,U31)</x:f>
         <x:v>cs@saraswatigroupdb.com</x:v>
       </x:c>
       <x:c r="H31" s="30" t="str">
-        <x:f>IF(V31&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB31)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC31)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC31)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC31)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC31)),"判定无效",IF(V31&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I31" s="30" t="str">
-        <x:f>IF(X31&lt;&gt;"",X31,W31)</x:f>
         <x:v>+91 1923 222 814</x:v>
       </x:c>
       <x:c r="J31" s="30" t="str">
         <x:v>www.saraswati-group.com</x:v>
       </x:c>
       <x:c r="K31" s="35" t="n">
-        <x:f>ROUND((IF(G31&lt;&gt;"",40,0)+IF(I31&lt;&gt;"",25,0)+IF(J31&lt;&gt;"",20,0)+IF(Z31&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H31="已验证有效",40,IF(V31&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y31)),25,0)+IF(J31&lt;&gt;"",20,0)+IF(AA31&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="L31" s="30" t="str">
@@ -3307,42 +3398,45 @@
         <x:v>+91 1923 222 814</x:v>
       </x:c>
       <x:c r="X31" s="30" t="str"/>
-      <x:c r="Y31" s="30" t="str"/>
+      <x:c r="Y31" s="30" t="str">
+        <x:v>+91 1923 222 814:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z31" s="30" t="str"/>
       <x:c r="AA31" s="30" t="str"/>
-      <x:c r="AB31" s="30" t="str">
+      <x:c r="AB31" s="30" t="str"/>
+      <x:c r="AC31" s="30" t="str">
         <x:v>cs@saraswatigroupdb.com:1</x:v>
       </x:c>
-      <x:c r="AC31" s="30" t="str">
+      <x:c r="AD31" s="30" t="str">
         <x:v>Masking film</x:v>
       </x:c>
-      <x:c r="AD31" s="30" t="str">
+      <x:c r="AE31" s="30" t="str">
         <x:v>Masking film; Protection film; Clear film; PS sheet</x:v>
       </x:c>
-      <x:c r="AE31" s="30" t="str">
+      <x:c r="AF31" s="30" t="str">
         <x:v>MASKING FILM (PRE PROTECTION FILM),FILM CLEAR FILM FOR PS SHEET,50*1250*1500(20 ROLLS)(ACTUAL USER)MASKING FILM (PRE PROTECTION FILM)</x:v>
       </x:c>
-      <x:c r="AF31" s="30" t="str">
+      <x:c r="AG31" s="30" t="str">
         <x:v>Pre - protection film; Surface masking film; Clear masking film; PS sheet protection film; Temporary masking film</x:v>
       </x:c>
-      <x:c r="AG31" s="30" t="str">
+      <x:c r="AH31" s="30" t="str">
         <x:v>Plastic resin; Polymer; Additives; Solvents; Pigments</x:v>
       </x:c>
-      <x:c r="AH31" s="30" t="str">
+      <x:c r="AI31" s="30" t="str">
         <x:v>Electronics manufacturing; Automotive painting; Furniture production; Glass manufacturing; Construction</x:v>
       </x:c>
-      <x:c r="AI31" s="30" t="str">
+      <x:c r="AJ31" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ31" s="30" t="str">
+      <x:c r="AK31" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK31" s="30" t="str">
+      <x:c r="AL31" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL31" s="30" t="str"/>
       <x:c r="AM31" s="30" t="str"/>
-      <x:c r="AN31" s="34" t="n">
+      <x:c r="AN31" s="30" t="str"/>
+      <x:c r="AO31" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -3366,22 +3460,20 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G32" s="30" t="str">
-        <x:f>IF(V32&lt;&gt;"",V32,U32)</x:f>
         <x:v>deepak.goyal@airworks.in</x:v>
       </x:c>
       <x:c r="H32" s="30" t="str">
-        <x:f>IF(V32&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB32)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC32)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC32)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC32)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC32)),"判定无效",IF(V32&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I32" s="30" t="str">
-        <x:f>IF(X32&lt;&gt;"",X32,W32)</x:f>
         <x:v>+91 124 464 2200</x:v>
       </x:c>
       <x:c r="J32" s="30" t="str">
         <x:v>www.airworks.in</x:v>
       </x:c>
       <x:c r="K32" s="35" t="n">
-        <x:f>ROUND((IF(G32&lt;&gt;"",40,0)+IF(I32&lt;&gt;"",25,0)+IF(J32&lt;&gt;"",20,0)+IF(Z32&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H32="已验证有效",40,IF(V32&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y32)),25,0)+IF(J32&lt;&gt;"",20,0)+IF(AA32&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="L32" s="30" t="str">
@@ -3415,44 +3507,47 @@
         <x:v>+91 124 464 2200</x:v>
       </x:c>
       <x:c r="X32" s="30" t="str"/>
-      <x:c r="Y32" s="30" t="str"/>
-      <x:c r="Z32" s="30" t="str">
+      <x:c r="Y32" s="30" t="str">
+        <x:v>+91 124 464 2200:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
+      <x:c r="Z32" s="30" t="str"/>
+      <x:c r="AA32" s="30" t="str">
         <x:v>https://www.facebook.com/AirworksIndiaenggPvtLtd; https://www.linkedin.com/company/air-works</x:v>
       </x:c>
-      <x:c r="AA32" s="30" t="str"/>
-      <x:c r="AB32" s="30" t="str">
+      <x:c r="AB32" s="30" t="str"/>
+      <x:c r="AC32" s="30" t="str">
         <x:v>deepak.goyal@airworks.in:1</x:v>
       </x:c>
-      <x:c r="AC32" s="30" t="str">
+      <x:c r="AD32" s="30" t="str">
         <x:v>Masking Film</x:v>
       </x:c>
-      <x:c r="AD32" s="30" t="str">
+      <x:c r="AE32" s="30" t="str">
         <x:v>Masking Film; Aircraft use; Blue</x:v>
       </x:c>
-      <x:c r="AE32" s="30" t="str">
+      <x:c r="AF32" s="30" t="str">
         <x:v>WTE-MF-17-G Masking Film- 6m x 100m x 17mu Blue(Carton:-98cmx 15 x 15 - Per Roll)(FOR AIRCRAFT USE)(ACTUAL USE)18 ROLLSWTE-MF-17-G Masking Film- 6m x 100m x 17mu Blue(Carton:-98cm</x:v>
       </x:c>
-      <x:c r="AF32" s="30" t="str">
+      <x:c r="AG32" s="30" t="str">
         <x:v>Painter's tape; Protective film; Covering film; Surface protection film; Temporary masking film</x:v>
       </x:c>
-      <x:c r="AG32" s="30" t="str">
+      <x:c r="AH32" s="30" t="str">
         <x:v>Plastic resin; Polymer; Additives; Pigments; Adhesive</x:v>
       </x:c>
-      <x:c r="AH32" s="30" t="str">
+      <x:c r="AI32" s="30" t="str">
         <x:v>Aircraft manufacturing; Aircraft maintenance; Automotive painting; Industrial coating; Construction painting</x:v>
       </x:c>
-      <x:c r="AI32" s="30" t="str">
+      <x:c r="AJ32" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ32" s="30" t="str">
+      <x:c r="AK32" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK32" s="30" t="str">
+      <x:c r="AL32" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL32" s="30" t="str"/>
       <x:c r="AM32" s="30" t="str"/>
-      <x:c r="AN32" s="34" t="n">
+      <x:c r="AN32" s="30" t="str"/>
+      <x:c r="AO32" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -3476,22 +3571,20 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G33" s="30" t="str">
-        <x:f>IF(V33&lt;&gt;"",V33,U33)</x:f>
         <x:v>info@sumaxindia.com</x:v>
       </x:c>
       <x:c r="H33" s="30" t="str">
-        <x:f>IF(V33&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB33)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC33)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC33)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC33)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC33)),"判定无效",IF(V33&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I33" s="30" t="str">
-        <x:f>IF(X33&lt;&gt;"",X33,W33)</x:f>
         <x:v>+91 40 2773 7001</x:v>
       </x:c>
       <x:c r="J33" s="30" t="str">
         <x:v>www.sumaxindia.com</x:v>
       </x:c>
       <x:c r="K33" s="35" t="n">
-        <x:f>ROUND((IF(G33&lt;&gt;"",40,0)+IF(I33&lt;&gt;"",25,0)+IF(J33&lt;&gt;"",20,0)+IF(Z33&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H33="已验证有效",40,IF(V33&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y33)),25,0)+IF(J33&lt;&gt;"",20,0)+IF(AA33&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="L33" s="30" t="str">
@@ -3523,42 +3616,45 @@
         <x:v>+91 40 2773 7001</x:v>
       </x:c>
       <x:c r="X33" s="30" t="str"/>
-      <x:c r="Y33" s="30" t="str"/>
+      <x:c r="Y33" s="30" t="str">
+        <x:v>+91 40 2773 7001:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z33" s="30" t="str"/>
       <x:c r="AA33" s="30" t="str"/>
-      <x:c r="AB33" s="30" t="str">
+      <x:c r="AB33" s="30" t="str"/>
+      <x:c r="AC33" s="30" t="str">
         <x:v>info@sumaxindia.com:1</x:v>
       </x:c>
-      <x:c r="AC33" s="30" t="str">
+      <x:c r="AD33" s="30" t="str">
         <x:v>Masking Film</x:v>
       </x:c>
-      <x:c r="AD33" s="30" t="str">
+      <x:c r="AE33" s="30" t="str">
         <x:v>Masking; Film</x:v>
       </x:c>
-      <x:c r="AE33" s="30" t="str">
+      <x:c r="AF33" s="30" t="str">
         <x:v>MASKING FILM (535 MMX1200M) 1 PCS</x:v>
       </x:c>
-      <x:c r="AF33" s="30" t="str">
+      <x:c r="AG33" s="30" t="str">
         <x:v>Painter's tape film; Protective masking film; Temporary masking film; Construction masking film; Decorative masking film</x:v>
       </x:c>
-      <x:c r="AG33" s="30" t="str">
+      <x:c r="AH33" s="30" t="str">
         <x:v>Plastic resin; Polymer; Chemical additives; Adhesive; Base film material</x:v>
       </x:c>
-      <x:c r="AH33" s="30" t="str">
+      <x:c r="AI33" s="30" t="str">
         <x:v>Painting projects; Construction sites; Automotive refinishing; Furniture manufacturing; Decorative work</x:v>
       </x:c>
-      <x:c r="AI33" s="30" t="str">
+      <x:c r="AJ33" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ33" s="30" t="str">
+      <x:c r="AK33" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK33" s="30" t="str">
+      <x:c r="AL33" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL33" s="30" t="str"/>
       <x:c r="AM33" s="30" t="str"/>
-      <x:c r="AN33" s="34" t="n">
+      <x:c r="AN33" s="30" t="str"/>
+      <x:c r="AO33" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -3582,22 +3678,20 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G34" s="30" t="str">
-        <x:f>IF(V34&lt;&gt;"",V34,U34)</x:f>
-        <x:v>aipl.sunsui@ajitindustries.com; marketing@ajitindustries.com</x:v>
+        <x:v>marketing@ajitindustries.com</x:v>
       </x:c>
       <x:c r="H34" s="30" t="str">
-        <x:f>IF(V34&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB34)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC34)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC34)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC34)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC34)),"判定无效",IF(V34&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I34" s="30" t="str">
-        <x:f>IF(X34&lt;&gt;"",X34,W34)</x:f>
         <x:v>+91 11 4901 0101</x:v>
       </x:c>
       <x:c r="J34" s="30" t="str">
         <x:v>http://www.ajitindustries.com/</x:v>
       </x:c>
       <x:c r="K34" s="35" t="n">
-        <x:f>ROUND((IF(G34&lt;&gt;"",40,0)+IF(I34&lt;&gt;"",25,0)+IF(J34&lt;&gt;"",20,0)+IF(Z34&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H34="已验证有效",40,IF(V34&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y34)),25,0)+IF(J34&lt;&gt;"",20,0)+IF(AA34&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="L34" s="30" t="str">
@@ -3631,34 +3725,37 @@
         <x:v>+91 11 4901 0101</x:v>
       </x:c>
       <x:c r="X34" s="30" t="str"/>
-      <x:c r="Y34" s="30" t="str"/>
+      <x:c r="Y34" s="30" t="str">
+        <x:v>+91 11 4901 0101:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z34" s="30" t="str"/>
       <x:c r="AA34" s="30" t="str"/>
-      <x:c r="AB34" s="30" t="str">
-        <x:v>aipl.sunsui@ajitindustries.com:0; marketing@ajitindustries.com:1</x:v>
-      </x:c>
-      <x:c r="AC34" s="30" t="str"/>
-      <x:c r="AD34" s="30" t="str">
+      <x:c r="AB34" s="30" t="str"/>
+      <x:c r="AC34" s="30" t="str">
+        <x:v>aipl.sunsui@ajitindustries.com:2; marketing@ajitindustries.com:1</x:v>
+      </x:c>
+      <x:c r="AD34" s="30" t="str"/>
+      <x:c r="AE34" s="30" t="str">
         <x:v>roll; tria; masking film; arg; e roll</x:v>
       </x:c>
-      <x:c r="AE34" s="30" t="str">
+      <x:c r="AF34" s="30" t="str">
         <x:v>PE MASKING FILM IN LARGE ROLL SIZE: 2700MM*1600M (ROLL 600)(FOR INDUSTRIAL USE)PE MASKING FILM IN</x:v>
       </x:c>
-      <x:c r="AF34" s="30" t="str"/>
       <x:c r="AG34" s="30" t="str"/>
       <x:c r="AH34" s="30" t="str"/>
-      <x:c r="AI34" s="30" t="str">
+      <x:c r="AI34" s="30" t="str"/>
+      <x:c r="AJ34" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ34" s="30" t="str">
+      <x:c r="AK34" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK34" s="30" t="str">
+      <x:c r="AL34" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL34" s="30" t="str"/>
       <x:c r="AM34" s="30" t="str"/>
-      <x:c r="AN34" s="34" t="n">
+      <x:c r="AN34" s="30" t="str"/>
+      <x:c r="AO34" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -3682,22 +3779,20 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G35" s="30" t="str">
-        <x:f>IF(V35&lt;&gt;"",V35,U35)</x:f>
-        <x:v>info@modularfurniturebpl.com; pryentp@hotmail.com</x:v>
+        <x:v>pryentp@hotmail.com</x:v>
       </x:c>
       <x:c r="H35" s="30" t="str">
-        <x:f>IF(V35&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB35)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC35)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC35)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC35)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC35)),"判定无效",IF(V35&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I35" s="30" t="str">
-        <x:f>IF(X35&lt;&gt;"",X35,W35)</x:f>
-        <x:v>919425; +91 94250 08422; +91 94250 08433; +91 94250 26178</x:v>
+        <x:v>+91 94250 08422</x:v>
       </x:c>
       <x:c r="J35" s="30" t="str">
         <x:v>modularfurniturebpl.com</x:v>
       </x:c>
       <x:c r="K35" s="35" t="n">
-        <x:f>ROUND((IF(G35&lt;&gt;"",40,0)+IF(I35&lt;&gt;"",25,0)+IF(J35&lt;&gt;"",20,0)+IF(Z35&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H35="已验证有效",40,IF(V35&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y35)),25,0)+IF(J35&lt;&gt;"",20,0)+IF(AA35&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="L35" s="30" t="str">
@@ -3730,45 +3825,48 @@
       </x:c>
       <x:c r="X35" s="30" t="str"/>
       <x:c r="Y35" s="30" t="str">
+        <x:v>919425:状态2/类型0/WhatsApp2; +91 94250 08422:状态1/类型2/WhatsApp1; +91 94250 08433:状态1/类型2/WhatsApp2; +91 94250 26178:状态1/类型2/WhatsApp1</x:v>
+      </x:c>
+      <x:c r="Z35" s="30" t="str">
         <x:v>+91 94250 08422; +91 94250 26178</x:v>
       </x:c>
-      <x:c r="Z35" s="30" t="str">
+      <x:c r="AA35" s="30" t="str">
         <x:v>https://www.facebook.com/pages/Priyanka-Enterprises/278369785647345; https://www.linkedin.com/company/priyanka-enterprise</x:v>
       </x:c>
-      <x:c r="AA35" s="30" t="str"/>
-      <x:c r="AB35" s="30" t="str">
-        <x:v>info@modularfurniturebpl.com:0; pryentp@hotmail.com:1</x:v>
-      </x:c>
+      <x:c r="AB35" s="30" t="str"/>
       <x:c r="AC35" s="30" t="str">
+        <x:v>info@modularfurniturebpl.com:2; pryentp@hotmail.com:1</x:v>
+      </x:c>
+      <x:c r="AD35" s="30" t="str">
         <x:v>Pretaped masking film; Masking tape</x:v>
       </x:c>
-      <x:c r="AD35" s="30" t="str">
+      <x:c r="AE35" s="30" t="str">
         <x:v>Pretaped masking film; Masking tape; HDPE; Shrink wrapped; Color label</x:v>
       </x:c>
-      <x:c r="AE35" s="30" t="str">
+      <x:c r="AF35" s="30" t="str">
         <x:v>PRETAPED MASKING FILM - 1M X 25M,PRETAPED MASKING FILM, HDPE, MASKING TAPE, EACH ROLL SHRINK WRAPPED WITH COLOR LABEL (2PRETAPED MASKING FILM - 1M X 25M,PRETAPED MASKING FILM, HDPE</x:v>
       </x:c>
-      <x:c r="AF35" s="30" t="str">
+      <x:c r="AG35" s="30" t="str">
         <x:v>Masking film with tape; Pre - taped film for masking; Self - taped masking film; HDPE masking film; Taped masking sheet</x:v>
       </x:c>
-      <x:c r="AG35" s="30" t="str">
+      <x:c r="AH35" s="30" t="str">
         <x:v>High - density polyethylene resin; Plastic additives; Adhesive materials; Polymer raw materials; Tape backing materials</x:v>
       </x:c>
-      <x:c r="AH35" s="30" t="str">
+      <x:c r="AI35" s="30" t="str">
         <x:v>Painting industry; Automotive refinishing; Construction projects; Furniture manufacturing; DIY home improvement</x:v>
       </x:c>
-      <x:c r="AI35" s="30" t="str">
+      <x:c r="AJ35" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ35" s="30" t="str">
+      <x:c r="AK35" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK35" s="30" t="str">
+      <x:c r="AL35" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL35" s="30" t="str"/>
       <x:c r="AM35" s="30" t="str"/>
-      <x:c r="AN35" s="34" t="n">
+      <x:c r="AN35" s="30" t="str"/>
+      <x:c r="AO35" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -3792,22 +3890,20 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G36" s="30" t="str">
-        <x:f>IF(V36&lt;&gt;"",V36,U36)</x:f>
         <x:v>sharecmpt.gno@saint-gobain.com</x:v>
       </x:c>
       <x:c r="H36" s="30" t="str">
-        <x:f>IF(V36&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB36)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC36)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC36)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC36)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC36)),"判定无效",IF(V36&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I36" s="30" t="str">
-        <x:f>IF(X36&lt;&gt;"",X36,W36)</x:f>
-        <x:v>00975261212261166; 01204061800899; 016124236502425851; 0202551089193; 0222723002126; 0224013257825852590; 04027713040; 065722254152228432; 07104676464; 079400399010203; 0802559400425587248; 08030978888; 0877228573135; 098050253045; +91 22 4021 2121; 9327266444</x:v>
+        <x:v>+91 22 4021 2121</x:v>
       </x:c>
       <x:c r="J36" s="30" t="str">
         <x:v>www.grindwellnorton.com</x:v>
       </x:c>
       <x:c r="K36" s="35" t="n">
-        <x:f>ROUND((IF(G36&lt;&gt;"",40,0)+IF(I36&lt;&gt;"",25,0)+IF(J36&lt;&gt;"",20,0)+IF(Z36&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H36="已验证有效",40,IF(V36&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y36)),25,0)+IF(J36&lt;&gt;"",20,0)+IF(AA36&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="L36" s="30" t="str">
@@ -3841,44 +3937,47 @@
         <x:v>00975261212261166; 01204061800899; 016124236502425851; 0202551089193; 0222723002126; 0224013257825852590; 04027713040; 065722254152228432; 07104676464; 079400399010203; 0802559400425587248; 08030978888; 0877228573135; 098050253045; +91 22 4021 2121; 9327266444</x:v>
       </x:c>
       <x:c r="X36" s="30" t="str"/>
-      <x:c r="Y36" s="30" t="str"/>
-      <x:c r="Z36" s="30" t="str">
+      <x:c r="Y36" s="30" t="str">
+        <x:v>00975261212261166:状态2/类型0/WhatsApp0; 01204061800899:状态2/类型0/WhatsApp0; 016124236502425851:状态2/类型0/WhatsApp0; 0202551089193:状态2/类型0/WhatsApp0; 0222723002126:状态2/类型0/WhatsApp0; 0224013257825852590:状态2/类型0/WhatsApp0; 04027713040:状态2/类型1/WhatsApp0; 065722254152228432:状态2/类型0/WhatsApp0; 07104676464:状态2/类型0/WhatsApp0; 079400399010203:状态2/类型0/WhatsApp0; 0802559400425587248:状态2/类型0/WhatsApp0; 08030978888:状态2/类型0/WhatsApp0; 0877228573135:状态2/类型0/WhatsApp0; 098050253045:状态2/类型0/WhatsApp0; +91 22 4021 2121:状态1/类型1/WhatsApp2; 9327266444:状态2/类型0/WhatsApp2</x:v>
+      </x:c>
+      <x:c r="Z36" s="30" t="str"/>
+      <x:c r="AA36" s="30" t="str">
         <x:v>https://www.facebook.com/saintgobaingroup; https://www.linkedin.com/company/grindwell-norton-ltd; https://www.linkedin.com/company/saint-gobain-group-india; https://www.pinterest.com/saintgobainnews; https://www.youtube.com/user/SaintGobainTV</x:v>
       </x:c>
-      <x:c r="AA36" s="30" t="str"/>
-      <x:c r="AB36" s="30" t="str">
+      <x:c r="AB36" s="30" t="str"/>
+      <x:c r="AC36" s="30" t="str">
         <x:v>sharecmpt.gno@saint-gobain.com:1</x:v>
       </x:c>
-      <x:c r="AC36" s="30" t="str">
+      <x:c r="AD36" s="30" t="str">
         <x:v>Plastic Masking Film</x:v>
       </x:c>
-      <x:c r="AD36" s="30" t="str">
+      <x:c r="AE36" s="30" t="str">
         <x:v>Plastic; Masking Film; MFG Use</x:v>
       </x:c>
-      <x:c r="AE36" s="30" t="str">
+      <x:c r="AF36" s="30" t="str">
         <x:v>PLASTIC MASKING FILM 9MIC X 4M X 150M 66254455280 600ROLLS (FOR MFG USE)PLASTIC MASKING FILM 9MIC X 4M X 150M 66254455280 600ROLLS (</x:v>
       </x:c>
-      <x:c r="AF36" s="30" t="str">
+      <x:c r="AG36" s="30" t="str">
         <x:v>Plastic Film Mask; Masking Plastic Sheeting; Plastic Protective Film; Film Masking; Plastic Covering Film</x:v>
       </x:c>
-      <x:c r="AG36" s="30" t="str">
+      <x:c r="AH36" s="30" t="str">
         <x:v>Plastic Resin; Polymer; Additives; Plasticizer; Colorant</x:v>
       </x:c>
-      <x:c r="AH36" s="30" t="str">
+      <x:c r="AI36" s="30" t="str">
         <x:v>Automotive Painting; Furniture Manufacturing; Electronics Assembly; Construction; Printing</x:v>
       </x:c>
-      <x:c r="AI36" s="30" t="str">
+      <x:c r="AJ36" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ36" s="30" t="str">
+      <x:c r="AK36" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK36" s="30" t="str">
+      <x:c r="AL36" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL36" s="30" t="str"/>
       <x:c r="AM36" s="30" t="str"/>
-      <x:c r="AN36" s="34" t="n">
+      <x:c r="AN36" s="30" t="str"/>
+      <x:c r="AO36" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -3900,22 +3999,20 @@
       </x:c>
       <x:c r="F37" s="30" t="str"/>
       <x:c r="G37" s="30" t="str">
-        <x:f>IF(V37&lt;&gt;"",V37,U37)</x:f>
         <x:v>bonded.gno@saint-gobain.com</x:v>
       </x:c>
       <x:c r="H37" s="30" t="str">
-        <x:f>IF(V37&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB37)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC37)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC37)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC37)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC37)),"判定无效",IF(V37&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I37" s="30" t="str">
-        <x:f>IF(X37&lt;&gt;"",X37,W37)</x:f>
         <x:v>+91 22 4021 2121</x:v>
       </x:c>
       <x:c r="J37" s="30" t="str">
         <x:v>http://www.grindwellnorton.co.in/</x:v>
       </x:c>
       <x:c r="K37" s="35" t="n">
-        <x:f>ROUND((IF(G37&lt;&gt;"",40,0)+IF(I37&lt;&gt;"",25,0)+IF(J37&lt;&gt;"",20,0)+IF(Z37&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H37="已验证有效",40,IF(V37&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y37)),25,0)+IF(J37&lt;&gt;"",20,0)+IF(AA37&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="L37" s="30" t="str">
@@ -3949,42 +4046,45 @@
         <x:v>+91 22 4021 2121</x:v>
       </x:c>
       <x:c r="X37" s="30" t="str"/>
-      <x:c r="Y37" s="30" t="str"/>
+      <x:c r="Y37" s="30" t="str">
+        <x:v>+91 22 4021 2121:状态1/类型1/WhatsApp2</x:v>
+      </x:c>
       <x:c r="Z37" s="30" t="str"/>
       <x:c r="AA37" s="30" t="str"/>
-      <x:c r="AB37" s="30" t="str">
-        <x:v>bonded.gno@saint-gobain.com:0</x:v>
-      </x:c>
+      <x:c r="AB37" s="30" t="str"/>
       <x:c r="AC37" s="30" t="str">
+        <x:v>bonded.gno@saint-gobain.com:1</x:v>
+      </x:c>
+      <x:c r="AD37" s="30" t="str">
         <x:v>Plastic masking film</x:v>
       </x:c>
-      <x:c r="AD37" s="30" t="str">
+      <x:c r="AE37" s="30" t="str">
         <x:v>Plastic; Masking film; MFG use</x:v>
       </x:c>
-      <x:c r="AE37" s="30" t="str">
+      <x:c r="AF37" s="30" t="str">
         <x:v>PLASTIC MASKING FILM 9MIC X 4M X 150M 66254455280 600ROLLS (FOR MFG USE)PLASTIC MASKING FILM 9MIC X 4M X 150M 66254455280 600ROLLS (</x:v>
       </x:c>
-      <x:c r="AF37" s="30" t="str">
+      <x:c r="AG37" s="30" t="str">
         <x:v>Plastic film mask; Masking plastic sheet; Plastic protective film; Film for masking; Plastic masking sheet</x:v>
       </x:c>
-      <x:c r="AG37" s="30" t="str">
+      <x:c r="AH37" s="30" t="str">
         <x:v>Plastic resin; Polymer; Additives; Plastic raw material; Plastic compound</x:v>
       </x:c>
-      <x:c r="AH37" s="30" t="str">
+      <x:c r="AI37" s="30" t="str">
         <x:v>Automotive painting; Furniture manufacturing; Electronics production; Construction painting; Metal finishing</x:v>
       </x:c>
-      <x:c r="AI37" s="30" t="str">
+      <x:c r="AJ37" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ37" s="30" t="str">
+      <x:c r="AK37" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK37" s="30" t="str">
+      <x:c r="AL37" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL37" s="30" t="str"/>
       <x:c r="AM37" s="30" t="str"/>
-      <x:c r="AN37" s="34" t="n">
+      <x:c r="AN37" s="30" t="str"/>
+      <x:c r="AO37" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -4008,21 +4108,18 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G38" s="30" t="str">
-        <x:f>IF(V38&lt;&gt;"",V38,U38)</x:f>
         <x:v>accounts@starcke.in</x:v>
       </x:c>
       <x:c r="H38" s="30" t="str">
-        <x:f>IF(V38&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB38)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
-      </x:c>
-      <x:c r="I38" s="30" t="str">
-        <x:f>IF(X38&lt;&gt;"",X38,W38)</x:f>
-      </x:c>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC38)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC38)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC38)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC38)),"判定无效",IF(V38&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
+      </x:c>
+      <x:c r="I38" s="30" t="str"/>
       <x:c r="J38" s="30" t="str">
         <x:v>www.starckeindia.com</x:v>
       </x:c>
       <x:c r="K38" s="35" t="n">
-        <x:f>ROUND((IF(G38&lt;&gt;"",40,0)+IF(I38&lt;&gt;"",25,0)+IF(J38&lt;&gt;"",20,0)+IF(Z38&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H38="已验证有效",40,IF(V38&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y38)),25,0)+IF(J38&lt;&gt;"",20,0)+IF(AA38&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="L38" s="30" t="str">
@@ -4057,35 +4154,36 @@
       <x:c r="Y38" s="30" t="str"/>
       <x:c r="Z38" s="30" t="str"/>
       <x:c r="AA38" s="30" t="str"/>
-      <x:c r="AB38" s="30" t="str">
+      <x:c r="AB38" s="30" t="str"/>
+      <x:c r="AC38" s="30" t="str">
         <x:v>accounts@starcke.in:1</x:v>
       </x:c>
-      <x:c r="AC38" s="30" t="str"/>
       <x:c r="AD38" s="30" t="str"/>
-      <x:c r="AE38" s="30" t="str">
+      <x:c r="AE38" s="30" t="str"/>
+      <x:c r="AF38" s="30" t="str">
         <x:v>MASKING FILM (4mx200m with LOGO) (200 CTNS) (200 ROLL) MASKING FILM (4mx200m with LOGO) (200 CTNS) (200 ROLL)</x:v>
       </x:c>
-      <x:c r="AF38" s="30" t="str"/>
       <x:c r="AG38" s="30" t="str"/>
       <x:c r="AH38" s="30" t="str"/>
-      <x:c r="AI38" s="30" t="str">
+      <x:c r="AI38" s="30" t="str"/>
+      <x:c r="AJ38" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ38" s="30" t="str">
+      <x:c r="AK38" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK38" s="30" t="str">
+      <x:c r="AL38" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL38" s="30" t="str"/>
       <x:c r="AM38" s="30" t="str"/>
-      <x:c r="AN38" s="34" t="n">
+      <x:c r="AN38" s="30" t="str"/>
+      <x:c r="AO38" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="44" customHeight="1">
       <x:c r="A39" s="30" t="str">
-        <x:v>API联系方式已获取</x:v>
+        <x:v>已补充有效决策人邮箱</x:v>
       </x:c>
       <x:c r="B39" s="30" t="str">
         <x:v>常规-全球</x:v>
@@ -4103,22 +4201,21 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G39" s="30" t="str">
-        <x:f>IF(V39&lt;&gt;"",V39,U39)</x:f>
-        <x:v>career@martfury.com; contact@martfury.com; customercare@martfury.com; info@superconduits.com; media@martfury.com; vendorsupport@martfury.com</x:v>
+        <x:v>jain.naman1984@gmail.com</x:v>
       </x:c>
       <x:c r="H39" s="30" t="str">
-        <x:f>IF(V39&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB39)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC39)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC39)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC39)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC39)),"判定无效",IF(V39&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
       </x:c>
       <x:c r="I39" s="30" t="str">
-        <x:f>IF(X39&lt;&gt;"",X39,W39)</x:f>
+        <x:v>+91 99993 27453</x:v>
       </x:c>
       <x:c r="J39" s="30" t="str">
         <x:v>superconduits.com</x:v>
       </x:c>
       <x:c r="K39" s="35" t="n">
-        <x:f>ROUND((IF(G39&lt;&gt;"",40,0)+IF(I39&lt;&gt;"",25,0)+IF(J39&lt;&gt;"",20,0)+IF(Z39&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.75</x:v>
+        <x:f>ROUND((IF(H39="已验证有效",40,IF(V39&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y39)),25,0)+IF(J39&lt;&gt;"",20,0)+IF(AA39&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L39" s="30" t="str">
         <x:v>待联系</x:v>
@@ -4142,49 +4239,60 @@
         <x:v>45690.666666666664</x:v>
       </x:c>
       <x:c r="U39" s="30" t="str">
-        <x:v>career@martfury.com; contact@martfury.com; customercare@martfury.com; info@superconduits.com; media@martfury.com; vendorsupport@martfury.com</x:v>
-      </x:c>
-      <x:c r="V39" s="30" t="str"/>
+        <x:v>career@martfury.com; contact@martfury.com; customercare@martfury.com; info@superconduits.com; media@martfury.com; vendorsupport@martfury.com; jain.naman1984@gmail.com</x:v>
+      </x:c>
+      <x:c r="V39" s="30" t="str">
+        <x:v>supsalcorp@gmail.com</x:v>
+      </x:c>
       <x:c r="W39" s="30" t="str"/>
-      <x:c r="X39" s="30" t="str"/>
-      <x:c r="Y39" s="30" t="str"/>
-      <x:c r="Z39" s="30" t="str">
-        <x:v>https://www.linkedin.com/company/super-sales-corporation</x:v>
-      </x:c>
-      <x:c r="AA39" s="30" t="str"/>
-      <x:c r="AB39" s="30" t="str">
-        <x:v>career@martfury.com:0; contact@martfury.com:0; customercare@martfury.com:0; info@superconduits.com:0; media@martfury.com:0; vendorsupport@martfury.com:0</x:v>
-      </x:c>
+      <x:c r="X39" s="30" t="str">
+        <x:v>+91 99993 27453</x:v>
+      </x:c>
+      <x:c r="Y39" s="30" t="str">
+        <x:v>+91 99993 27453:状态1/类型2/WhatsApp1</x:v>
+      </x:c>
+      <x:c r="Z39" s="30" t="str"/>
+      <x:c r="AA39" s="30" t="str">
+        <x:v>https://www.linkedin.com/company/super-sales-corporation; https://www.linkedin.com/in/jainnaman</x:v>
+      </x:c>
+      <x:c r="AB39" s="30" t="str"/>
       <x:c r="AC39" s="30" t="str">
+        <x:v>career@martfury.com:2; contact@martfury.com:2; customercare@martfury.com:2; info@superconduits.com:2; media@martfury.com:2; vendorsupport@martfury.com:2; jain.naman1984@gmail.com:1; supsalcorp@gmail.com:3</x:v>
+      </x:c>
+      <x:c r="AD39" s="30" t="str">
         <x:v>Pre-taped Masking Film</x:v>
       </x:c>
-      <x:c r="AD39" s="30" t="str">
+      <x:c r="AE39" s="30" t="str">
         <x:v>Pre-taped; Masking Film</x:v>
       </x:c>
-      <x:c r="AE39" s="30" t="str">
+      <x:c r="AF39" s="30" t="str">
         <x:v>PRE-TAPED MASKING FILM,STYLE NO:80MM*45M(5400 ROLL) PRE-TAPED MASKING FILM,STYLE NO:80MM*45M(5400 ROLL)</x:v>
       </x:c>
-      <x:c r="AF39" s="30" t="str">
+      <x:c r="AG39" s="30" t="str">
         <x:v>Taped Masking Film; Masking Tape Film; Pre - applied Masking Film; Self - taped Masking Film; Adhesive Masking Film</x:v>
       </x:c>
-      <x:c r="AG39" s="30" t="str">
+      <x:c r="AH39" s="30" t="str">
         <x:v>Plastic Resin; Adhesive; Polymer; Film Base Material; Tape</x:v>
       </x:c>
-      <x:c r="AH39" s="30" t="str">
+      <x:c r="AI39" s="30" t="str">
         <x:v>Automotive Painting; Furniture Finishing; Construction Painting; DIY Projects; Industrial Coating</x:v>
       </x:c>
-      <x:c r="AI39" s="30" t="str">
+      <x:c r="AJ39" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ39" s="30" t="str">
+      <x:c r="AK39" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK39" s="30" t="str">
-        <x:v>UpKuajing customs company contact API</x:v>
-      </x:c>
-      <x:c r="AL39" s="30" t="str"/>
-      <x:c r="AM39" s="30" t="str"/>
-      <x:c r="AN39" s="34" t="n">
+      <x:c r="AL39" s="30" t="str">
+        <x:v>UpKuajing customs company contact API; UpKuajing reviewed person contact API</x:v>
+      </x:c>
+      <x:c r="AM39" s="30" t="str">
+        <x:v>https://www.scamadviser.com/check-website/superconduits.com</x:v>
+      </x:c>
+      <x:c r="AN39" s="30" t="str">
+        <x:v>域名登记信息聚合；superconduits.com 的域名登记联系人邮箱；只有验证有效才纳入首选邮箱候选。 验证状态=3。; 人物补充：Naman Jain（Executive Partner）；企业合伙人，且公司精确匹配 Super Sales Corporation。</x:v>
+      </x:c>
+      <x:c r="AO39" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -4208,22 +4316,21 @@
         <x:v>LK</x:v>
       </x:c>
       <x:c r="G40" s="30" t="str">
-        <x:f>IF(V40&lt;&gt;"",V40,U40)</x:f>
-        <x:v>jeff.smith@aquadynamicconsultancy.com</x:v>
+        <x:v>udaya@aquadynamics.lk</x:v>
       </x:c>
       <x:c r="H40" s="30" t="str">
-        <x:f>IF(V40&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB40)),"API已验证","未验证"))</x:f>
-        <x:v>未验证</x:v>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC40)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC40)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC40)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC40)),"判定无效",IF(V40&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>验证不确定</x:v>
       </x:c>
       <x:c r="I40" s="30" t="str">
-        <x:f>IF(X40&lt;&gt;"",X40,W40)</x:f>
+        <x:v>+94 31 5553500</x:v>
       </x:c>
       <x:c r="J40" s="30" t="str">
         <x:v>http://www.aquadynamicconsultancy.com</x:v>
       </x:c>
       <x:c r="K40" s="35" t="n">
-        <x:f>ROUND((IF(G40&lt;&gt;"",40,0)+IF(I40&lt;&gt;"",25,0)+IF(J40&lt;&gt;"",20,0)+IF(Z40&lt;&gt;"",15,0))/100,2)</x:f>
-        <x:v>0.6</x:v>
+        <x:f>ROUND((IF(H40="已验证有效",40,IF(V40&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y40)),25,0)+IF(J40&lt;&gt;"",20,0)+IF(AA40&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="L40" s="30" t="str">
         <x:v>待联系</x:v>
@@ -4249,39 +4356,52 @@
         <x:v>46078.666666666664</x:v>
       </x:c>
       <x:c r="U40" s="30" t="str">
-        <x:v>jeff.smith@aquadynamicconsultancy.com</x:v>
-      </x:c>
-      <x:c r="V40" s="30" t="str"/>
+        <x:v>jeff.smith@aquadynamicconsultancy.com; danesh@aquadynamics.lk</x:v>
+      </x:c>
+      <x:c r="V40" s="30" t="str">
+        <x:v>udaya@aquadynamics.lk</x:v>
+      </x:c>
       <x:c r="W40" s="30" t="str"/>
-      <x:c r="X40" s="30" t="str"/>
-      <x:c r="Y40" s="30" t="str"/>
+      <x:c r="X40" s="30" t="str">
+        <x:v>+94 31 5553500; +94 31 2235069; +94 77 7773669</x:v>
+      </x:c>
+      <x:c r="Y40" s="30" t="str">
+        <x:v>+94 31 5553500:状态1/类型1/WhatsApp2; +94 31 2235069:状态3/类型0/WhatsApp0; +94 77 7773669:状态3/类型0/WhatsApp0</x:v>
+      </x:c>
       <x:c r="Z40" s="30" t="str"/>
-      <x:c r="AA40" s="30" t="str"/>
-      <x:c r="AB40" s="30" t="str">
-        <x:v>jeff.smith@aquadynamicconsultancy.com:0</x:v>
-      </x:c>
-      <x:c r="AC40" s="30" t="str"/>
-      <x:c r="AD40" s="30" t="str">
+      <x:c r="AA40" s="30" t="str">
+        <x:v>https://www.linkedin.com/in/danesh-weerarathne-8a5b9330</x:v>
+      </x:c>
+      <x:c r="AB40" s="30" t="str"/>
+      <x:c r="AC40" s="30" t="str">
+        <x:v>jeff.smith@aquadynamicconsultancy.com:2; danesh@aquadynamics.lk:2; udaya@aquadynamics.lk:3</x:v>
+      </x:c>
+      <x:c r="AD40" s="30" t="str"/>
+      <x:c r="AE40" s="30" t="str">
         <x:v>masking film; masking; film for printing; rolls</x:v>
       </x:c>
-      <x:c r="AE40" s="30" t="str">
+      <x:c r="AF40" s="30" t="str">
         <x:v>54 ROLLS MASKING FILMS MASKING FILM FOR PRINTING</x:v>
       </x:c>
-      <x:c r="AF40" s="30" t="str"/>
       <x:c r="AG40" s="30" t="str"/>
       <x:c r="AH40" s="30" t="str"/>
-      <x:c r="AI40" s="30" t="str">
+      <x:c r="AI40" s="30" t="str"/>
+      <x:c r="AJ40" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ40" s="30" t="str">
+      <x:c r="AK40" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK40" s="30" t="str">
-        <x:v>UpKuajing customs company contact API</x:v>
-      </x:c>
-      <x:c r="AL40" s="30" t="str"/>
-      <x:c r="AM40" s="30" t="str"/>
-      <x:c r="AN40" s="34" t="n">
+      <x:c r="AL40" s="30" t="str">
+        <x:v>UpKuajing customs company contact API; UpKuajing reviewed person contact API</x:v>
+      </x:c>
+      <x:c r="AM40" s="30" t="str">
+        <x:v>https://rainbowpages.lk/other/unclassified/aqua-dynamics-pvt-ltd/</x:v>
+      </x:c>
+      <x:c r="AN40" s="30" t="str">
+        <x:v>本地商业目录；Sri Lanka Rainbow Pages 列出的公司邮箱；只有验证有效才纳入首选邮箱候选。 验证状态=3。; 人物补充：Danesh Weerarathne（Production Manager）；生产负责人，且公司精确匹配 Aqua Dynamics。</x:v>
+      </x:c>
+      <x:c r="AO40" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -4305,19 +4425,16 @@
         <x:v>IN</x:v>
       </x:c>
       <x:c r="G41" s="30" t="str">
-        <x:f>IF(V41&lt;&gt;"",V41,U41)</x:f>
         <x:v>commercial@specialty-films.com</x:v>
       </x:c>
       <x:c r="H41" s="30" t="str">
-        <x:f>IF(V41&lt;&gt;"","官网已验证",IF(ISNUMBER(SEARCH(":1",AB41)),"API已验证","未验证"))</x:f>
-        <x:v>API已验证</x:v>
-      </x:c>
-      <x:c r="I41" s="30" t="str">
-        <x:f>IF(X41&lt;&gt;"",X41,W41)</x:f>
-      </x:c>
+        <x:f>IF(ISNUMBER(SEARCH(":1",AC41)),"已验证有效",IF(ISNUMBER(SEARCH(":3",AC41)),"验证不确定",IF(ISNUMBER(SEARCH(":0",AC41)),"接口未能检测",IF(ISNUMBER(SEARCH(":2",AC41)),"判定无效",IF(V41&lt;&gt;"","官网已确认-未验证","无邮箱")))))</x:f>
+        <x:v>已验证有效</x:v>
+      </x:c>
+      <x:c r="I41" s="30" t="str"/>
       <x:c r="J41" s="30" t="str"/>
       <x:c r="K41" s="35" t="n">
-        <x:f>ROUND((IF(G41&lt;&gt;"",40,0)+IF(I41&lt;&gt;"",25,0)+IF(J41&lt;&gt;"",20,0)+IF(Z41&lt;&gt;"",15,0))/100,2)</x:f>
+        <x:f>ROUND((IF(H41="已验证有效",40,IF(V41&lt;&gt;"",20,0))+IF(ISNUMBER(SEARCH("状态1",Y41)),25,0)+IF(J41&lt;&gt;"",20,0)+IF(AA41&lt;&gt;"",15,0))/100,2)</x:f>
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="L41" s="30" t="str">
@@ -4352,31 +4469,32 @@
       <x:c r="Y41" s="30" t="str"/>
       <x:c r="Z41" s="30" t="str"/>
       <x:c r="AA41" s="30" t="str"/>
-      <x:c r="AB41" s="30" t="str">
+      <x:c r="AB41" s="30" t="str"/>
+      <x:c r="AC41" s="30" t="str">
         <x:v>commercial@specialty-films.com:1</x:v>
       </x:c>
-      <x:c r="AC41" s="30" t="str"/>
-      <x:c r="AD41" s="30" t="str">
+      <x:c r="AD41" s="30" t="str"/>
+      <x:c r="AE41" s="30" t="str">
         <x:v>print; masking film</x:v>
       </x:c>
-      <x:c r="AE41" s="30" t="str">
+      <x:c r="AF41" s="30" t="str">
         <x:v>MASKING FILM-PRINTED</x:v>
       </x:c>
-      <x:c r="AF41" s="30" t="str"/>
       <x:c r="AG41" s="30" t="str"/>
       <x:c r="AH41" s="30" t="str"/>
-      <x:c r="AI41" s="30" t="str">
+      <x:c r="AI41" s="30" t="str"/>
+      <x:c r="AJ41" s="30" t="str">
         <x:v>masking film</x:v>
       </x:c>
-      <x:c r="AJ41" s="30" t="str">
+      <x:c r="AK41" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
       </x:c>
-      <x:c r="AK41" s="30" t="str">
+      <x:c r="AL41" s="30" t="str">
         <x:v>UpKuajing customs company contact API</x:v>
       </x:c>
-      <x:c r="AL41" s="30" t="str"/>
       <x:c r="AM41" s="30" t="str"/>
-      <x:c r="AN41" s="34" t="n">
+      <x:c r="AN41" s="30" t="str"/>
+      <x:c r="AO41" s="34" t="n">
         <x:v>46220</x:v>
       </x:c>
     </x:row>
@@ -4392,15 +4510,15 @@
     <x:mergeCell ref="U3:X3"/>
     <x:mergeCell ref="Y3:AB3"/>
     <x:mergeCell ref="AC3:AF3"/>
-    <x:mergeCell ref="AG3:AN3"/>
-    <x:mergeCell ref="A4:AN4"/>
+    <x:mergeCell ref="AG3:AO3"/>
+    <x:mergeCell ref="A4:AO4"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B7:B41">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="高-欧美"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="H7:H41">
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="已验证"/>
-    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="未验证"/>
+    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="已验证有效"/>
+    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="验证不确定"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="K7:K41">
     <x:cfRule type="colorScale" priority="4">
@@ -4421,7 +4539,911 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2c0e7ec7b074538"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcffbd55c5bb846a1"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="66" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="38" t="str">
+        <x:v>有效联系方式成本与流程结论</x:v>
+      </x:c>
+      <x:c r="B1" s="38"/>
+      <x:c r="C1" s="38"/>
+      <x:c r="D1" s="38"/>
+      <x:c r="E1" s="38"/>
+      <x:c r="F1" s="38"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="40" t="str">
+        <x:v>指标</x:v>
+      </x:c>
+      <x:c r="B3" s="40" t="str">
+        <x:v>结果</x:v>
+      </x:c>
+      <x:c r="C3" s="40" t="str">
+        <x:v>严格口径</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="41" t="str">
+        <x:v>公司总数</x:v>
+      </x:c>
+      <x:c r="B4" s="41" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C4" s="41" t="str">
+        <x:v>一行一家公司ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="41" t="str">
+        <x:v>有已验证有效邮箱的公司</x:v>
+      </x:c>
+      <x:c r="B5" s="41" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="C5" s="41" t="str">
+        <x:v>邮箱状态=1；官网存在但投递性不确定不算</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="41" t="str">
+        <x:v>有已验证有效电话的公司</x:v>
+      </x:c>
+      <x:c r="B6" s="41" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="C6" s="41" t="str">
+        <x:v>电话状态=1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="41" t="str">
+        <x:v>至少一种有效联系方式</x:v>
+      </x:c>
+      <x:c r="B7" s="41" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C7" s="41" t="str">
+        <x:v>有效邮箱或有效电话</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="41" t="str">
+        <x:v>已验证有效邮箱地址</x:v>
+      </x:c>
+      <x:c r="B8" s="41" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C8" s="41" t="str">
+        <x:v>所有公司行内状态=1的邮箱地址数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="41" t="str">
+        <x:v>OpenAPI累计费用</x:v>
+      </x:c>
+      <x:c r="B9" s="42" t="n">
+        <x:v>81.6</x:v>
+      </x:c>
+      <x:c r="C9" s="41" t="str">
+        <x:v>人民币；已审计本项目全部调用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="41" t="str">
+        <x:v>每家有效邮箱公司成本</x:v>
+      </x:c>
+      <x:c r="B10" s="42" t="n">
+        <x:v>3.14</x:v>
+      </x:c>
+      <x:c r="C10" s="41" t="str">
+        <x:v>81.60 ÷ 26；主指标</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="41" t="str">
+        <x:v>每家有效联系方式成本</x:v>
+      </x:c>
+      <x:c r="B11" s="42" t="n">
+        <x:v>2.33</x:v>
+      </x:c>
+      <x:c r="C11" s="41" t="str">
+        <x:v>81.60 ÷ 35；邮箱或电话</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="41" t="str">
+        <x:v>预算剩余</x:v>
+      </x:c>
+      <x:c r="B12" s="42" t="n">
+        <x:v>18.4</x:v>
+      </x:c>
+      <x:c r="C12" s="41" t="str">
+        <x:v>100.00 - 81.60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="41"/>
+      <x:c r="B13" s="41"/>
+      <x:c r="C13" s="41"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="40" t="str">
+        <x:v>费用构成</x:v>
+      </x:c>
+      <x:c r="B14" s="40" t="str">
+        <x:v>金额（元）</x:v>
+      </x:c>
+      <x:c r="C14" s="40" t="str">
+        <x:v>说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="41" t="str">
+        <x:v>海关客户搜索</x:v>
+      </x:c>
+      <x:c r="B15" s="42" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="C15" s="41" t="str">
+        <x:v>产品买家搜索</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="41" t="str">
+        <x:v>海关公司联系方式</x:v>
+      </x:c>
+      <x:c r="B16" s="42" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="C16" s="41" t="str">
+        <x:v>早期35家公司及重复调用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="41" t="str">
+        <x:v>人物搜索</x:v>
+      </x:c>
+      <x:c r="B17" s="42" t="n">
+        <x:v>19.5</x:v>
+      </x:c>
+      <x:c r="C17" s="41" t="str">
+        <x:v>混合搜索1页 + 逐公司12页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="41" t="str">
+        <x:v>人物联系方式</x:v>
+      </x:c>
+      <x:c r="B18" s="42" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C18" s="41" t="str">
+        <x:v>人工审查后仅购买6人</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="41" t="str">
+        <x:v>邮箱验证</x:v>
+      </x:c>
+      <x:c r="B19" s="42" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C19" s="41" t="str">
+        <x:v>API、官网及人物新增邮箱</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="41" t="str">
+        <x:v>电话验证</x:v>
+      </x:c>
+      <x:c r="B20" s="42" t="n">
+        <x:v>6.6</x:v>
+      </x:c>
+      <x:c r="C20" s="41" t="str">
+        <x:v>主批58个 + 权威来源新增8个</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="41"/>
+      <x:c r="B21" s="41"/>
+      <x:c r="C21" s="41"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="40" t="str">
+        <x:v>流程改进</x:v>
+      </x:c>
+      <x:c r="B22" s="40" t="str">
+        <x:v>优先级</x:v>
+      </x:c>
+      <x:c r="C22" s="40" t="str">
+        <x:v>执行规则</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="41" t="str">
+        <x:v>先做法人实体去重</x:v>
+      </x:c>
+      <x:c r="B23" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C23" s="41" t="str">
+        <x:v>公司名称+官网域名+国家归一化；重复实体复用已验证联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="41" t="str">
+        <x:v>所有来源进入统一验证队列</x:v>
+      </x:c>
+      <x:c r="B24" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C24" s="41" t="str">
+        <x:v>API、官网、人物邮箱增量入库后立即验证；禁止只验API字段</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="41" t="str">
+        <x:v>人物搜索按公司逐个执行</x:v>
+      </x:c>
+      <x:c r="B25" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C25" s="41" t="str">
+        <x:v>人工确认公司精确匹配后，每家公司最多购买1位高相关人员</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="41" t="str">
+        <x:v>状态3/0不盲目重试</x:v>
+      </x:c>
+      <x:c r="B26" s="41" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C26" s="41" t="str">
+        <x:v>先查官网或换人物；避免反垃圾拦截导致重复付费</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="41" t="str">
+        <x:v>发送后用真实退信闭环</x:v>
+      </x:c>
+      <x:c r="B27" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C27" s="41" t="str">
+        <x:v>小批量投递、记录硬退信、永久抑制无效地址；验证状态1仍非送达保证</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="56" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="37" t="str">
+        <x:v>客户总表字段说明（按主表顺序）</x:v>
+      </x:c>
+      <x:c r="B1" s="37"/>
+      <x:c r="C1" s="37"/>
+      <x:c r="D1" s="37"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="40" t="str">
+        <x:v>字段</x:v>
+      </x:c>
+      <x:c r="B3" s="40" t="str">
+        <x:v>人话解释</x:v>
+      </x:c>
+      <x:c r="C3" s="40" t="str">
+        <x:v>来源/计算</x:v>
+      </x:c>
+      <x:c r="D3" s="40" t="str">
+        <x:v>是否关键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="41" t="str">
+        <x:v>研究状态</x:v>
+      </x:c>
+      <x:c r="B4" s="41" t="str">
+        <x:v>这家公司目前调研到哪一步</x:v>
+      </x:c>
+      <x:c r="C4" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D4" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="41" t="str">
+        <x:v>市场优先级</x:v>
+      </x:c>
+      <x:c r="B5" s="41" t="str">
+        <x:v>欧美优先或全球常规</x:v>
+      </x:c>
+      <x:c r="C5" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D5" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="41" t="str">
+        <x:v>品类</x:v>
+      </x:c>
+      <x:c r="B6" s="41" t="str">
+        <x:v>命中 tape 或 masking film</x:v>
+      </x:c>
+      <x:c r="C6" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D6" s="41" t="str">
+        <x:v>关键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="41" t="str">
+        <x:v>公司ID</x:v>
+      </x:c>
+      <x:c r="B7" s="41" t="str">
+        <x:v>跨境魔方中的公司唯一编号</x:v>
+      </x:c>
+      <x:c r="C7" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D7" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="41" t="str">
+        <x:v>公司名称</x:v>
+      </x:c>
+      <x:c r="B8" s="41" t="str">
+        <x:v>公司名称；一行只放一家</x:v>
+      </x:c>
+      <x:c r="C8" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D8" s="41" t="str">
+        <x:v>关键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="41" t="str">
+        <x:v>国家/地区</x:v>
+      </x:c>
+      <x:c r="B9" s="41" t="str">
+        <x:v>公司国家二字码</x:v>
+      </x:c>
+      <x:c r="C9" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D9" s="41" t="str">
+        <x:v>关键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="41" t="str">
+        <x:v>首选邮箱</x:v>
+      </x:c>
+      <x:c r="B10" s="41" t="str">
+        <x:v>优先取官网补充邮箱，否则取API/人物邮箱</x:v>
+      </x:c>
+      <x:c r="C10" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D10" s="41" t="str">
+        <x:v>关键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="41" t="str">
+        <x:v>邮箱可用状态</x:v>
+      </x:c>
+      <x:c r="B11" s="41" t="str">
+        <x:v>有效、无效、不确定或接口未能检测</x:v>
+      </x:c>
+      <x:c r="C11" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D11" s="41" t="str">
+        <x:v>关键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="41" t="str">
+        <x:v>首选电话</x:v>
+      </x:c>
+      <x:c r="B12" s="41" t="str">
+        <x:v>优先取官网电话，否则取API电话</x:v>
+      </x:c>
+      <x:c r="C12" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D12" s="41" t="str">
+        <x:v>关键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="41" t="str">
+        <x:v>官网</x:v>
+      </x:c>
+      <x:c r="B13" s="41" t="str">
+        <x:v>公司网站</x:v>
+      </x:c>
+      <x:c r="C13" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D13" s="41" t="str">
+        <x:v>关键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="41" t="str">
+        <x:v>联系完整度</x:v>
+      </x:c>
+      <x:c r="B14" s="41" t="str">
+        <x:v>按有效邮箱、有效电话、官网、社媒加权</x:v>
+      </x:c>
+      <x:c r="C14" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D14" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="41" t="str">
+        <x:v>跟进状态</x:v>
+      </x:c>
+      <x:c r="B15" s="41" t="str">
+        <x:v>人工维护的销售进度</x:v>
+      </x:c>
+      <x:c r="C15" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D15" s="41" t="str">
+        <x:v>关键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="41" t="str">
+        <x:v>负责人</x:v>
+      </x:c>
+      <x:c r="B16" s="41" t="str">
+        <x:v>人工填写跟进人</x:v>
+      </x:c>
+      <x:c r="C16" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D16" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="41" t="str">
+        <x:v>API地址</x:v>
+      </x:c>
+      <x:c r="B17" s="41" t="str">
+        <x:v>跨境魔方返回的公司地址</x:v>
+      </x:c>
+      <x:c r="C17" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D17" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="41" t="str">
+        <x:v>官网核验地址</x:v>
+      </x:c>
+      <x:c r="B18" s="41" t="str">
+        <x:v>官网或权威来源确认的地址</x:v>
+      </x:c>
+      <x:c r="C18" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D18" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="41" t="str">
+        <x:v>经营范围</x:v>
+      </x:c>
+      <x:c r="B19" s="41" t="str">
+        <x:v>公司经营或产品范围</x:v>
+      </x:c>
+      <x:c r="C19" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D19" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="41" t="str">
+        <x:v>匹配贸易次数</x:v>
+      </x:c>
+      <x:c r="B20" s="41" t="str">
+        <x:v>与本品类匹配的贸易记录数</x:v>
+      </x:c>
+      <x:c r="C20" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D20" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="41" t="str">
+        <x:v>贸易总次数</x:v>
+      </x:c>
+      <x:c r="B21" s="41" t="str">
+        <x:v>该公司全部贸易记录数</x:v>
+      </x:c>
+      <x:c r="C21" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D21" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="41" t="str">
+        <x:v>匹配占比</x:v>
+      </x:c>
+      <x:c r="B22" s="41" t="str">
+        <x:v>匹配贸易次数占总贸易次数</x:v>
+      </x:c>
+      <x:c r="C22" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D22" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="41" t="str">
+        <x:v>最近贸易日期</x:v>
+      </x:c>
+      <x:c r="B23" s="41" t="str">
+        <x:v>最近一笔相关贸易日期</x:v>
+      </x:c>
+      <x:c r="C23" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D23" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="41" t="str">
+        <x:v>API邮箱</x:v>
+      </x:c>
+      <x:c r="B24" s="41" t="str">
+        <x:v>海关公司API和审查后人物API获取的邮箱</x:v>
+      </x:c>
+      <x:c r="C24" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D24" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="41" t="str">
+        <x:v>官网补充邮箱</x:v>
+      </x:c>
+      <x:c r="B25" s="41" t="str">
+        <x:v>官网、政府或权威目录补充的邮箱</x:v>
+      </x:c>
+      <x:c r="C25" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D25" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="41" t="str">
+        <x:v>API电话</x:v>
+      </x:c>
+      <x:c r="B26" s="41" t="str">
+        <x:v>跨境魔方返回的电话</x:v>
+      </x:c>
+      <x:c r="C26" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D26" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="41" t="str">
+        <x:v>官网补充电话</x:v>
+      </x:c>
+      <x:c r="B27" s="41" t="str">
+        <x:v>官网、政府或权威目录补充的电话</x:v>
+      </x:c>
+      <x:c r="C27" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D27" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="41" t="str">
+        <x:v>电话验证详情</x:v>
+      </x:c>
+      <x:c r="B28" s="41" t="str">
+        <x:v>每个号码的有效状态、类型及WhatsApp状态</x:v>
+      </x:c>
+      <x:c r="C28" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D28" s="41" t="str">
+        <x:v>关键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="41" t="str">
+        <x:v>WhatsApp</x:v>
+      </x:c>
+      <x:c r="B29" s="41" t="str">
+        <x:v>明确识别的WhatsApp号码</x:v>
+      </x:c>
+      <x:c r="C29" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D29" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="41" t="str">
+        <x:v>社交媒体</x:v>
+      </x:c>
+      <x:c r="B30" s="41" t="str">
+        <x:v>LinkedIn等链接</x:v>
+      </x:c>
+      <x:c r="C30" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D30" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="41" t="str">
+        <x:v>官网联系渠道</x:v>
+      </x:c>
+      <x:c r="B31" s="41" t="str">
+        <x:v>官网表单、客服入口等</x:v>
+      </x:c>
+      <x:c r="C31" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D31" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="41" t="str">
+        <x:v>邮箱验证详情</x:v>
+      </x:c>
+      <x:c r="B32" s="41" t="str">
+        <x:v>每个邮箱及状态码；1有效、2无效、3不确定、0未能检测</x:v>
+      </x:c>
+      <x:c r="C32" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D32" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="41" t="str">
+        <x:v>产品名称</x:v>
+      </x:c>
+      <x:c r="B33" s="41" t="str">
+        <x:v>API结构化产品名</x:v>
+      </x:c>
+      <x:c r="C33" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D33" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="41" t="str">
+        <x:v>产品标签</x:v>
+      </x:c>
+      <x:c r="B34" s="41" t="str">
+        <x:v>API提取的产品关键词</x:v>
+      </x:c>
+      <x:c r="C34" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D34" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="41" t="str">
+        <x:v>产品描述/命中证据</x:v>
+      </x:c>
+      <x:c r="B35" s="41" t="str">
+        <x:v>原始报关品名；用于证明为何列入</x:v>
+      </x:c>
+      <x:c r="C35" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D35" s="41" t="str">
+        <x:v>关键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="41" t="str">
+        <x:v>产品别名</x:v>
+      </x:c>
+      <x:c r="B36" s="41" t="str">
+        <x:v>API返回的近义词</x:v>
+      </x:c>
+      <x:c r="C36" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D36" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="41" t="str">
+        <x:v>上游词</x:v>
+      </x:c>
+      <x:c r="B37" s="41" t="str">
+        <x:v>API返回的上游关联词</x:v>
+      </x:c>
+      <x:c r="C37" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D37" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="41" t="str">
+        <x:v>下游词</x:v>
+      </x:c>
+      <x:c r="B38" s="41" t="str">
+        <x:v>API返回的下游关联词</x:v>
+      </x:c>
+      <x:c r="C38" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D38" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="41" t="str">
+        <x:v>搜索词</x:v>
+      </x:c>
+      <x:c r="B39" s="41" t="str">
+        <x:v>找到该公司的查询词</x:v>
+      </x:c>
+      <x:c r="C39" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D39" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="41" t="str">
+        <x:v>搜索原始来源</x:v>
+      </x:c>
+      <x:c r="B40" s="41" t="str">
+        <x:v>对应原始搜索文件</x:v>
+      </x:c>
+      <x:c r="C40" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D40" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="41" t="str">
+        <x:v>API联系方式来源</x:v>
+      </x:c>
+      <x:c r="B41" s="41" t="str">
+        <x:v>联系方式来自哪个API</x:v>
+      </x:c>
+      <x:c r="C41" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D41" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="41" t="str">
+        <x:v>官网核验来源</x:v>
+      </x:c>
+      <x:c r="B42" s="41" t="str">
+        <x:v>核验网页或权威文件链接</x:v>
+      </x:c>
+      <x:c r="C42" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D42" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="41" t="str">
+        <x:v>官网核验说明</x:v>
+      </x:c>
+      <x:c r="B43" s="41" t="str">
+        <x:v>人工核验结论、人物职位和排除原因</x:v>
+      </x:c>
+      <x:c r="C43" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D43" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="41" t="str">
+        <x:v>最后核验日期</x:v>
+      </x:c>
+      <x:c r="B44" s="41" t="str">
+        <x:v>本行最后一次数据核验日期</x:v>
+      </x:c>
+      <x:c r="C44" s="41" t="str">
+        <x:v>API、官网或公式</x:v>
+      </x:c>
+      <x:c r="D44" s="41" t="str">
+        <x:v>辅助/追溯</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify valid email metrics and harden handoff
</commit_message>
<xml_diff>
--- a/deliverables/tape-masking-film-customer-master.xlsx
+++ b/deliverables/tape-masking-film-customer-master.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="Ra17befd378a0476e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本与流程" sheetId="2" r:id="R8bdb0886f8d2416b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R05c792e53b1b481f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="R3655c476312748f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本与流程" sheetId="2" r:id="Rad3f0a5f476d4200"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="Rda00b9b8b56f4db6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
     <x:numFmt numFmtId="203" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="204" formatCode="0%"/>
-    <x:numFmt numFmtId="205" formatCode="¥0.00"/>
+    <x:numFmt numFmtId="205" formatCode="&quot;¥&quot;#,##0.00"/>
   </x:numFmts>
   <x:fonts count="9">
     <x:font>
@@ -124,7 +124,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -215,8 +215,23 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -4539,7 +4554,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcffbd55c5bb846a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6ba128b26154fbc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4574,255 +4589,293 @@
         <x:v>严格口径</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="26" customHeight="1">
       <x:c r="A4" s="41" t="str">
         <x:v>公司总数</x:v>
       </x:c>
-      <x:c r="B4" s="41" t="n">
+      <x:c r="B4" s="44" t="n">
         <x:v>35</x:v>
       </x:c>
       <x:c r="C4" s="41" t="str">
         <x:v>一行一家公司ID</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="26" customHeight="1">
       <x:c r="A5" s="41" t="str">
-        <x:v>有已验证有效邮箱的公司</x:v>
-      </x:c>
-      <x:c r="B5" s="41" t="n">
+        <x:v>拥有有效邮箱的公司</x:v>
+      </x:c>
+      <x:c r="B5" s="44" t="n">
         <x:v>26</x:v>
       </x:c>
       <x:c r="C5" s="41" t="str">
-        <x:v>邮箱状态=1；官网存在但投递性不确定不算</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
+        <x:v>每家公司至少有1个状态=1的邮箱；核心获客指标</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26" customHeight="1">
       <x:c r="A6" s="41" t="str">
+        <x:v>去重后的有效邮箱地址</x:v>
+      </x:c>
+      <x:c r="B6" s="44" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="C6" s="41" t="str">
+        <x:v>按邮箱文本跨公司去重；同一邮箱重复出现只算1个</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26" customHeight="1">
+      <x:c r="A7" s="41" t="str">
+        <x:v>公司—邮箱有效关联记录</x:v>
+      </x:c>
+      <x:c r="B7" s="44" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C7" s="41" t="str">
+        <x:v>公司行内状态=1的关联数，未跨公司去重；仅供数据审计</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="26" customHeight="1">
+      <x:c r="A8" s="41" t="str">
         <x:v>有已验证有效电话的公司</x:v>
       </x:c>
-      <x:c r="B6" s="41" t="n">
+      <x:c r="B8" s="44" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="C6" s="41" t="str">
+      <x:c r="C8" s="41" t="str">
         <x:v>电话状态=1</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="41" t="str">
+    <x:row r="9" ht="26" customHeight="1">
+      <x:c r="A9" s="41" t="str">
         <x:v>至少一种有效联系方式</x:v>
       </x:c>
-      <x:c r="B7" s="41" t="n">
+      <x:c r="B9" s="44" t="n">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="C7" s="41" t="str">
+      <x:c r="C9" s="41" t="str">
         <x:v>有效邮箱或有效电话</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="41" t="str">
-        <x:v>已验证有效邮箱地址</x:v>
-      </x:c>
-      <x:c r="B8" s="41" t="n">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="C8" s="41" t="str">
-        <x:v>所有公司行内状态=1的邮箱地址数</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="41" t="str">
+    <x:row r="10" ht="26" customHeight="1">
+      <x:c r="A10" s="41" t="str">
         <x:v>OpenAPI累计费用</x:v>
       </x:c>
-      <x:c r="B9" s="42" t="n">
+      <x:c r="B10" s="45" t="n">
         <x:v>81.6</x:v>
       </x:c>
-      <x:c r="C9" s="41" t="str">
+      <x:c r="C10" s="41" t="str">
         <x:v>人民币；已审计本项目全部调用</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="41" t="str">
-        <x:v>每家有效邮箱公司成本</x:v>
-      </x:c>
-      <x:c r="B10" s="42" t="n">
+    <x:row r="11" ht="26" customHeight="1">
+      <x:c r="A11" s="41" t="str">
+        <x:v>每家拥有有效邮箱的公司成本</x:v>
+      </x:c>
+      <x:c r="B11" s="45" t="n">
+        <x:f>ROUND(B10/B5,2)</x:f>
         <x:v>3.14</x:v>
       </x:c>
-      <x:c r="C10" s="41" t="str">
-        <x:v>81.60 ÷ 26；主指标</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="41" t="str">
+      <x:c r="C11" s="41" t="str">
+        <x:v>累计费用 ÷ 拥有有效邮箱的公司；核心获客成本</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26" customHeight="1">
+      <x:c r="A12" s="41" t="str">
+        <x:v>每个去重有效邮箱成本</x:v>
+      </x:c>
+      <x:c r="B12" s="45" t="n">
+        <x:f>ROUND(B10/B6,2)</x:f>
+        <x:v>2.91</x:v>
+      </x:c>
+      <x:c r="C12" s="41" t="str">
+        <x:v>累计费用 ÷ 去重邮箱数；按独立邮箱地址计算</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26" customHeight="1">
+      <x:c r="A13" s="41" t="str">
+        <x:v>每条公司—邮箱关联成本</x:v>
+      </x:c>
+      <x:c r="B13" s="45" t="n">
+        <x:f>ROUND(B10/B7,2)</x:f>
+        <x:v>2.63</x:v>
+      </x:c>
+      <x:c r="C13" s="41" t="str">
+        <x:v>累计费用 ÷ 关联记录数；技术统计，不代表独立邮箱数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26" customHeight="1">
+      <x:c r="A14" s="41" t="str">
         <x:v>每家有效联系方式成本</x:v>
       </x:c>
-      <x:c r="B11" s="42" t="n">
+      <x:c r="B14" s="45" t="n">
+        <x:f>ROUND(B10/B9,2)</x:f>
         <x:v>2.33</x:v>
       </x:c>
-      <x:c r="C11" s="41" t="str">
-        <x:v>81.60 ÷ 35；邮箱或电话</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="41" t="str">
+      <x:c r="C14" s="41" t="str">
+        <x:v>累计费用 ÷ 至少一种有效联系方式的公司</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="26" customHeight="1">
+      <x:c r="A15" s="41" t="str">
         <x:v>预算剩余</x:v>
       </x:c>
-      <x:c r="B12" s="42" t="n">
+      <x:c r="B15" s="45" t="n">
+        <x:f>ROUND(100-B10,2)</x:f>
         <x:v>18.4</x:v>
       </x:c>
-      <x:c r="C12" s="41" t="str">
-        <x:v>100.00 - 81.60</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="41"/>
-      <x:c r="B13" s="41"/>
-      <x:c r="C13" s="41"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="40" t="str">
+      <x:c r="C15" s="41" t="str">
+        <x:v>¥100.00 - 累计费用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="41"/>
+      <x:c r="B16" s="46"/>
+      <x:c r="C16" s="41"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="40" t="str">
         <x:v>费用构成</x:v>
       </x:c>
-      <x:c r="B14" s="40" t="str">
+      <x:c r="B17" s="47" t="str">
         <x:v>金额（元）</x:v>
       </x:c>
-      <x:c r="C14" s="40" t="str">
+      <x:c r="C17" s="40" t="str">
         <x:v>说明</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="41" t="str">
-        <x:v>海关客户搜索</x:v>
-      </x:c>
-      <x:c r="B15" s="42" t="n">
-        <x:v>7.5</x:v>
-      </x:c>
-      <x:c r="C15" s="41" t="str">
-        <x:v>产品买家搜索</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="41" t="str">
-        <x:v>海关公司联系方式</x:v>
-      </x:c>
-      <x:c r="B16" s="42" t="n">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="C16" s="41" t="str">
-        <x:v>早期35家公司及重复调用</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="41" t="str">
-        <x:v>人物搜索</x:v>
-      </x:c>
-      <x:c r="B17" s="42" t="n">
-        <x:v>19.5</x:v>
-      </x:c>
-      <x:c r="C17" s="41" t="str">
-        <x:v>混合搜索1页 + 逐公司12页</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="41" t="str">
-        <x:v>人物联系方式</x:v>
-      </x:c>
-      <x:c r="B18" s="42" t="n">
-        <x:v>3</x:v>
+        <x:v>海关客户搜索</x:v>
+      </x:c>
+      <x:c r="B18" s="45" t="n">
+        <x:v>7.5</x:v>
       </x:c>
       <x:c r="C18" s="41" t="str">
-        <x:v>人工审查后仅购买6人</x:v>
+        <x:v>产品买家搜索</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="41" t="str">
-        <x:v>邮箱验证</x:v>
-      </x:c>
-      <x:c r="B19" s="42" t="n">
-        <x:v>3</x:v>
+        <x:v>海关公司联系方式</x:v>
+      </x:c>
+      <x:c r="B19" s="45" t="n">
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C19" s="41" t="str">
-        <x:v>API、官网及人物新增邮箱</x:v>
+        <x:v>早期35家公司及重复调用</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="41" t="str">
-        <x:v>电话验证</x:v>
-      </x:c>
-      <x:c r="B20" s="42" t="n">
-        <x:v>6.6</x:v>
+        <x:v>人物搜索</x:v>
+      </x:c>
+      <x:c r="B20" s="45" t="n">
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="C20" s="41" t="str">
-        <x:v>主批58个 + 权威来源新增8个</x:v>
+        <x:v>混合搜索1页 + 逐公司12页</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="41"/>
-      <x:c r="B21" s="41"/>
-      <x:c r="C21" s="41"/>
+      <x:c r="A21" s="41" t="str">
+        <x:v>人物联系方式</x:v>
+      </x:c>
+      <x:c r="B21" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C21" s="41" t="str">
+        <x:v>人工审查后仅购买6人</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="40" t="str">
-        <x:v>流程改进</x:v>
-      </x:c>
-      <x:c r="B22" s="40" t="str">
-        <x:v>优先级</x:v>
-      </x:c>
-      <x:c r="C22" s="40" t="str">
-        <x:v>执行规则</x:v>
+      <x:c r="A22" s="41" t="str">
+        <x:v>邮箱验证</x:v>
+      </x:c>
+      <x:c r="B22" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C22" s="41" t="str">
+        <x:v>API、官网及人物新增邮箱</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="41" t="str">
-        <x:v>先做法人实体去重</x:v>
-      </x:c>
-      <x:c r="B23" s="41" t="str">
-        <x:v>P0</x:v>
+        <x:v>电话验证</x:v>
+      </x:c>
+      <x:c r="B23" s="45" t="n">
+        <x:v>6.6</x:v>
       </x:c>
       <x:c r="C23" s="41" t="str">
-        <x:v>公司名称+官网域名+国家归一化；重复实体复用已验证联系方式</x:v>
+        <x:v>主批58个 + 权威来源新增8个</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="41" t="str">
-        <x:v>所有来源进入统一验证队列</x:v>
-      </x:c>
-      <x:c r="B24" s="41" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C24" s="41" t="str">
-        <x:v>API、官网、人物邮箱增量入库后立即验证；禁止只验API字段</x:v>
-      </x:c>
+      <x:c r="A24" s="41"/>
+      <x:c r="B24" s="41"/>
+      <x:c r="C24" s="41"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="41" t="str">
-        <x:v>人物搜索按公司逐个执行</x:v>
-      </x:c>
-      <x:c r="B25" s="41" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C25" s="41" t="str">
-        <x:v>人工确认公司精确匹配后，每家公司最多购买1位高相关人员</x:v>
+      <x:c r="A25" s="40" t="str">
+        <x:v>流程改进</x:v>
+      </x:c>
+      <x:c r="B25" s="40" t="str">
+        <x:v>优先级</x:v>
+      </x:c>
+      <x:c r="C25" s="40" t="str">
+        <x:v>执行规则</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="41" t="str">
-        <x:v>状态3/0不盲目重试</x:v>
+        <x:v>先做法人实体去重</x:v>
       </x:c>
       <x:c r="B26" s="41" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C26" s="41" t="str">
-        <x:v>先查官网或换人物；避免反垃圾拦截导致重复付费</x:v>
+        <x:v>公司名称+官网域名+国家归一化；重复实体复用已验证联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="41" t="str">
-        <x:v>发送后用真实退信闭环</x:v>
+        <x:v>所有来源进入统一验证队列</x:v>
       </x:c>
       <x:c r="B27" s="41" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C27" s="41" t="str">
+        <x:v>API、官网、人物邮箱增量入库后立即验证；禁止只验API字段</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="41" t="str">
+        <x:v>人物搜索按公司逐个执行</x:v>
+      </x:c>
+      <x:c r="B28" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C28" s="41" t="str">
+        <x:v>人工确认公司精确匹配后，每家公司最多购买1位高相关人员</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="41" t="str">
+        <x:v>状态3/0不盲目重试</x:v>
+      </x:c>
+      <x:c r="B29" s="41" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C29" s="41" t="str">
+        <x:v>先查官网或换人物；避免反垃圾拦截导致重复付费</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="41" t="str">
+        <x:v>发送后用真实退信闭环</x:v>
+      </x:c>
+      <x:c r="B30" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C30" s="41" t="str">
         <x:v>小批量投递、记录硬退信、永久抑制无效地址；验证状态1仍非送达保证</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Use company-level contact coverage metrics
</commit_message>
<xml_diff>
--- a/deliverables/tape-masking-film-customer-master.xlsx
+++ b/deliverables/tape-masking-film-customer-master.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="R3655c476312748f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本与流程" sheetId="2" r:id="Rad3f0a5f476d4200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="Rda00b9b8b56f4db6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="R23d17af5de9548a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本与流程" sheetId="2" r:id="R5fb2f0b64c5c4388"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="Rd11019b04c2d4f7f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -666,14 +666,14 @@
       <x:c r="G3" s="16"/>
       <x:c r="H3" s="16"/>
       <x:c r="I3" s="15" t="str">
-        <x:v>欧美优先</x:v>
+        <x:v>有效联系方式公司</x:v>
       </x:c>
       <x:c r="J3" s="15"/>
       <x:c r="K3" s="15"/>
       <x:c r="L3" s="15"/>
       <x:c r="M3" s="16" t="n">
-        <x:f>COUNTIF(B7:B41,"高-欧美")</x:f>
-        <x:v>5</x:v>
+        <x:f>'成本与流程'!B5</x:f>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="N3" s="16"/>
       <x:c r="O3" s="16"/>
@@ -4554,7 +4554,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6ba128b26154fbc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R886d1018b9d94528"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4570,7 +4570,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="38" t="str">
-        <x:v>有效联系方式成本与流程结论</x:v>
+        <x:v>公司级有效联系方式成本与流程结论</x:v>
       </x:c>
       <x:c r="B1" s="38"/>
       <x:c r="C1" s="38"/>
@@ -4602,280 +4602,328 @@
     </x:row>
     <x:row r="5" ht="26" customHeight="1">
       <x:c r="A5" s="41" t="str">
-        <x:v>拥有有效邮箱的公司</x:v>
+        <x:v>拥有至少一种有效联系方式的公司</x:v>
       </x:c>
       <x:c r="B5" s="44" t="n">
-        <x:v>26</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C5" s="41" t="str">
-        <x:v>每家公司至少有1个状态=1的邮箱；核心获客指标</x:v>
+        <x:v>至少1个状态=1的邮箱或电话；核心总业务指标</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26" customHeight="1">
       <x:c r="A6" s="41" t="str">
-        <x:v>去重后的有效邮箱地址</x:v>
+        <x:v>拥有有效邮箱的公司</x:v>
       </x:c>
       <x:c r="B6" s="44" t="n">
-        <x:v>28</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C6" s="41" t="str">
-        <x:v>按邮箱文本跨公司去重；同一邮箱重复出现只算1个</x:v>
+        <x:v>至少1个状态=1的邮箱；不按邮箱数量重复计算</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="26" customHeight="1">
       <x:c r="A7" s="41" t="str">
-        <x:v>公司—邮箱有效关联记录</x:v>
+        <x:v>拥有有效电话的公司</x:v>
       </x:c>
       <x:c r="B7" s="44" t="n">
-        <x:v>31</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C7" s="41" t="str">
-        <x:v>公司行内状态=1的关联数，未跨公司去重；仅供数据审计</x:v>
+        <x:v>至少1个状态=1的电话；不按电话数量重复计算</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26" customHeight="1">
       <x:c r="A8" s="41" t="str">
-        <x:v>有已验证有效电话的公司</x:v>
+        <x:v>邮箱和电话都有的公司</x:v>
       </x:c>
       <x:c r="B8" s="44" t="n">
-        <x:v>28</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C8" s="41" t="str">
-        <x:v>电话状态=1</x:v>
+        <x:v>同时计入邮箱公司和电话公司</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
       <x:c r="A9" s="41" t="str">
-        <x:v>至少一种有效联系方式</x:v>
+        <x:v>只有有效邮箱的公司</x:v>
       </x:c>
       <x:c r="B9" s="44" t="n">
-        <x:v>35</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C9" s="41" t="str">
-        <x:v>有效邮箱或有效电话</x:v>
+        <x:v>有有效邮箱、无有效电话</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="26" customHeight="1">
       <x:c r="A10" s="41" t="str">
-        <x:v>OpenAPI累计费用</x:v>
-      </x:c>
-      <x:c r="B10" s="45" t="n">
-        <x:v>81.6</x:v>
+        <x:v>只有有效电话的公司</x:v>
+      </x:c>
+      <x:c r="B10" s="44" t="n">
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C10" s="41" t="str">
-        <x:v>人民币；已审计本项目全部调用</x:v>
+        <x:v>无有效邮箱、有有效电话</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26" customHeight="1">
       <x:c r="A11" s="41" t="str">
-        <x:v>每家拥有有效邮箱的公司成本</x:v>
-      </x:c>
-      <x:c r="B11" s="45" t="n">
-        <x:f>ROUND(B10/B5,2)</x:f>
-        <x:v>3.14</x:v>
+        <x:v>两者都没有的公司</x:v>
+      </x:c>
+      <x:c r="B11" s="44" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C11" s="41" t="str">
-        <x:v>累计费用 ÷ 拥有有效邮箱的公司；核心获客成本</x:v>
+        <x:v>无状态=1的邮箱，也无状态=1的电话</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="26" customHeight="1">
       <x:c r="A12" s="41" t="str">
-        <x:v>每个去重有效邮箱成本</x:v>
+        <x:v>OpenAPI累计费用</x:v>
       </x:c>
       <x:c r="B12" s="45" t="n">
-        <x:f>ROUND(B10/B6,2)</x:f>
-        <x:v>2.91</x:v>
+        <x:v>81.6</x:v>
       </x:c>
       <x:c r="C12" s="41" t="str">
-        <x:v>累计费用 ÷ 去重邮箱数；按独立邮箱地址计算</x:v>
+        <x:v>人民币；已审计本项目全部调用</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="26" customHeight="1">
       <x:c r="A13" s="41" t="str">
-        <x:v>每条公司—邮箱关联成本</x:v>
+        <x:v>每家有效联系方式公司成本</x:v>
       </x:c>
       <x:c r="B13" s="45" t="n">
-        <x:f>ROUND(B10/B7,2)</x:f>
-        <x:v>2.63</x:v>
+        <x:f>ROUND(B12/B5,2)</x:f>
+        <x:v>2.33</x:v>
       </x:c>
       <x:c r="C13" s="41" t="str">
-        <x:v>累计费用 ÷ 关联记录数；技术统计，不代表独立邮箱数</x:v>
+        <x:v>累计费用 ÷ 拥有至少一种有效联系方式的公司</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="26" customHeight="1">
       <x:c r="A14" s="41" t="str">
-        <x:v>每家有效联系方式成本</x:v>
+        <x:v>每家有效邮箱公司成本</x:v>
       </x:c>
       <x:c r="B14" s="45" t="n">
-        <x:f>ROUND(B10/B9,2)</x:f>
-        <x:v>2.33</x:v>
+        <x:f>ROUND(B12/B6,2)</x:f>
+        <x:v>3.14</x:v>
       </x:c>
       <x:c r="C14" s="41" t="str">
-        <x:v>累计费用 ÷ 至少一种有效联系方式的公司</x:v>
+        <x:v>累计费用 ÷ 拥有有效邮箱的公司</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
       <x:c r="A15" s="41" t="str">
+        <x:v>每家有效电话公司成本</x:v>
+      </x:c>
+      <x:c r="B15" s="45" t="n">
+        <x:f>ROUND(B12/B7,2)</x:f>
+        <x:v>2.91</x:v>
+      </x:c>
+      <x:c r="C15" s="41" t="str">
+        <x:v>累计费用 ÷ 拥有有效电话的公司</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="26" customHeight="1">
+      <x:c r="A16" s="41" t="str">
         <x:v>预算剩余</x:v>
       </x:c>
-      <x:c r="B15" s="45" t="n">
-        <x:f>ROUND(100-B10,2)</x:f>
+      <x:c r="B16" s="45" t="n">
+        <x:f>ROUND(100-B12,2)</x:f>
         <x:v>18.4</x:v>
       </x:c>
-      <x:c r="C15" s="41" t="str">
+      <x:c r="C16" s="41" t="str">
         <x:v>¥100.00 - 累计费用</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="41"/>
-      <x:c r="B16" s="46"/>
-      <x:c r="C16" s="41"/>
-    </x:row>
     <x:row r="17">
-      <x:c r="A17" s="40" t="str">
-        <x:v>费用构成</x:v>
-      </x:c>
-      <x:c r="B17" s="47" t="str">
-        <x:v>金额（元）</x:v>
-      </x:c>
-      <x:c r="C17" s="40" t="str">
+      <x:c r="A17" s="41"/>
+      <x:c r="B17" s="46"/>
+      <x:c r="C17" s="41"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="40" t="str">
+        <x:v>邮箱技术审计</x:v>
+      </x:c>
+      <x:c r="B18" s="47" t="str">
+        <x:v>数量</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="str">
         <x:v>说明</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="41" t="str">
-        <x:v>海关客户搜索</x:v>
-      </x:c>
-      <x:c r="B18" s="45" t="n">
-        <x:v>7.5</x:v>
-      </x:c>
-      <x:c r="C18" s="41" t="str">
-        <x:v>产品买家搜索</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="41" t="str">
-        <x:v>海关公司联系方式</x:v>
-      </x:c>
-      <x:c r="B19" s="45" t="n">
-        <x:v>42</x:v>
+        <x:v>去重后的有效邮箱地址</x:v>
+      </x:c>
+      <x:c r="B19" s="44" t="n">
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C19" s="41" t="str">
-        <x:v>早期35家公司及重复调用</x:v>
+        <x:v>按邮箱文本跨公司去重；不是公司级业务指标</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="41" t="str">
-        <x:v>人物搜索</x:v>
-      </x:c>
-      <x:c r="B20" s="45" t="n">
-        <x:v>19.5</x:v>
+        <x:v>公司—邮箱有效关联记录</x:v>
+      </x:c>
+      <x:c r="B20" s="44" t="n">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C20" s="41" t="str">
-        <x:v>混合搜索1页 + 逐公司12页</x:v>
+        <x:v>未跨公司去重；仅供数据审计</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="41" t="str">
-        <x:v>人物联系方式</x:v>
-      </x:c>
-      <x:c r="B21" s="45" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C21" s="41" t="str">
-        <x:v>人工审查后仅购买6人</x:v>
-      </x:c>
+      <x:c r="A21" s="41"/>
+      <x:c r="B21" s="46"/>
+      <x:c r="C21" s="41"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="41" t="str">
-        <x:v>邮箱验证</x:v>
-      </x:c>
-      <x:c r="B22" s="45" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C22" s="41" t="str">
-        <x:v>API、官网及人物新增邮箱</x:v>
+      <x:c r="A22" s="40" t="str">
+        <x:v>费用构成</x:v>
+      </x:c>
+      <x:c r="B22" s="47" t="str">
+        <x:v>金额（元）</x:v>
+      </x:c>
+      <x:c r="C22" s="40" t="str">
+        <x:v>说明</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="41" t="str">
-        <x:v>电话验证</x:v>
+        <x:v>海关客户搜索</x:v>
       </x:c>
       <x:c r="B23" s="45" t="n">
-        <x:v>6.6</x:v>
+        <x:v>7.5</x:v>
       </x:c>
       <x:c r="C23" s="41" t="str">
-        <x:v>主批58个 + 权威来源新增8个</x:v>
+        <x:v>产品买家搜索</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="41"/>
-      <x:c r="B24" s="41"/>
-      <x:c r="C24" s="41"/>
+      <x:c r="A24" s="41" t="str">
+        <x:v>海关公司联系方式</x:v>
+      </x:c>
+      <x:c r="B24" s="45" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="C24" s="41" t="str">
+        <x:v>早期35家公司及重复调用</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="40" t="str">
-        <x:v>流程改进</x:v>
-      </x:c>
-      <x:c r="B25" s="40" t="str">
-        <x:v>优先级</x:v>
-      </x:c>
-      <x:c r="C25" s="40" t="str">
-        <x:v>执行规则</x:v>
+      <x:c r="A25" s="41" t="str">
+        <x:v>人物搜索</x:v>
+      </x:c>
+      <x:c r="B25" s="45" t="n">
+        <x:v>19.5</x:v>
+      </x:c>
+      <x:c r="C25" s="41" t="str">
+        <x:v>混合搜索1页 + 逐公司12页</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="41" t="str">
-        <x:v>先做法人实体去重</x:v>
-      </x:c>
-      <x:c r="B26" s="41" t="str">
-        <x:v>P0</x:v>
+        <x:v>人物联系方式</x:v>
+      </x:c>
+      <x:c r="B26" s="45" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C26" s="41" t="str">
-        <x:v>公司名称+官网域名+国家归一化；重复实体复用已验证联系方式</x:v>
+        <x:v>人工审查后仅购买6人</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="41" t="str">
-        <x:v>所有来源进入统一验证队列</x:v>
-      </x:c>
-      <x:c r="B27" s="41" t="str">
-        <x:v>P0</x:v>
+        <x:v>邮箱验证</x:v>
+      </x:c>
+      <x:c r="B27" s="45" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C27" s="41" t="str">
-        <x:v>API、官网、人物邮箱增量入库后立即验证；禁止只验API字段</x:v>
+        <x:v>API、官网及人物新增邮箱</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="41" t="str">
+        <x:v>电话验证</x:v>
+      </x:c>
+      <x:c r="B28" s="45" t="n">
+        <x:v>6.6</x:v>
+      </x:c>
+      <x:c r="C28" s="41" t="str">
+        <x:v>主批58个 + 权威来源新增8个</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="41"/>
+      <x:c r="B29" s="41"/>
+      <x:c r="C29" s="41"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="40" t="str">
+        <x:v>流程改进</x:v>
+      </x:c>
+      <x:c r="B30" s="40" t="str">
+        <x:v>优先级</x:v>
+      </x:c>
+      <x:c r="C30" s="40" t="str">
+        <x:v>执行规则</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="41" t="str">
+        <x:v>先做法人实体去重</x:v>
+      </x:c>
+      <x:c r="B31" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C31" s="41" t="str">
+        <x:v>公司名称+官网域名+国家归一化；重复实体复用已验证联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="41" t="str">
+        <x:v>所有来源进入统一验证队列</x:v>
+      </x:c>
+      <x:c r="B32" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C32" s="41" t="str">
+        <x:v>API、官网、人物邮箱增量入库后立即验证；禁止只验API字段</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="41" t="str">
         <x:v>人物搜索按公司逐个执行</x:v>
       </x:c>
-      <x:c r="B28" s="41" t="str">
+      <x:c r="B33" s="41" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C28" s="41" t="str">
+      <x:c r="C33" s="41" t="str">
         <x:v>人工确认公司精确匹配后，每家公司最多购买1位高相关人员</x:v>
       </x:c>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="41" t="str">
+    <x:row r="34">
+      <x:c r="A34" s="41" t="str">
         <x:v>状态3/0不盲目重试</x:v>
       </x:c>
-      <x:c r="B29" s="41" t="str">
+      <x:c r="B34" s="41" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="C29" s="41" t="str">
+      <x:c r="C34" s="41" t="str">
         <x:v>先查官网或换人物；避免反垃圾拦截导致重复付费</x:v>
       </x:c>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="41" t="str">
+    <x:row r="35">
+      <x:c r="A35" s="41" t="str">
         <x:v>发送后用真实退信闭环</x:v>
       </x:c>
-      <x:c r="B30" s="41" t="str">
+      <x:c r="B35" s="41" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C30" s="41" t="str">
+      <x:c r="C35" s="41" t="str">
         <x:v>小批量投递、记录硬退信、永久抑制无效地址；验证状态1仍非送达保证</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Localize customer workbook fields to Chinese
</commit_message>
<xml_diff>
--- a/deliverables/tape-masking-film-customer-master.xlsx
+++ b/deliverables/tape-masking-film-customer-master.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="R23d17af5de9548a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本与流程" sheetId="2" r:id="R5fb2f0b64c5c4388"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="Rd11019b04c2d4f7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="R261df0f1ac154483"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本与流程" sheetId="2" r:id="Rf05eafd48cbd4fce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R701f027fb43341e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -279,10 +279,10 @@
   <x:tableColumns count="41">
     <x:tableColumn id="1" name="研究状态"/>
     <x:tableColumn id="2" name="市场优先级"/>
-    <x:tableColumn id="3" name="品类"/>
+    <x:tableColumn id="3" name="产品品类（中文）"/>
     <x:tableColumn id="4" name="公司ID"/>
     <x:tableColumn id="5" name="公司名称"/>
-    <x:tableColumn id="6" name="国家/地区"/>
+    <x:tableColumn id="6" name="国家/地区（中文）"/>
     <x:tableColumn id="7" name="首选邮箱"/>
     <x:tableColumn id="8" name="邮箱可用状态"/>
     <x:tableColumn id="9" name="首选电话"/>
@@ -290,9 +290,9 @@
     <x:tableColumn id="11" name="联系完整度"/>
     <x:tableColumn id="12" name="跟进状态"/>
     <x:tableColumn id="13" name="负责人"/>
-    <x:tableColumn id="14" name="API地址"/>
-    <x:tableColumn id="15" name="官网核验地址"/>
-    <x:tableColumn id="16" name="经营范围"/>
+    <x:tableColumn id="14" name="API地址（原文）"/>
+    <x:tableColumn id="15" name="官网核验地址（原文）"/>
+    <x:tableColumn id="16" name="经营范围（原文）"/>
     <x:tableColumn id="17" name="匹配贸易次数"/>
     <x:tableColumn id="18" name="贸易总次数"/>
     <x:tableColumn id="19" name="匹配占比"/>
@@ -308,11 +308,11 @@
     <x:tableColumn id="29" name="邮箱验证详情"/>
     <x:tableColumn id="30" name="产品名称"/>
     <x:tableColumn id="31" name="产品标签"/>
-    <x:tableColumn id="32" name="产品描述/命中证据"/>
+    <x:tableColumn id="32" name="报关品名/命中证据（原文）"/>
     <x:tableColumn id="33" name="产品别名"/>
     <x:tableColumn id="34" name="上游词"/>
     <x:tableColumn id="35" name="下游词"/>
-    <x:tableColumn id="36" name="搜索词"/>
+    <x:tableColumn id="36" name="搜索词（中文）"/>
     <x:tableColumn id="37" name="搜索原始来源"/>
     <x:tableColumn id="38" name="API联系方式来源"/>
     <x:tableColumn id="39" name="官网核验来源"/>
@@ -563,7 +563,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="7" t="str">
-        <x:v>Tape &amp; Masking Film 全球客户总表</x:v>
+        <x:v>胶带与遮蔽膜全球客户总表</x:v>
       </x:c>
       <x:c r="B1" s="7"/>
       <x:c r="C1" s="7"/>
@@ -769,7 +769,7 @@
         <x:v>市场优先级</x:v>
       </x:c>
       <x:c r="C6" s="27" t="str">
-        <x:v>品类</x:v>
+        <x:v>产品品类（中文）</x:v>
       </x:c>
       <x:c r="D6" s="27" t="str">
         <x:v>公司ID</x:v>
@@ -778,7 +778,7 @@
         <x:v>公司名称</x:v>
       </x:c>
       <x:c r="F6" s="27" t="str">
-        <x:v>国家/地区</x:v>
+        <x:v>国家/地区（中文）</x:v>
       </x:c>
       <x:c r="G6" s="27" t="str">
         <x:v>首选邮箱</x:v>
@@ -802,13 +802,13 @@
         <x:v>负责人</x:v>
       </x:c>
       <x:c r="N6" s="27" t="str">
-        <x:v>API地址</x:v>
+        <x:v>API地址（原文）</x:v>
       </x:c>
       <x:c r="O6" s="27" t="str">
-        <x:v>官网核验地址</x:v>
+        <x:v>官网核验地址（原文）</x:v>
       </x:c>
       <x:c r="P6" s="27" t="str">
-        <x:v>经营范围</x:v>
+        <x:v>经营范围（原文）</x:v>
       </x:c>
       <x:c r="Q6" s="27" t="str">
         <x:v>匹配贸易次数</x:v>
@@ -856,7 +856,7 @@
         <x:v>产品标签</x:v>
       </x:c>
       <x:c r="AF6" s="27" t="str">
-        <x:v>产品描述/命中证据</x:v>
+        <x:v>报关品名/命中证据（原文）</x:v>
       </x:c>
       <x:c r="AG6" s="27" t="str">
         <x:v>产品别名</x:v>
@@ -868,7 +868,7 @@
         <x:v>下游词</x:v>
       </x:c>
       <x:c r="AJ6" s="27" t="str">
-        <x:v>搜索词</x:v>
+        <x:v>搜索词（中文）</x:v>
       </x:c>
       <x:c r="AK6" s="27" t="str">
         <x:v>搜索原始来源</x:v>
@@ -894,7 +894,7 @@
         <x:v>高-欧美</x:v>
       </x:c>
       <x:c r="C7" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D7" s="31" t="str">
         <x:v>71462461</x:v>
@@ -903,7 +903,7 @@
         <x:v>POLI-FILM AMERICA INC.</x:v>
       </x:c>
       <x:c r="F7" s="30" t="str">
-        <x:v>GB</x:v>
+        <x:v>英国</x:v>
       </x:c>
       <x:c r="G7" s="30" t="str">
         <x:v>echrisman@polifilm.us</x:v>
@@ -961,7 +961,7 @@
       <x:c r="AH7" s="30" t="str"/>
       <x:c r="AI7" s="30" t="str"/>
       <x:c r="AJ7" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK7" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -983,7 +983,7 @@
         <x:v>高-欧美</x:v>
       </x:c>
       <x:c r="C8" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D8" s="31" t="str">
         <x:v>13957403</x:v>
@@ -992,7 +992,7 @@
         <x:v>poli film mexico</x:v>
       </x:c>
       <x:c r="F8" s="30" t="str">
-        <x:v>US</x:v>
+        <x:v>美国</x:v>
       </x:c>
       <x:c r="G8" s="30" t="str">
         <x:v>restrada@poli-film.net</x:v>
@@ -1047,7 +1047,7 @@
       </x:c>
       <x:c r="AD8" s="30" t="str"/>
       <x:c r="AE8" s="30" t="str">
-        <x:v>tin; polyethylene; masking film; poly ethylene; po le; cat; ion; rolls</x:v>
+        <x:v>tin；聚乙烯；遮蔽膜；聚乙烯；po le；cat；ion；卷材</x:v>
       </x:c>
       <x:c r="AF8" s="30" t="str">
         <x:v>POLYETHYLENE MASKING FILM - ROLLS OF POLY ETHYLENE MASKING FILM(..)PACK ED ONTO PALLETS REF# ,W-- PO #PO LEG// =CONSIGNEE &amp; NOTIFY CONTINUE: TEL:+- TAX IDEN TIFICATION NUMBE R:PME--T&lt;br/&gt;</x:v>
@@ -1056,7 +1056,7 @@
       <x:c r="AH8" s="30" t="str"/>
       <x:c r="AI8" s="30" t="str"/>
       <x:c r="AJ8" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK8" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -1078,7 +1078,7 @@
         <x:v>高-欧美</x:v>
       </x:c>
       <x:c r="C9" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D9" s="31" t="str">
         <x:v>229078</x:v>
@@ -1087,7 +1087,7 @@
         <x:v>pacoa</x:v>
       </x:c>
       <x:c r="F9" s="30" t="str">
-        <x:v>US</x:v>
+        <x:v>美国</x:v>
       </x:c>
       <x:c r="G9" s="30" t="str">
         <x:v>jtaub@pacoa.com</x:v>
@@ -1156,7 +1156,7 @@
       </x:c>
       <x:c r="AD9" s="30" t="str"/>
       <x:c r="AE9" s="30" t="str">
-        <x:v>wood; plastic drop cloth; ipm; caution tape; sol; masking film; packing material; hat; xxxxx</x:v>
+        <x:v>wood；塑料防护布；ipm；警示胶带；sol；遮蔽膜；包装材料；hat；xxxxx</x:v>
       </x:c>
       <x:c r="AF9" s="30" t="str">
         <x:v>2,886 CTNS OF PLASTIC DROP CLOTH, MASKING FILM AND CAUTION TAPE P.O. NO.: XXXXXX WE CERT IFY THAT THIS SHIPMENT CONTAINS NO SOLID WOODPACKING MATERIALS.&lt;br/&gt;</x:v>
@@ -1165,7 +1165,7 @@
       <x:c r="AH9" s="30" t="str"/>
       <x:c r="AI9" s="30" t="str"/>
       <x:c r="AJ9" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK9" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -1191,7 +1191,7 @@
         <x:v>高-欧美</x:v>
       </x:c>
       <x:c r="C10" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D10" s="31" t="str">
         <x:v>209484</x:v>
@@ -1200,7 +1200,7 @@
         <x:v>thermwell products</x:v>
       </x:c>
       <x:c r="F10" s="30" t="str">
-        <x:v>US</x:v>
+        <x:v>美国</x:v>
       </x:c>
       <x:c r="G10" s="30" t="str">
         <x:v>support@frostking.com</x:v>
@@ -1269,7 +1269,7 @@
       </x:c>
       <x:c r="AD10" s="30" t="str"/>
       <x:c r="AE10" s="30" t="str">
-        <x:v>plastic masking film</x:v>
+        <x:v>塑料遮蔽膜</x:v>
       </x:c>
       <x:c r="AF10" s="30" t="str">
         <x:v>PLASTIC MASKING FILM,HS:392010&lt;br/&gt;</x:v>
@@ -1278,7 +1278,7 @@
       <x:c r="AH10" s="30" t="str"/>
       <x:c r="AI10" s="30" t="str"/>
       <x:c r="AJ10" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK10" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -1304,7 +1304,7 @@
         <x:v>高-欧美</x:v>
       </x:c>
       <x:c r="C11" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D11" s="31" t="str">
         <x:v>71495262</x:v>
@@ -1313,7 +1313,7 @@
         <x:v>TPLOGIX, INC</x:v>
       </x:c>
       <x:c r="F11" s="30" t="str">
-        <x:v>US</x:v>
+        <x:v>美国</x:v>
       </x:c>
       <x:c r="G11" s="30" t="str">
         <x:v>csr1@tplogix.com</x:v>
@@ -1385,7 +1385,7 @@
       <x:c r="AH11" s="30" t="str"/>
       <x:c r="AI11" s="30" t="str"/>
       <x:c r="AJ11" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK11" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -1411,7 +1411,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C12" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D12" s="31" t="str">
         <x:v>20189222</x:v>
@@ -1420,7 +1420,7 @@
         <x:v>DIXON TECHNOLOGIES (INDIA) LIMITED</x:v>
       </x:c>
       <x:c r="F12" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G12" s="30" t="str">
         <x:v>investorrelations@dixoninfo.com</x:v>
@@ -1480,25 +1480,25 @@
         <x:v>investorrelations@dixoninfo.com:1</x:v>
       </x:c>
       <x:c r="AD12" s="30" t="str">
-        <x:v>Rubber Tape; Parts for LED TV</x:v>
+        <x:v>橡胶胶带；LED电视零部件</x:v>
       </x:c>
       <x:c r="AE12" s="30" t="str">
-        <x:v>Rubber; Tape; TPE; LED TV; Parts</x:v>
+        <x:v>橡胶；胶带；TPE；LED电视；零部件</x:v>
       </x:c>
       <x:c r="AF12" s="30" t="str">
         <x:v>RUBBER,TAPE,TPE,300X4.5X2,32,43,55DOTBL-0609-0000019-10-PARTS FOR LED TV-FOCPARTS FOR LED TV</x:v>
       </x:c>
       <x:c r="AG12" s="30" t="str">
-        <x:v>Rubber Adhesive Tape; LED TV Accessories; TPE Tape; TV Parts; Rubber Strip</x:v>
+        <x:v>橡胶胶粘带；LED电视配件；TPE胶带；电视零部件；橡胶条</x:v>
       </x:c>
       <x:c r="AH12" s="30" t="str">
-        <x:v>Rubber Resin; TPE Polymer; Plastic; Metal; Electronic Components</x:v>
+        <x:v>橡胶树脂；TPE聚合物；塑料；金属；电子元件</x:v>
       </x:c>
       <x:c r="AI12" s="30" t="str">
-        <x:v>LED TVs; Monitor; Display Devices; Home Appliances; Consumer Electronics</x:v>
+        <x:v>LED电视；显示器；显示设备；家用电器；消费电子</x:v>
       </x:c>
       <x:c r="AJ12" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK12" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -1520,7 +1520,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C13" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D13" s="31" t="str">
         <x:v>1945196</x:v>
@@ -1529,7 +1529,7 @@
         <x:v>laarcourier express s.a.</x:v>
       </x:c>
       <x:c r="F13" s="30" t="str">
-        <x:v>EC</x:v>
+        <x:v>厄瓜多尔</x:v>
       </x:c>
       <x:c r="G13" s="30" t="str">
         <x:v>ccoque@grupolaar.com</x:v>
@@ -1588,7 +1588,7 @@
       </x:c>
       <x:c r="AD13" s="30" t="str"/>
       <x:c r="AE13" s="30" t="str">
-        <x:v>coffee maker; glove; bedspread; pressure transmitter</x:v>
+        <x:v>coffee maker；glove；bedspread；pressure transmitter</x:v>
       </x:c>
       <x:c r="AF13" s="30" t="str">
         <x:v>TWO-PIECE SWIMSUIT 35911615558 SOMBRERO DE COPA VACIO 10712856281 VESTIDO 9850584530 SOMBRERO DE COPA VACIO 89050573348 TWO-PIECE SWIMSUIT 4804392116 REPAIR TAPE 44363863818 LONG SLEEVE CREW NECK FOR</x:v>
@@ -1597,7 +1597,7 @@
       <x:c r="AH13" s="30" t="str"/>
       <x:c r="AI13" s="30" t="str"/>
       <x:c r="AJ13" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK13" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -1619,7 +1619,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C14" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D14" s="31" t="str">
         <x:v>20189128</x:v>
@@ -1628,7 +1628,7 @@
         <x:v>SAMSUNG INDIA ELECTRONICS PRIVATE LIMITED</x:v>
       </x:c>
       <x:c r="F14" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G14" s="30" t="str">
         <x:v>kiran.shindemumbai@gmail.com</x:v>
@@ -1698,7 +1698,7 @@
       <x:c r="AH14" s="30" t="str"/>
       <x:c r="AI14" s="30" t="str"/>
       <x:c r="AJ14" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK14" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -1722,7 +1722,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C15" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D15" s="31" t="str">
         <x:v>20195417</x:v>
@@ -1731,7 +1731,7 @@
         <x:v>VIVO MOBILE INDIA PRIVATE LIMITED</x:v>
       </x:c>
       <x:c r="F15" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G15" s="30" t="str">
         <x:v>support.in@vivo.com</x:v>
@@ -1801,7 +1801,7 @@
       <x:c r="AH15" s="30" t="str"/>
       <x:c r="AI15" s="30" t="str"/>
       <x:c r="AJ15" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK15" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -1823,7 +1823,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C16" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D16" s="31" t="str">
         <x:v>80133</x:v>
@@ -1832,7 +1832,7 @@
         <x:v>brandix apparel india pvt.ltd.</x:v>
       </x:c>
       <x:c r="F16" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G16" s="30" t="str">
         <x:v>info@brandix.com</x:v>
@@ -1887,7 +1887,7 @@
       </x:c>
       <x:c r="AD16" s="30" t="str"/>
       <x:c r="AE16" s="30" t="str">
-        <x:v>fabric elastic; tape; narrow woven</x:v>
+        <x:v>弹性织物；胶带；窄幅织物</x:v>
       </x:c>
       <x:c r="AF16" s="30" t="str">
         <x:v>NARROW WOVEN FABRIC ELASTIC TAPE 7000 MTRS BEL 8588023</x:v>
@@ -1896,7 +1896,7 @@
       <x:c r="AH16" s="30" t="str"/>
       <x:c r="AI16" s="30" t="str"/>
       <x:c r="AJ16" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK16" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -1918,7 +1918,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C17" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D17" s="31" t="str">
         <x:v>4421112</x:v>
@@ -1927,7 +1927,7 @@
         <x:v>công ty tnhh honest việt nam</x:v>
       </x:c>
       <x:c r="F17" s="30" t="str">
-        <x:v>VN</x:v>
+        <x:v>越南</x:v>
       </x:c>
       <x:c r="G17" s="30" t="str">
         <x:v>hue.dt@honestvietnam.com.vn</x:v>
@@ -1988,7 +1988,7 @@
       </x:c>
       <x:c r="AD17" s="30" t="str"/>
       <x:c r="AE17" s="30" t="str">
-        <x:v>camshaft; adhesive tape</x:v>
+        <x:v>camshaft；胶粘带</x:v>
       </x:c>
       <x:c r="AF17" s="30" t="str">
         <x:v>PS-1#&amp;Trục bằng thép</x:v>
@@ -1997,7 +1997,7 @@
       <x:c r="AH17" s="30" t="str"/>
       <x:c r="AI17" s="30" t="str"/>
       <x:c r="AJ17" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK17" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -2023,7 +2023,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C18" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D18" s="31" t="str">
         <x:v>369752</x:v>
@@ -2032,7 +2032,7 @@
         <x:v>genus electrotech ltd.</x:v>
       </x:c>
       <x:c r="F18" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G18" s="30" t="str">
         <x:v>info@genuselectrotech.com</x:v>
@@ -2097,7 +2097,7 @@
       </x:c>
       <x:c r="AD18" s="30" t="str"/>
       <x:c r="AE18" s="30" t="str">
-        <x:v>fixture; ail; vhb tape</x:v>
+        <x:v>fixture；ail；vhb tape</x:v>
       </x:c>
       <x:c r="AF18" s="30" t="str">
         <x:v>VHB TAPE PRESSURE HOLDING FIXTURE REST DETAILS AS PER INV &amp;PL VHB TAPE PRESSURE HOLDING FIXTURE REST DETAILS AS PER INV &amp;</x:v>
@@ -2106,7 +2106,7 @@
       <x:c r="AH18" s="30" t="str"/>
       <x:c r="AI18" s="30" t="str"/>
       <x:c r="AJ18" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK18" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -2128,7 +2128,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C19" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D19" s="31" t="str">
         <x:v>67944548</x:v>
@@ -2137,7 +2137,7 @@
         <x:v>oriental commerce co.ltd.</x:v>
       </x:c>
       <x:c r="F19" s="30" t="str">
-        <x:v>KR</x:v>
+        <x:v>韩国</x:v>
       </x:c>
       <x:c r="G19" s="30" t="str">
         <x:v>sim291@hanmail.net</x:v>
@@ -2196,7 +2196,7 @@
       </x:c>
       <x:c r="AD19" s="30" t="str"/>
       <x:c r="AE19" s="30" t="str">
-        <x:v>textile insulation tape</x:v>
+        <x:v>纺织绝缘胶带</x:v>
       </x:c>
       <x:c r="AF19" s="30" t="str">
         <x:v>CLT-26-2037#&amp;Vải dệt đã cao su hóa 200MIC X 50MM X 25M #&amp;VN</x:v>
@@ -2205,7 +2205,7 @@
       <x:c r="AH19" s="30" t="str"/>
       <x:c r="AI19" s="30" t="str"/>
       <x:c r="AJ19" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK19" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -2227,7 +2227,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C20" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D20" s="31" t="str">
         <x:v>1005206</x:v>
@@ -2236,7 +2236,7 @@
         <x:v>jworld co.ltd.</x:v>
       </x:c>
       <x:c r="F20" s="30" t="str">
-        <x:v>KR</x:v>
+        <x:v>韩国</x:v>
       </x:c>
       <x:c r="G20" s="30" t="str">
         <x:v>jworld@jworld21.com</x:v>
@@ -2304,7 +2304,7 @@
       <x:c r="AH20" s="30" t="str"/>
       <x:c r="AI20" s="30" t="str"/>
       <x:c r="AJ20" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK20" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -2326,7 +2326,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C21" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D21" s="31" t="str">
         <x:v>28403</x:v>
@@ -2335,7 +2335,7 @@
         <x:v>suzuki motor de mexico s a</x:v>
       </x:c>
       <x:c r="F21" s="30" t="str">
-        <x:v>MX</x:v>
+        <x:v>墨西哥</x:v>
       </x:c>
       <x:c r="G21" s="30" t="str">
         <x:v>privacidad@suzuki.com.mx</x:v>
@@ -2396,7 +2396,7 @@
       </x:c>
       <x:c r="AD21" s="30" t="str"/>
       <x:c r="AE21" s="30" t="str">
-        <x:v>green tape; yellow ribbon</x:v>
+        <x:v>绿色胶带；黄色带材</x:v>
       </x:c>
       <x:c r="AF21" s="30" t="str">
         <x:v>CINTA COD 83926 54P10 0CE</x:v>
@@ -2405,7 +2405,7 @@
       <x:c r="AH21" s="30" t="str"/>
       <x:c r="AI21" s="30" t="str"/>
       <x:c r="AJ21" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK21" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -2427,7 +2427,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C22" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D22" s="31" t="str">
         <x:v>368379</x:v>
@@ -2436,7 +2436,7 @@
         <x:v>haier appliances india pvt.ltd.</x:v>
       </x:c>
       <x:c r="F22" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G22" s="30" t="str">
         <x:v>chuktiii@gmail.com</x:v>
@@ -2503,7 +2503,7 @@
       </x:c>
       <x:c r="AD22" s="30" t="str"/>
       <x:c r="AE22" s="30" t="str">
-        <x:v>packing tap; t code; e 80; x7; model; assembly component</x:v>
+        <x:v>包装胶带；t code；e 80；x7；model；装配部件</x:v>
       </x:c>
       <x:c r="AF22" s="30" t="str">
         <x:v>PACKING TAPE 800MX72X0.045MM 50P7GT-P PART CODE: 0090303389MODEL NO 50P7GT-P (ASSEMBLY COMPONENT)PACKING TAPE 800MX72X0.045MM 50P7GT-P PART CODE: 0090303389</x:v>
@@ -2512,7 +2512,7 @@
       <x:c r="AH22" s="30" t="str"/>
       <x:c r="AI22" s="30" t="str"/>
       <x:c r="AJ22" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK22" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -2538,7 +2538,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C23" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D23" s="31" t="str">
         <x:v>22316517</x:v>
@@ -2547,7 +2547,7 @@
         <x:v>TRIUMPH INTERNATIONAL (INDIA) PRIVATE LIMITED</x:v>
       </x:c>
       <x:c r="F23" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G23" s="30" t="str">
         <x:v>murugan.selvaraj@triumph.com</x:v>
@@ -2609,7 +2609,7 @@
       <x:c r="AH23" s="30" t="str"/>
       <x:c r="AI23" s="30" t="str"/>
       <x:c r="AJ23" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK23" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -2631,7 +2631,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C24" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D24" s="31" t="str">
         <x:v>20410195</x:v>
@@ -2640,7 +2640,7 @@
         <x:v>ASTI ELECTRONICS CORPORATION</x:v>
       </x:c>
       <x:c r="F24" s="30" t="str">
-        <x:v>VN</x:v>
+        <x:v>越南</x:v>
       </x:c>
       <x:c r="G24" s="30" t="str">
         <x:v>admin@asti.com.vn</x:v>
@@ -2706,7 +2706,7 @@
       <x:c r="AH24" s="30" t="str"/>
       <x:c r="AI24" s="30" t="str"/>
       <x:c r="AJ24" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK24" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -2728,7 +2728,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C25" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D25" s="31" t="str">
         <x:v>8206989</x:v>
@@ -2737,7 +2737,7 @@
         <x:v>triumph international india</x:v>
       </x:c>
       <x:c r="F25" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G25" s="30" t="str">
         <x:v>info.india@triumph.com</x:v>
@@ -2798,7 +2798,7 @@
       </x:c>
       <x:c r="AD25" s="30" t="str"/>
       <x:c r="AE25" s="30" t="str">
-        <x:v>eye tape; pearl</x:v>
+        <x:v>eye tape；pearl</x:v>
       </x:c>
       <x:c r="AF25" s="30" t="str">
         <x:v>PRECUT EYE TAPE 000 S0182S 38MM A PEARL GR 38198 PO 4512863360 12863362PRECUT EYE TAPE</x:v>
@@ -2807,7 +2807,7 @@
       <x:c r="AH25" s="30" t="str"/>
       <x:c r="AI25" s="30" t="str"/>
       <x:c r="AJ25" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK25" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -2829,7 +2829,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C26" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D26" s="31" t="str">
         <x:v>78071611</x:v>
@@ -2838,7 +2838,7 @@
         <x:v>INNO FLEX</x:v>
       </x:c>
       <x:c r="F26" s="30" t="str">
-        <x:v>KR</x:v>
+        <x:v>韩国</x:v>
       </x:c>
       <x:c r="G26" s="30" t="str">
         <x:v>cosmotech@korea.com</x:v>
@@ -2896,25 +2896,25 @@
         <x:v>cosmotech@korea.com:3</x:v>
       </x:c>
       <x:c r="AD26" s="30" t="str">
-        <x:v>TAPE-1 P1 DUO</x:v>
+        <x:v>TAPE-1 P1 DUO（胶带型号）</x:v>
       </x:c>
       <x:c r="AE26" s="30" t="str">
-        <x:v>tape; plastic; self - adhesive; recycled</x:v>
+        <x:v>胶带；塑料；自粘；再生材料</x:v>
       </x:c>
       <x:c r="AF26" s="30" t="str">
         <x:v>TAPE-1 P1 DUO#&amp;Miếng plastic tự dán TAPE-1 P1 DUO (TOP TAPE TESA61885), kt 120.08*12.50mm, hàng mới 100% tái xuất mục 44 TK 107230146220#&amp;KR</x:v>
       </x:c>
       <x:c r="AG26" s="30" t="str">
-        <x:v>Adhesive tape; Self - sticking tape; Plastic tape; Duo tape; TESA tape</x:v>
+        <x:v>胶粘带；自粘胶带；塑料胶带；双面胶带；德莎胶带</x:v>
       </x:c>
       <x:c r="AH26" s="30" t="str">
-        <x:v>Plastic resin; Adhesive; Polymer; Additives; Recycled plastic</x:v>
+        <x:v>塑料树脂；胶粘剂；聚合物；添加剂；再生塑料</x:v>
       </x:c>
       <x:c r="AI26" s="30" t="str">
-        <x:v>Packaging; Labeling; Crafts; Electronics assembly; Office use</x:v>
+        <x:v>包装；标签制作；手工艺；电子装配；办公用途</x:v>
       </x:c>
       <x:c r="AJ26" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK26" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -2936,7 +2936,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C27" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D27" s="31" t="str">
         <x:v>5141777</x:v>
@@ -2945,7 +2945,7 @@
         <x:v>han soll textiles ltd.</x:v>
       </x:c>
       <x:c r="F27" s="30" t="str">
-        <x:v>KR</x:v>
+        <x:v>韩国</x:v>
       </x:c>
       <x:c r="G27" s="30" t="str">
         <x:v>annapark@hansoll.com</x:v>
@@ -3006,7 +3006,7 @@
       </x:c>
       <x:c r="AD27" s="30" t="str"/>
       <x:c r="AE27" s="30" t="str">
-        <x:v>accessories of plastics</x:v>
+        <x:v>塑料配件</x:v>
       </x:c>
       <x:c r="AF27" s="30" t="str">
         <x:v>DÂY CHỐNG DÃN 0608 (MOBILON TAPE SHL-0608; DÂY VIỀN 0608; Kích thước: 6 MM x 0.08 MM; 826,491.41 MÉT; SỬ DỤNG TRONG MAY MẶC; CHẤT LIỆU: POLYURE THANE; HÀNG MỚI 100%)#&amp;KR</x:v>
@@ -3015,7 +3015,7 @@
       <x:c r="AH27" s="30" t="str"/>
       <x:c r="AI27" s="30" t="str"/>
       <x:c r="AJ27" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK27" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -3037,7 +3037,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C28" s="30" t="str">
-        <x:v>tape; masking film</x:v>
+        <x:v>胶带；遮蔽膜</x:v>
       </x:c>
       <x:c r="D28" s="31" t="str">
         <x:v>20482013</x:v>
@@ -3046,7 +3046,7 @@
         <x:v>AJIT INDUSTRIES PRIVATE LIMITED</x:v>
       </x:c>
       <x:c r="F28" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G28" s="30" t="str">
         <x:v>marketing@ajitindustries.com</x:v>
@@ -3108,25 +3108,25 @@
         <x:v>marketing@ajitindustries.com:1; suneet@ajitindustries.com:1</x:v>
       </x:c>
       <x:c r="AD28" s="30" t="str">
-        <x:v>PE Masking Film</x:v>
+        <x:v>PE遮蔽膜</x:v>
       </x:c>
       <x:c r="AE28" s="30" t="str">
-        <x:v>PE; Masking film; Industrial use</x:v>
+        <x:v>PE；遮蔽膜；工业用途</x:v>
       </x:c>
       <x:c r="AF28" s="30" t="str">
         <x:v>MASKING TAPE (IN JUMBO ROLLS)PRODUCT CODE:770UU;COLOR:BEIGE;SIZE:1570mm x 2000m (RLS:53)(PIMS NO:ORIGINAL DPIIT-PPR-2025MASKING TAPE (IN JUMBO ROLLS)PRODUCT CODE:770UU;COLOR:BEIGE;; PE MASKING FILM IN LARGE ROLL SIZE: 2700MM*1600M (ROLL 600)(FOR INDUSTRIAL USE)PE MASKING FILM IN</x:v>
       </x:c>
       <x:c r="AG28" s="30" t="str">
-        <x:v>PE protective film; PE masking tape; Polyethylene masking film; Industrial masking film; PE covering film</x:v>
+        <x:v>PE保护膜；PE遮蔽胶带；聚乙烯遮蔽膜；工业遮蔽膜；PE覆盖膜</x:v>
       </x:c>
       <x:c r="AH28" s="30" t="str">
-        <x:v>Polyethylene resin; Plastic additives; Petroleum; Ethylene; Catalyst</x:v>
+        <x:v>聚乙烯树脂；塑料添加剂；石油；乙烯；催化剂</x:v>
       </x:c>
       <x:c r="AI28" s="30" t="str">
-        <x:v>Automotive painting; Electronics manufacturing; Furniture production; Construction; Metal processing</x:v>
+        <x:v>汽车涂装；电子制造；家具生产；建筑施工；金属加工</x:v>
       </x:c>
       <x:c r="AJ28" s="30" t="str">
-        <x:v>tape; masking film</x:v>
+        <x:v>胶带；遮蔽膜</x:v>
       </x:c>
       <x:c r="AK28" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search; masking-film-buyers-exact-search</x:v>
@@ -3148,7 +3148,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C29" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D29" s="31" t="str">
         <x:v>86190</x:v>
@@ -3157,7 +3157,7 @@
         <x:v>vivo mobile india pvt ltd</x:v>
       </x:c>
       <x:c r="F29" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G29" s="30" t="str">
         <x:v>support.in@vivo.com</x:v>
@@ -3212,7 +3212,7 @@
       </x:c>
       <x:c r="AD29" s="30" t="str"/>
       <x:c r="AE29" s="30" t="str">
-        <x:v>paper; arts; water contact indicator tape; mobile phone 5</x:v>
+        <x:v>纸；工艺品；遇水指示胶带；手机用途</x:v>
       </x:c>
       <x:c r="AF29" s="30" t="str">
         <x:v>5181866 WATER CONTACT INDICATOR TAPE PAPER PARTS FOR MFG OF MOBILE PHONE 5181866 WATER CONTACT INDICATOR TAPE PAPER PARTS FOR MFG</x:v>
@@ -3221,7 +3221,7 @@
       <x:c r="AH29" s="30" t="str"/>
       <x:c r="AI29" s="30" t="str"/>
       <x:c r="AJ29" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK29" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -3247,7 +3247,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C30" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="D30" s="31" t="str">
         <x:v>20432358</x:v>
@@ -3256,7 +3256,7 @@
         <x:v>TESA TAPES (INDIA) PRIVATE LIMITED</x:v>
       </x:c>
       <x:c r="F30" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G30" s="30" t="str">
         <x:v>marketing.india@tesa.com</x:v>
@@ -3328,7 +3328,7 @@
       <x:c r="AH30" s="30" t="str"/>
       <x:c r="AI30" s="30" t="str"/>
       <x:c r="AJ30" s="30" t="str">
-        <x:v>tape</x:v>
+        <x:v>胶带</x:v>
       </x:c>
       <x:c r="AK30" s="30" t="str">
         <x:v>tape-buyers-fuzzy-search</x:v>
@@ -3354,7 +3354,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C31" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D31" s="31" t="str">
         <x:v>28739610</x:v>
@@ -3363,7 +3363,7 @@
         <x:v>SARASWATI PLASTOTECH INDIA PRIVATE LIMITED</x:v>
       </x:c>
       <x:c r="F31" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G31" s="30" t="str">
         <x:v>cs@saraswatigroupdb.com</x:v>
@@ -3423,25 +3423,25 @@
         <x:v>cs@saraswatigroupdb.com:1</x:v>
       </x:c>
       <x:c r="AD31" s="30" t="str">
-        <x:v>Masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AE31" s="30" t="str">
-        <x:v>Masking film; Protection film; Clear film; PS sheet</x:v>
+        <x:v>遮蔽膜；保护膜；透明薄膜；PS片材</x:v>
       </x:c>
       <x:c r="AF31" s="30" t="str">
         <x:v>MASKING FILM (PRE PROTECTION FILM),FILM CLEAR FILM FOR PS SHEET,50*1250*1500(20 ROLLS)(ACTUAL USER)MASKING FILM (PRE PROTECTION FILM)</x:v>
       </x:c>
       <x:c r="AG31" s="30" t="str">
-        <x:v>Pre - protection film; Surface masking film; Clear masking film; PS sheet protection film; Temporary masking film</x:v>
+        <x:v>预保护膜；表面遮蔽膜；透明遮蔽膜；PS片材保护膜；临时遮蔽膜</x:v>
       </x:c>
       <x:c r="AH31" s="30" t="str">
-        <x:v>Plastic resin; Polymer; Additives; Solvents; Pigments</x:v>
+        <x:v>塑料树脂；聚合物；添加剂；溶剂；颜料</x:v>
       </x:c>
       <x:c r="AI31" s="30" t="str">
-        <x:v>Electronics manufacturing; Automotive painting; Furniture production; Glass manufacturing; Construction</x:v>
+        <x:v>电子制造；汽车涂装；家具生产；玻璃制造；建筑施工</x:v>
       </x:c>
       <x:c r="AJ31" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK31" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -3463,7 +3463,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C32" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D32" s="31" t="str">
         <x:v>20208403</x:v>
@@ -3472,7 +3472,7 @@
         <x:v>AIR WORKS INDIA (ENGINEERING)PVT LTD</x:v>
       </x:c>
       <x:c r="F32" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G32" s="30" t="str">
         <x:v>deepak.goyal@airworks.in</x:v>
@@ -3534,25 +3534,25 @@
         <x:v>deepak.goyal@airworks.in:1</x:v>
       </x:c>
       <x:c r="AD32" s="30" t="str">
-        <x:v>Masking Film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AE32" s="30" t="str">
-        <x:v>Masking Film; Aircraft use; Blue</x:v>
+        <x:v>遮蔽膜；航空用途；Blue</x:v>
       </x:c>
       <x:c r="AF32" s="30" t="str">
         <x:v>WTE-MF-17-G Masking Film- 6m x 100m x 17mu Blue(Carton:-98cmx 15 x 15 - Per Roll)(FOR AIRCRAFT USE)(ACTUAL USE)18 ROLLSWTE-MF-17-G Masking Film- 6m x 100m x 17mu Blue(Carton:-98cm</x:v>
       </x:c>
       <x:c r="AG32" s="30" t="str">
-        <x:v>Painter's tape; Protective film; Covering film; Surface protection film; Temporary masking film</x:v>
+        <x:v>涂装遮蔽胶带；保护膜；覆盖膜；表面保护膜；临时遮蔽膜</x:v>
       </x:c>
       <x:c r="AH32" s="30" t="str">
-        <x:v>Plastic resin; Polymer; Additives; Pigments; Adhesive</x:v>
+        <x:v>塑料树脂；聚合物；添加剂；颜料；胶粘剂</x:v>
       </x:c>
       <x:c r="AI32" s="30" t="str">
-        <x:v>Aircraft manufacturing; Aircraft maintenance; Automotive painting; Industrial coating; Construction painting</x:v>
+        <x:v>飞机制造；飞机维护；汽车涂装；工业涂装；建筑涂装</x:v>
       </x:c>
       <x:c r="AJ32" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK32" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -3574,7 +3574,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C33" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D33" s="31" t="str">
         <x:v>22311398</x:v>
@@ -3583,7 +3583,7 @@
         <x:v>SUMAX ENGINEERING PRIVATE LIMITED</x:v>
       </x:c>
       <x:c r="F33" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G33" s="30" t="str">
         <x:v>info@sumaxindia.com</x:v>
@@ -3641,25 +3641,25 @@
         <x:v>info@sumaxindia.com:1</x:v>
       </x:c>
       <x:c r="AD33" s="30" t="str">
-        <x:v>Masking Film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AE33" s="30" t="str">
-        <x:v>Masking; Film</x:v>
+        <x:v>遮蔽；薄膜</x:v>
       </x:c>
       <x:c r="AF33" s="30" t="str">
         <x:v>MASKING FILM (535 MMX1200M) 1 PCS</x:v>
       </x:c>
       <x:c r="AG33" s="30" t="str">
-        <x:v>Painter's tape film; Protective masking film; Temporary masking film; Construction masking film; Decorative masking film</x:v>
+        <x:v>涂装遮蔽膜；保护遮蔽膜；临时遮蔽膜；施工遮蔽膜；装饰遮蔽膜</x:v>
       </x:c>
       <x:c r="AH33" s="30" t="str">
-        <x:v>Plastic resin; Polymer; Chemical additives; Adhesive; Base film material</x:v>
+        <x:v>塑料树脂；聚合物；化学添加剂；胶粘剂；基膜材料</x:v>
       </x:c>
       <x:c r="AI33" s="30" t="str">
-        <x:v>Painting projects; Construction sites; Automotive refinishing; Furniture manufacturing; Decorative work</x:v>
+        <x:v>涂装工程；施工现场；汽车修补涂装；家具制造；装饰工程</x:v>
       </x:c>
       <x:c r="AJ33" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK33" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -3681,7 +3681,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C34" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D34" s="31" t="str">
         <x:v>370961</x:v>
@@ -3690,7 +3690,7 @@
         <x:v>ajit industries pvt ltd.</x:v>
       </x:c>
       <x:c r="F34" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G34" s="30" t="str">
         <x:v>marketing@ajitindustries.com</x:v>
@@ -3751,7 +3751,7 @@
       </x:c>
       <x:c r="AD34" s="30" t="str"/>
       <x:c r="AE34" s="30" t="str">
-        <x:v>roll; tria; masking film; arg; e roll</x:v>
+        <x:v>卷材；tria；遮蔽膜；arg；e roll</x:v>
       </x:c>
       <x:c r="AF34" s="30" t="str">
         <x:v>PE MASKING FILM IN LARGE ROLL SIZE: 2700MM*1600M (ROLL 600)(FOR INDUSTRIAL USE)PE MASKING FILM IN</x:v>
@@ -3760,7 +3760,7 @@
       <x:c r="AH34" s="30" t="str"/>
       <x:c r="AI34" s="30" t="str"/>
       <x:c r="AJ34" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK34" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -3782,7 +3782,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C35" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D35" s="31" t="str">
         <x:v>27951674</x:v>
@@ -3791,7 +3791,7 @@
         <x:v>PRIYANKA ENTERPRISE</x:v>
       </x:c>
       <x:c r="F35" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G35" s="30" t="str">
         <x:v>pryentp@hotmail.com</x:v>
@@ -3853,25 +3853,25 @@
         <x:v>info@modularfurniturebpl.com:2; pryentp@hotmail.com:1</x:v>
       </x:c>
       <x:c r="AD35" s="30" t="str">
-        <x:v>Pretaped masking film; Masking tape</x:v>
+        <x:v>预贴胶带遮蔽膜；遮蔽胶带</x:v>
       </x:c>
       <x:c r="AE35" s="30" t="str">
-        <x:v>Pretaped masking film; Masking tape; HDPE; Shrink wrapped; Color label</x:v>
+        <x:v>预贴胶带遮蔽膜；遮蔽胶带；高密度聚乙烯；收缩包装；彩色标签</x:v>
       </x:c>
       <x:c r="AF35" s="30" t="str">
         <x:v>PRETAPED MASKING FILM - 1M X 25M,PRETAPED MASKING FILM, HDPE, MASKING TAPE, EACH ROLL SHRINK WRAPPED WITH COLOR LABEL (2PRETAPED MASKING FILM - 1M X 25M,PRETAPED MASKING FILM, HDPE</x:v>
       </x:c>
       <x:c r="AG35" s="30" t="str">
-        <x:v>Masking film with tape; Pre - taped film for masking; Self - taped masking film; HDPE masking film; Taped masking sheet</x:v>
+        <x:v>带胶带遮蔽膜；预贴胶带遮蔽膜；自带胶遮蔽膜；HDPE遮蔽膜；带胶遮蔽片</x:v>
       </x:c>
       <x:c r="AH35" s="30" t="str">
-        <x:v>High - density polyethylene resin; Plastic additives; Adhesive materials; Polymer raw materials; Tape backing materials</x:v>
+        <x:v>高密度聚乙烯树脂；塑料添加剂；胶粘材料；聚合物原料；胶带基材</x:v>
       </x:c>
       <x:c r="AI35" s="30" t="str">
-        <x:v>Painting industry; Automotive refinishing; Construction projects; Furniture manufacturing; DIY home improvement</x:v>
+        <x:v>涂装行业；汽车修补涂装；建筑工程；家具制造；家居DIY</x:v>
       </x:c>
       <x:c r="AJ35" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK35" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -3893,7 +3893,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C36" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D36" s="31" t="str">
         <x:v>20199535</x:v>
@@ -3902,7 +3902,7 @@
         <x:v>GRINDWELL NORTON LIMITED</x:v>
       </x:c>
       <x:c r="F36" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G36" s="30" t="str">
         <x:v>sharecmpt.gno@saint-gobain.com</x:v>
@@ -3964,25 +3964,25 @@
         <x:v>sharecmpt.gno@saint-gobain.com:1</x:v>
       </x:c>
       <x:c r="AD36" s="30" t="str">
-        <x:v>Plastic Masking Film</x:v>
+        <x:v>塑料遮蔽膜</x:v>
       </x:c>
       <x:c r="AE36" s="30" t="str">
-        <x:v>Plastic; Masking Film; MFG Use</x:v>
+        <x:v>塑料；遮蔽膜；制造用途</x:v>
       </x:c>
       <x:c r="AF36" s="30" t="str">
         <x:v>PLASTIC MASKING FILM 9MIC X 4M X 150M 66254455280 600ROLLS (FOR MFG USE)PLASTIC MASKING FILM 9MIC X 4M X 150M 66254455280 600ROLLS (</x:v>
       </x:c>
       <x:c r="AG36" s="30" t="str">
-        <x:v>Plastic Film Mask; Masking Plastic Sheeting; Plastic Protective Film; Film Masking; Plastic Covering Film</x:v>
+        <x:v>塑料遮蔽膜；塑料遮蔽片材；塑料保护膜；薄膜遮蔽；塑料覆盖膜</x:v>
       </x:c>
       <x:c r="AH36" s="30" t="str">
-        <x:v>Plastic Resin; Polymer; Additives; Plasticizer; Colorant</x:v>
+        <x:v>塑料树脂；聚合物；添加剂；增塑剂；着色剂</x:v>
       </x:c>
       <x:c r="AI36" s="30" t="str">
-        <x:v>Automotive Painting; Furniture Manufacturing; Electronics Assembly; Construction; Printing</x:v>
+        <x:v>汽车涂装；家具制造；电子装配；建筑施工；印刷</x:v>
       </x:c>
       <x:c r="AJ36" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK36" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -4004,7 +4004,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C37" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D37" s="31" t="str">
         <x:v>168017</x:v>
@@ -4012,7 +4012,9 @@
       <x:c r="E37" s="30" t="str">
         <x:v>grindwell norton ltd</x:v>
       </x:c>
-      <x:c r="F37" s="30" t="str"/>
+      <x:c r="F37" s="30" t="str">
+        <x:v>未标明</x:v>
+      </x:c>
       <x:c r="G37" s="30" t="str">
         <x:v>bonded.gno@saint-gobain.com</x:v>
       </x:c>
@@ -4071,25 +4073,25 @@
         <x:v>bonded.gno@saint-gobain.com:1</x:v>
       </x:c>
       <x:c r="AD37" s="30" t="str">
-        <x:v>Plastic masking film</x:v>
+        <x:v>塑料遮蔽膜</x:v>
       </x:c>
       <x:c r="AE37" s="30" t="str">
-        <x:v>Plastic; Masking film; MFG use</x:v>
+        <x:v>塑料；遮蔽膜；制造用途</x:v>
       </x:c>
       <x:c r="AF37" s="30" t="str">
         <x:v>PLASTIC MASKING FILM 9MIC X 4M X 150M 66254455280 600ROLLS (FOR MFG USE)PLASTIC MASKING FILM 9MIC X 4M X 150M 66254455280 600ROLLS (</x:v>
       </x:c>
       <x:c r="AG37" s="30" t="str">
-        <x:v>Plastic film mask; Masking plastic sheet; Plastic protective film; Film for masking; Plastic masking sheet</x:v>
+        <x:v>塑料遮蔽膜；塑料遮蔽片；塑料保护膜；遮蔽用薄膜；塑料遮蔽片</x:v>
       </x:c>
       <x:c r="AH37" s="30" t="str">
-        <x:v>Plastic resin; Polymer; Additives; Plastic raw material; Plastic compound</x:v>
+        <x:v>塑料树脂；聚合物；添加剂；塑料原料；塑料配混料</x:v>
       </x:c>
       <x:c r="AI37" s="30" t="str">
-        <x:v>Automotive painting; Furniture manufacturing; Electronics production; Construction painting; Metal finishing</x:v>
+        <x:v>汽车涂装；家具制造；电子生产；建筑涂装；金属表面处理</x:v>
       </x:c>
       <x:c r="AJ37" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK37" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -4111,7 +4113,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C38" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D38" s="31" t="str">
         <x:v>22315229</x:v>
@@ -4120,7 +4122,7 @@
         <x:v>STARCKE ABRASIVES INDIA PRIVATE LIMITED</x:v>
       </x:c>
       <x:c r="F38" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G38" s="30" t="str">
         <x:v>accounts@starcke.in</x:v>
@@ -4182,7 +4184,7 @@
       <x:c r="AH38" s="30" t="str"/>
       <x:c r="AI38" s="30" t="str"/>
       <x:c r="AJ38" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK38" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -4204,7 +4206,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C39" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D39" s="31" t="str">
         <x:v>28930762</x:v>
@@ -4213,7 +4215,7 @@
         <x:v>SUPER SALES CORPORATION</x:v>
       </x:c>
       <x:c r="F39" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G39" s="30" t="str">
         <x:v>jain.naman1984@gmail.com</x:v>
@@ -4275,25 +4277,25 @@
         <x:v>career@martfury.com:2; contact@martfury.com:2; customercare@martfury.com:2; info@superconduits.com:2; media@martfury.com:2; vendorsupport@martfury.com:2; jain.naman1984@gmail.com:1; supsalcorp@gmail.com:3</x:v>
       </x:c>
       <x:c r="AD39" s="30" t="str">
-        <x:v>Pre-taped Masking Film</x:v>
+        <x:v>预贴胶带遮蔽膜</x:v>
       </x:c>
       <x:c r="AE39" s="30" t="str">
-        <x:v>Pre-taped; Masking Film</x:v>
+        <x:v>Pre-taped；遮蔽膜</x:v>
       </x:c>
       <x:c r="AF39" s="30" t="str">
         <x:v>PRE-TAPED MASKING FILM,STYLE NO:80MM*45M(5400 ROLL) PRE-TAPED MASKING FILM,STYLE NO:80MM*45M(5400 ROLL)</x:v>
       </x:c>
       <x:c r="AG39" s="30" t="str">
-        <x:v>Taped Masking Film; Masking Tape Film; Pre - applied Masking Film; Self - taped Masking Film; Adhesive Masking Film</x:v>
+        <x:v>带胶遮蔽膜；胶带遮蔽膜；预贴遮蔽膜；自带胶遮蔽膜；自粘遮蔽膜</x:v>
       </x:c>
       <x:c r="AH39" s="30" t="str">
-        <x:v>Plastic Resin; Adhesive; Polymer; Film Base Material; Tape</x:v>
+        <x:v>塑料树脂；胶粘剂；聚合物；薄膜基材；胶带</x:v>
       </x:c>
       <x:c r="AI39" s="30" t="str">
-        <x:v>Automotive Painting; Furniture Finishing; Construction Painting; DIY Projects; Industrial Coating</x:v>
+        <x:v>汽车涂装；家具涂装；建筑涂装；DIY项目；工业涂装</x:v>
       </x:c>
       <x:c r="AJ39" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK39" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -4319,7 +4321,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C40" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D40" s="31" t="str">
         <x:v>67078</x:v>
@@ -4328,7 +4330,7 @@
         <x:v>aqua dynamics pvt ltd.</x:v>
       </x:c>
       <x:c r="F40" s="30" t="str">
-        <x:v>LK</x:v>
+        <x:v>斯里兰卡</x:v>
       </x:c>
       <x:c r="G40" s="30" t="str">
         <x:v>udaya@aquadynamics.lk</x:v>
@@ -4393,7 +4395,7 @@
       </x:c>
       <x:c r="AD40" s="30" t="str"/>
       <x:c r="AE40" s="30" t="str">
-        <x:v>masking film; masking; film for printing; rolls</x:v>
+        <x:v>遮蔽膜；遮蔽；印刷用薄膜；卷材</x:v>
       </x:c>
       <x:c r="AF40" s="30" t="str">
         <x:v>54 ROLLS MASKING FILMS MASKING FILM FOR PRINTING</x:v>
@@ -4402,7 +4404,7 @@
       <x:c r="AH40" s="30" t="str"/>
       <x:c r="AI40" s="30" t="str"/>
       <x:c r="AJ40" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK40" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -4428,7 +4430,7 @@
         <x:v>常规-全球</x:v>
       </x:c>
       <x:c r="C41" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="D41" s="31" t="str">
         <x:v>381348</x:v>
@@ -4437,7 +4439,7 @@
         <x:v>speciality polyfilms india pvt.ltd.</x:v>
       </x:c>
       <x:c r="F41" s="30" t="str">
-        <x:v>IN</x:v>
+        <x:v>印度</x:v>
       </x:c>
       <x:c r="G41" s="30" t="str">
         <x:v>commercial@specialty-films.com</x:v>
@@ -4490,7 +4492,7 @@
       </x:c>
       <x:c r="AD41" s="30" t="str"/>
       <x:c r="AE41" s="30" t="str">
-        <x:v>print; masking film</x:v>
+        <x:v>印刷；遮蔽膜</x:v>
       </x:c>
       <x:c r="AF41" s="30" t="str">
         <x:v>MASKING FILM-PRINTED</x:v>
@@ -4499,7 +4501,7 @@
       <x:c r="AH41" s="30" t="str"/>
       <x:c r="AI41" s="30" t="str"/>
       <x:c r="AJ41" s="30" t="str">
-        <x:v>masking film</x:v>
+        <x:v>遮蔽膜</x:v>
       </x:c>
       <x:c r="AK41" s="30" t="str">
         <x:v>masking-film-buyers-exact-search</x:v>
@@ -4554,7 +4556,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R886d1018b9d94528"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bb6d3aefc204935"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4997,10 +4999,10 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="41" t="str">
-        <x:v>品类</x:v>
+        <x:v>产品品类（中文）</x:v>
       </x:c>
       <x:c r="B6" s="41" t="str">
-        <x:v>命中 tape 或 masking film</x:v>
+        <x:v>胶带、遮蔽膜或两者都命中</x:v>
       </x:c>
       <x:c r="C6" s="41" t="str">
         <x:v>API、官网或公式</x:v>
@@ -5039,10 +5041,10 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="41" t="str">
-        <x:v>国家/地区</x:v>
+        <x:v>国家/地区（中文）</x:v>
       </x:c>
       <x:c r="B9" s="41" t="str">
-        <x:v>公司国家二字码</x:v>
+        <x:v>公司所在国家的中文名称</x:v>
       </x:c>
       <x:c r="C9" s="41" t="str">
         <x:v>API、官网或公式</x:v>
@@ -5151,10 +5153,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="41" t="str">
-        <x:v>API地址</x:v>
+        <x:v>API地址（原文）</x:v>
       </x:c>
       <x:c r="B17" s="41" t="str">
-        <x:v>跨境魔方返回的公司地址</x:v>
+        <x:v>跨境魔方返回的原始公司地址</x:v>
       </x:c>
       <x:c r="C17" s="41" t="str">
         <x:v>API、官网或公式</x:v>
@@ -5165,10 +5167,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="41" t="str">
-        <x:v>官网核验地址</x:v>
+        <x:v>官网核验地址（原文）</x:v>
       </x:c>
       <x:c r="B18" s="41" t="str">
-        <x:v>官网或权威来源确认的地址</x:v>
+        <x:v>官网或权威来源确认的原始地址</x:v>
       </x:c>
       <x:c r="C18" s="41" t="str">
         <x:v>API、官网或公式</x:v>
@@ -5179,10 +5181,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="41" t="str">
-        <x:v>经营范围</x:v>
+        <x:v>经营范围（原文）</x:v>
       </x:c>
       <x:c r="B19" s="41" t="str">
-        <x:v>公司经营或产品范围</x:v>
+        <x:v>API返回的公司经营或产品范围原文</x:v>
       </x:c>
       <x:c r="C19" s="41" t="str">
         <x:v>API、官网或公式</x:v>
@@ -5378,7 +5380,7 @@
         <x:v>产品名称</x:v>
       </x:c>
       <x:c r="B33" s="41" t="str">
-        <x:v>API结构化产品名</x:v>
+        <x:v>API结构化产品名；已知词优先显示中文</x:v>
       </x:c>
       <x:c r="C33" s="41" t="str">
         <x:v>API、官网或公式</x:v>
@@ -5392,7 +5394,7 @@
         <x:v>产品标签</x:v>
       </x:c>
       <x:c r="B34" s="41" t="str">
-        <x:v>API提取的产品关键词</x:v>
+        <x:v>API提取的产品关键词；已知词优先显示中文</x:v>
       </x:c>
       <x:c r="C34" s="41" t="str">
         <x:v>API、官网或公式</x:v>
@@ -5403,7 +5405,7 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="41" t="str">
-        <x:v>产品描述/命中证据</x:v>
+        <x:v>报关品名/命中证据（原文）</x:v>
       </x:c>
       <x:c r="B35" s="41" t="str">
         <x:v>原始报关品名；用于证明为何列入</x:v>
@@ -5420,7 +5422,7 @@
         <x:v>产品别名</x:v>
       </x:c>
       <x:c r="B36" s="41" t="str">
-        <x:v>API返回的近义词</x:v>
+        <x:v>API返回的近义词；已知词优先显示中文</x:v>
       </x:c>
       <x:c r="C36" s="41" t="str">
         <x:v>API、官网或公式</x:v>
@@ -5434,7 +5436,7 @@
         <x:v>上游词</x:v>
       </x:c>
       <x:c r="B37" s="41" t="str">
-        <x:v>API返回的上游关联词</x:v>
+        <x:v>API返回的上游关联词；已知词优先显示中文</x:v>
       </x:c>
       <x:c r="C37" s="41" t="str">
         <x:v>API、官网或公式</x:v>
@@ -5448,7 +5450,7 @@
         <x:v>下游词</x:v>
       </x:c>
       <x:c r="B38" s="41" t="str">
-        <x:v>API返回的下游关联词</x:v>
+        <x:v>API返回的下游关联词；已知词优先显示中文</x:v>
       </x:c>
       <x:c r="C38" s="41" t="str">
         <x:v>API、官网或公式</x:v>
@@ -5459,10 +5461,10 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="41" t="str">
-        <x:v>搜索词</x:v>
+        <x:v>搜索词（中文）</x:v>
       </x:c>
       <x:c r="B39" s="41" t="str">
-        <x:v>找到该公司的查询词</x:v>
+        <x:v>找到该公司的中文查询词</x:v>
       </x:c>
       <x:c r="C39" s="41" t="str">
         <x:v>API、官网或公式</x:v>

</xml_diff>

<commit_message>
Refresh company acquisition cost table
</commit_message>
<xml_diff>
--- a/deliverables/tape-masking-film-customer-master.xlsx
+++ b/deliverables/tape-masking-film-customer-master.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="Re892e12b2eec485c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本与流程" sheetId="2" r:id="Rb77da4a67daf42e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="Rc9fc614e7a1f46e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="R7bf6f7a824aa45cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本与流程" sheetId="2" r:id="Raeee53284a2741d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R7bad0854800a4ed3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,13 +15,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="8">
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
     <x:numFmt numFmtId="203" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="204" formatCode="0%"/>
-    <x:numFmt numFmtId="205" formatCode="&quot;¥&quot;#,##0.00"/>
+    <x:numFmt numFmtId="205" formatCode="#,##0&quot; 家&quot;"/>
+    <x:numFmt numFmtId="206" formatCode="&quot;¥&quot;#,##0.00&quot;/家&quot;"/>
+    <x:numFmt numFmtId="207" formatCode="&quot;¥&quot;#,##0.00"/>
   </x:numFmts>
   <x:fonts count="9">
     <x:font>
@@ -124,7 +126,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="48">
+  <x:cellXfs count="52">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -215,14 +217,17 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" wrapText="1"/>
@@ -231,6 +236,15 @@
       <x:alignment horizontal="right" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -673,7 +687,7 @@
       <x:c r="L3" s="15"/>
       <x:c r="M3" s="16" t="n">
         <x:f>'成本与流程'!B5</x:f>
-        <x:v>250</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="N3" s="16"/>
       <x:c r="O3" s="16"/>
@@ -26805,7 +26819,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recf177edac494896"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5483580c7b574dae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26816,7 +26830,8 @@
   <x:cols>
     <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="66" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="44" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -26831,352 +26846,375 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="40" t="str">
-        <x:v>指标</x:v>
+        <x:v>业务指标</x:v>
       </x:c>
       <x:c r="B3" s="40" t="str">
+        <x:v>公司数</x:v>
+      </x:c>
+      <x:c r="C3" s="40" t="str">
+        <x:v>计算方式</x:v>
+      </x:c>
+      <x:c r="D3" s="40" t="str">
+        <x:v>获客成本</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="41" t="str">
+        <x:v>拥有至少一种有效联系方式的公司</x:v>
+      </x:c>
+      <x:c r="B4" s="46" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="C4" s="41" t="str">
+        <x:v>¥361.60 ÷ 250</x:v>
+      </x:c>
+      <x:c r="D4" s="51" t="n">
+        <x:f>ROUND($B$14/B4,2)</x:f>
+        <x:v>1.45</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="41" t="str">
+        <x:v>拥有有效邮箱的公司</x:v>
+      </x:c>
+      <x:c r="B5" s="46" t="n">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="C5" s="41" t="str">
+        <x:v>¥361.60 ÷ 188</x:v>
+      </x:c>
+      <x:c r="D5" s="51" t="n">
+        <x:f>ROUND($B$14/B5,2)</x:f>
+        <x:v>1.92</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="41" t="str">
+        <x:v>拥有有效电话的公司</x:v>
+      </x:c>
+      <x:c r="B6" s="46" t="n">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C6" s="41" t="str">
+        <x:v>¥361.60 ÷ 196</x:v>
+      </x:c>
+      <x:c r="D6" s="51" t="n">
+        <x:f>ROUND($B$14/B6,2)</x:f>
+        <x:v>1.84</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="A7" s="41"/>
+      <x:c r="B7" s="47"/>
+      <x:c r="C7" s="41"/>
+      <x:c r="D7" s="41"/>
+    </x:row>
+    <x:row r="8" ht="28" customHeight="1">
+      <x:c r="A8" s="40" t="str">
+        <x:v>覆盖与预算</x:v>
+      </x:c>
+      <x:c r="B8" s="48" t="str">
         <x:v>结果</x:v>
       </x:c>
-      <x:c r="C3" s="40" t="str">
+      <x:c r="C8" s="40" t="str">
         <x:v>严格口径</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="41" t="str">
+      <x:c r="D8" s="41"/>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="41" t="str">
         <x:v>公司总数</x:v>
       </x:c>
-      <x:c r="B4" s="44" t="n">
+      <x:c r="B9" s="49" t="n">
         <x:v>250</x:v>
       </x:c>
-      <x:c r="C4" s="41" t="str">
+      <x:c r="C9" s="41" t="str">
         <x:v>一行一家公司ID</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="26" customHeight="1">
-      <x:c r="A5" s="41" t="str">
-        <x:v>拥有至少一种有效联系方式的公司</x:v>
-      </x:c>
-      <x:c r="B5" s="44" t="n">
-        <x:v>250</x:v>
-      </x:c>
-      <x:c r="C5" s="41" t="str">
-        <x:v>至少1个状态=1的邮箱或电话；核心总业务指标</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="26" customHeight="1">
-      <x:c r="A6" s="41" t="str">
-        <x:v>拥有有效邮箱的公司</x:v>
-      </x:c>
-      <x:c r="B6" s="44" t="n">
-        <x:v>188</x:v>
-      </x:c>
-      <x:c r="C6" s="41" t="str">
-        <x:v>至少1个状态=1的邮箱；不按邮箱数量重复计算</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="26" customHeight="1">
-      <x:c r="A7" s="41" t="str">
-        <x:v>拥有有效电话的公司</x:v>
-      </x:c>
-      <x:c r="B7" s="44" t="n">
-        <x:v>196</x:v>
-      </x:c>
-      <x:c r="C7" s="41" t="str">
-        <x:v>至少1个状态=1的电话；不按电话数量重复计算</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="26" customHeight="1">
-      <x:c r="A8" s="41" t="str">
+      <x:c r="D9" s="41"/>
+    </x:row>
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="A10" s="41" t="str">
         <x:v>邮箱和电话都有的公司</x:v>
       </x:c>
-      <x:c r="B8" s="44" t="n">
+      <x:c r="B10" s="49" t="n">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="C8" s="41" t="str">
+      <x:c r="C10" s="41" t="str">
         <x:v>同时计入邮箱公司和电话公司</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="41" t="str">
+      <x:c r="D10" s="41"/>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11" s="41" t="str">
         <x:v>只有有效邮箱的公司</x:v>
       </x:c>
-      <x:c r="B9" s="44" t="n">
+      <x:c r="B11" s="49" t="n">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="C9" s="41" t="str">
+      <x:c r="C11" s="41" t="str">
         <x:v>有有效邮箱、无有效电话</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="26" customHeight="1">
-      <x:c r="A10" s="41" t="str">
+      <x:c r="D11" s="41"/>
+    </x:row>
+    <x:row r="12" ht="28" customHeight="1">
+      <x:c r="A12" s="41" t="str">
         <x:v>只有有效电话的公司</x:v>
       </x:c>
-      <x:c r="B10" s="44" t="n">
+      <x:c r="B12" s="49" t="n">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="C10" s="41" t="str">
+      <x:c r="C12" s="41" t="str">
         <x:v>无有效邮箱、有有效电话</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="26" customHeight="1">
-      <x:c r="A11" s="41" t="str">
+      <x:c r="D12" s="41"/>
+    </x:row>
+    <x:row r="13" ht="28" customHeight="1">
+      <x:c r="A13" s="41" t="str">
         <x:v>两者都没有的公司</x:v>
       </x:c>
-      <x:c r="B11" s="44" t="n">
+      <x:c r="B13" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C11" s="41" t="str">
+      <x:c r="C13" s="41" t="str">
         <x:v>无状态=1的邮箱，也无状态=1的电话</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="26" customHeight="1">
-      <x:c r="A12" s="41" t="str">
+      <x:c r="D13" s="41"/>
+    </x:row>
+    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="A14" s="41" t="str">
         <x:v>OpenAPI累计费用</x:v>
       </x:c>
-      <x:c r="B12" s="45" t="n">
+      <x:c r="B14" s="50" t="n">
         <x:v>361.6</x:v>
       </x:c>
-      <x:c r="C12" s="41" t="str">
+      <x:c r="C14" s="41" t="str">
         <x:v>人民币；已审计本项目全部调用</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="26" customHeight="1">
-      <x:c r="A13" s="41" t="str">
-        <x:v>每家有效联系方式公司成本</x:v>
-      </x:c>
-      <x:c r="B13" s="45" t="n">
-        <x:f>ROUND(B12/B5,2)</x:f>
-        <x:v>1.45</x:v>
-      </x:c>
-      <x:c r="C13" s="41" t="str">
-        <x:v>累计费用 ÷ 拥有至少一种有效联系方式的公司</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="26" customHeight="1">
-      <x:c r="A14" s="41" t="str">
-        <x:v>每家有效邮箱公司成本</x:v>
-      </x:c>
-      <x:c r="B14" s="45" t="n">
-        <x:f>ROUND(B12/B6,2)</x:f>
-        <x:v>1.92</x:v>
-      </x:c>
-      <x:c r="C14" s="41" t="str">
-        <x:v>累计费用 ÷ 拥有有效邮箱的公司</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="26" customHeight="1">
+      <x:c r="D14" s="41"/>
+    </x:row>
+    <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="41" t="str">
-        <x:v>每家有效电话公司成本</x:v>
-      </x:c>
-      <x:c r="B15" s="45" t="n">
-        <x:f>ROUND(B12/B7,2)</x:f>
-        <x:v>1.84</x:v>
+        <x:v>预算剩余</x:v>
+      </x:c>
+      <x:c r="B15" s="50" t="n">
+        <x:f>ROUND(500-B14,2)</x:f>
+        <x:v>138.4</x:v>
       </x:c>
       <x:c r="C15" s="41" t="str">
-        <x:v>累计费用 ÷ 拥有有效电话的公司</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="26" customHeight="1">
-      <x:c r="A16" s="41" t="str">
-        <x:v>预算剩余</x:v>
-      </x:c>
-      <x:c r="B16" s="45" t="n">
-        <x:f>ROUND(500-B12,2)</x:f>
-        <x:v>138.4</x:v>
-      </x:c>
-      <x:c r="C16" s="41" t="str">
         <x:v>预算上限 ¥500.00 - 累计费用</x:v>
       </x:c>
+      <x:c r="D15" s="41"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="41"/>
+      <x:c r="B16" s="47"/>
+      <x:c r="C16" s="41"/>
+      <x:c r="D16" s="41"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="41"/>
-      <x:c r="B17" s="46"/>
-      <x:c r="C17" s="41"/>
+      <x:c r="A17" s="40" t="str">
+        <x:v>邮箱技术审计</x:v>
+      </x:c>
+      <x:c r="B17" s="48" t="str">
+        <x:v>数量</x:v>
+      </x:c>
+      <x:c r="C17" s="40" t="str">
+        <x:v>说明</x:v>
+      </x:c>
+      <x:c r="D17" s="41"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="40" t="str">
-        <x:v>邮箱技术审计</x:v>
-      </x:c>
-      <x:c r="B18" s="47" t="str">
-        <x:v>数量</x:v>
-      </x:c>
-      <x:c r="C18" s="40" t="str">
-        <x:v>说明</x:v>
-      </x:c>
+      <x:c r="A18" s="41" t="str">
+        <x:v>去重后的有效邮箱地址</x:v>
+      </x:c>
+      <x:c r="B18" s="49" t="n">
+        <x:v>277</x:v>
+      </x:c>
+      <x:c r="C18" s="41" t="str">
+        <x:v>按邮箱文本跨公司去重；不是公司级业务指标</x:v>
+      </x:c>
+      <x:c r="D18" s="41"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="41" t="str">
-        <x:v>去重后的有效邮箱地址</x:v>
-      </x:c>
-      <x:c r="B19" s="44" t="n">
-        <x:v>277</x:v>
+        <x:v>公司—邮箱有效关联记录</x:v>
+      </x:c>
+      <x:c r="B19" s="49" t="n">
+        <x:v>284</x:v>
       </x:c>
       <x:c r="C19" s="41" t="str">
-        <x:v>按邮箱文本跨公司去重；不是公司级业务指标</x:v>
-      </x:c>
+        <x:v>未跨公司去重；仅供数据审计</x:v>
+      </x:c>
+      <x:c r="D19" s="41"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="41" t="str">
-        <x:v>公司—邮箱有效关联记录</x:v>
-      </x:c>
-      <x:c r="B20" s="44" t="n">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="C20" s="41" t="str">
-        <x:v>未跨公司去重；仅供数据审计</x:v>
-      </x:c>
+      <x:c r="A20" s="41"/>
+      <x:c r="B20" s="47"/>
+      <x:c r="C20" s="41"/>
+      <x:c r="D20" s="41"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="41"/>
-      <x:c r="B21" s="46"/>
-      <x:c r="C21" s="41"/>
+      <x:c r="A21" s="40" t="str">
+        <x:v>费用构成</x:v>
+      </x:c>
+      <x:c r="B21" s="48" t="str">
+        <x:v>金额（元）</x:v>
+      </x:c>
+      <x:c r="C21" s="40" t="str">
+        <x:v>说明</x:v>
+      </x:c>
+      <x:c r="D21" s="41"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="40" t="str">
-        <x:v>费用构成</x:v>
-      </x:c>
-      <x:c r="B22" s="47" t="str">
-        <x:v>金额（元）</x:v>
-      </x:c>
-      <x:c r="C22" s="40" t="str">
-        <x:v>说明</x:v>
-      </x:c>
+      <x:c r="A22" s="41" t="str">
+        <x:v>海关客户搜索</x:v>
+      </x:c>
+      <x:c r="B22" s="50" t="n">
+        <x:v>49.5</x:v>
+      </x:c>
+      <x:c r="C22" s="41" t="str">
+        <x:v>七类产品搜索与同义词翻页</x:v>
+      </x:c>
+      <x:c r="D22" s="41"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="41" t="str">
-        <x:v>海关客户搜索</x:v>
-      </x:c>
-      <x:c r="B23" s="45" t="n">
-        <x:v>49.5</x:v>
+        <x:v>海关公司联系方式</x:v>
+      </x:c>
+      <x:c r="B23" s="50" t="n">
+        <x:v>280</x:v>
       </x:c>
       <x:c r="C23" s="41" t="str">
-        <x:v>七类产品搜索与同义词翻页</x:v>
-      </x:c>
+        <x:v>按公司ID去重后的批量联系方式</x:v>
+      </x:c>
+      <x:c r="D23" s="41"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="41" t="str">
-        <x:v>海关公司联系方式</x:v>
-      </x:c>
-      <x:c r="B24" s="45" t="n">
-        <x:v>280</x:v>
+        <x:v>人物搜索</x:v>
+      </x:c>
+      <x:c r="B24" s="50" t="n">
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="C24" s="41" t="str">
-        <x:v>按公司ID去重后的批量联系方式</x:v>
-      </x:c>
+        <x:v>混合搜索1页 + 逐公司12页</x:v>
+      </x:c>
+      <x:c r="D24" s="41"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="41" t="str">
-        <x:v>人物搜索</x:v>
-      </x:c>
-      <x:c r="B25" s="45" t="n">
-        <x:v>19.5</x:v>
+        <x:v>人物联系方式</x:v>
+      </x:c>
+      <x:c r="B25" s="50" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C25" s="41" t="str">
-        <x:v>混合搜索1页 + 逐公司12页</x:v>
-      </x:c>
+        <x:v>人工审查后仅购买6人</x:v>
+      </x:c>
+      <x:c r="D25" s="41"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="41" t="str">
-        <x:v>人物联系方式</x:v>
-      </x:c>
-      <x:c r="B26" s="45" t="n">
+        <x:v>邮箱验证</x:v>
+      </x:c>
+      <x:c r="B26" s="50" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="C26" s="41" t="str">
-        <x:v>人工审查后仅购买6人</x:v>
-      </x:c>
+        <x:v>API、官网及人物新增邮箱</x:v>
+      </x:c>
+      <x:c r="D26" s="41"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="41" t="str">
-        <x:v>邮箱验证</x:v>
-      </x:c>
-      <x:c r="B27" s="45" t="n">
-        <x:v>3</x:v>
+        <x:v>电话验证</x:v>
+      </x:c>
+      <x:c r="B27" s="50" t="n">
+        <x:v>6.6</x:v>
       </x:c>
       <x:c r="C27" s="41" t="str">
-        <x:v>API、官网及人物新增邮箱</x:v>
-      </x:c>
+        <x:v>主批58个 + 权威来源新增8个</x:v>
+      </x:c>
+      <x:c r="D27" s="41"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="41" t="str">
-        <x:v>电话验证</x:v>
-      </x:c>
-      <x:c r="B28" s="45" t="n">
-        <x:v>6.6</x:v>
-      </x:c>
-      <x:c r="C28" s="41" t="str">
-        <x:v>主批58个 + 权威来源新增8个</x:v>
-      </x:c>
+      <x:c r="A28" s="41"/>
+      <x:c r="B28" s="41"/>
+      <x:c r="C28" s="41"/>
+      <x:c r="D28" s="41"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="41"/>
-      <x:c r="B29" s="41"/>
-      <x:c r="C29" s="41"/>
+      <x:c r="A29" s="40" t="str">
+        <x:v>流程改进</x:v>
+      </x:c>
+      <x:c r="B29" s="40" t="str">
+        <x:v>优先级</x:v>
+      </x:c>
+      <x:c r="C29" s="40" t="str">
+        <x:v>执行规则</x:v>
+      </x:c>
+      <x:c r="D29" s="41"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="40" t="str">
-        <x:v>流程改进</x:v>
-      </x:c>
-      <x:c r="B30" s="40" t="str">
-        <x:v>优先级</x:v>
-      </x:c>
-      <x:c r="C30" s="40" t="str">
-        <x:v>执行规则</x:v>
-      </x:c>
+      <x:c r="A30" s="41" t="str">
+        <x:v>先做法人实体去重</x:v>
+      </x:c>
+      <x:c r="B30" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C30" s="41" t="str">
+        <x:v>公司名称+官网域名+国家归一化；重复实体复用已验证联系方式</x:v>
+      </x:c>
+      <x:c r="D30" s="41"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="41" t="str">
-        <x:v>先做法人实体去重</x:v>
+        <x:v>所有来源进入统一验证队列</x:v>
       </x:c>
       <x:c r="B31" s="41" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C31" s="41" t="str">
-        <x:v>公司名称+官网域名+国家归一化；重复实体复用已验证联系方式</x:v>
-      </x:c>
+        <x:v>API、官网、人物邮箱增量入库后立即验证；禁止只验API字段</x:v>
+      </x:c>
+      <x:c r="D31" s="41"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="41" t="str">
-        <x:v>所有来源进入统一验证队列</x:v>
+        <x:v>人物搜索按公司逐个执行</x:v>
       </x:c>
       <x:c r="B32" s="41" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C32" s="41" t="str">
-        <x:v>API、官网、人物邮箱增量入库后立即验证；禁止只验API字段</x:v>
-      </x:c>
+        <x:v>人工确认公司精确匹配后，每家公司最多购买1位高相关人员</x:v>
+      </x:c>
+      <x:c r="D32" s="41"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="41" t="str">
-        <x:v>人物搜索按公司逐个执行</x:v>
+        <x:v>状态3/0不盲目重试</x:v>
       </x:c>
       <x:c r="B33" s="41" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C33" s="41" t="str">
-        <x:v>人工确认公司精确匹配后，每家公司最多购买1位高相关人员</x:v>
-      </x:c>
+        <x:v>先查官网或换人物；避免反垃圾拦截导致重复付费</x:v>
+      </x:c>
+      <x:c r="D33" s="41"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="41" t="str">
-        <x:v>状态3/0不盲目重试</x:v>
+        <x:v>发送后用真实退信闭环</x:v>
       </x:c>
       <x:c r="B34" s="41" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C34" s="41" t="str">
-        <x:v>先查官网或换人物；避免反垃圾拦截导致重复付费</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="41" t="str">
-        <x:v>发送后用真实退信闭环</x:v>
-      </x:c>
-      <x:c r="B35" s="41" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C35" s="41" t="str">
         <x:v>小批量投递、记录硬退信、永久抑制无效地址；验证状态1仍非送达保证</x:v>
       </x:c>
+      <x:c r="D34" s="41"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Localize all business scopes in customer workbook
</commit_message>
<xml_diff>
--- a/deliverables/tape-masking-film-customer-master.xlsx
+++ b/deliverables/tape-masking-film-customer-master.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="R7bf6f7a824aa45cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本与流程" sheetId="2" r:id="Raeee53284a2741d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R7bad0854800a4ed3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户总表" sheetId="1" r:id="Rfbfec3b3f7ae4719"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本与流程" sheetId="2" r:id="R6961f001a84d450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="Rbbeff2ad57c64b64"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
     <x:tableColumn id="13" name="负责人"/>
     <x:tableColumn id="14" name="API地址（原文）"/>
     <x:tableColumn id="15" name="官网核验地址（原文）"/>
-    <x:tableColumn id="16" name="经营范围（原文）"/>
+    <x:tableColumn id="16" name="经营范围（中文）"/>
     <x:tableColumn id="17" name="匹配贸易次数"/>
     <x:tableColumn id="18" name="贸易总次数"/>
     <x:tableColumn id="19" name="匹配占比"/>
@@ -686,8 +686,8 @@
       <x:c r="K3" s="15"/>
       <x:c r="L3" s="15"/>
       <x:c r="M3" s="16" t="n">
-        <x:f>'成本与流程'!B5</x:f>
-        <x:v>188</x:v>
+        <x:f>'成本与流程'!B4</x:f>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="N3" s="16"/>
       <x:c r="O3" s="16"/>
@@ -822,7 +822,7 @@
         <x:v>官网核验地址（原文）</x:v>
       </x:c>
       <x:c r="P6" s="27" t="str">
-        <x:v>经营范围（原文）</x:v>
+        <x:v>经营范围（中文）</x:v>
       </x:c>
       <x:c r="Q6" s="27" t="str">
         <x:v>匹配贸易次数</x:v>
@@ -945,7 +945,7 @@
       </x:c>
       <x:c r="O7" s="30" t="str"/>
       <x:c r="P7" s="30" t="str">
-        <x:v>shell,shipping,bd,chi,cod,inforce,ion,hat,collated nail,oman fasteners,pro,nah,1000 c,unit,count,s 158,umber,lithium,model,sultana</x:v>
+        <x:v>外壳，航运，鳕鱼，强制，离子，帽子，排列钉，阿曼紧固件，1000，单位，计数，158，琥珀色，锂，模型，苏丹娜</x:v>
       </x:c>
       <x:c r="Q7" s="32" t="n">
         <x:v>2706</x:v>
@@ -1043,7 +1043,9 @@
         <x:v>Cerritos, California</x:v>
       </x:c>
       <x:c r="O8" s="30" t="str"/>
-      <x:c r="P8" s="30" t="str"/>
+      <x:c r="P8" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q8" s="32" t="n">
         <x:v>1587</x:v>
       </x:c>
@@ -1138,7 +1140,9 @@
         <x:v>City of Industry, California</x:v>
       </x:c>
       <x:c r="O9" s="30" t="str"/>
-      <x:c r="P9" s="30" t="str"/>
+      <x:c r="P9" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q9" s="32" t="n">
         <x:v>1008</x:v>
       </x:c>
@@ -1233,7 +1237,9 @@
         <x:v>Diamond Bar, California</x:v>
       </x:c>
       <x:c r="O10" s="30" t="str"/>
-      <x:c r="P10" s="30" t="str"/>
+      <x:c r="P10" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q10" s="32" t="n">
         <x:v>998</x:v>
       </x:c>
@@ -1333,7 +1339,7 @@
       </x:c>
       <x:c r="O11" s="30" t="str"/>
       <x:c r="P11" s="30" t="str">
-        <x:v>clear diamond,cat dish,holder set,baking cup,bag a,colour pencil,ng tube,pvc anti slip,foam sticker,cool,foam paint brush,d clip,window squeegee,plastic hoop,gs m,wort,cover,litte,xmas snowman,3 ton</x:v>
+        <x:v>透明钻石，猫盘，支架套装，烘焙杯，袋子，彩色铅笔，管，聚氯乙烯防滑，泡沫贴纸，酷，泡沫油漆刷，夹，窗户刮刀，塑料箍，麦芽汁，盖子，小，圣诞雪人，3吨</x:v>
       </x:c>
       <x:c r="Q11" s="32" t="n">
         <x:v>903</x:v>
@@ -1434,7 +1440,7 @@
       </x:c>
       <x:c r="O12" s="30" t="str"/>
       <x:c r="P12" s="30" t="str">
-        <x:v>bits,painting set,polyester fabric,colour pencil,sweat shirt,e 12,cool,desk lamp,small iron,precool,rings metal,mixed glass,xtreme,jingle bell,cotton bed linen,wooden pillar,istanbul,leren,kraft box,spice box</x:v>
+        <x:v>钻头、绘画套装、涤纶面料、彩色铅笔、运动衫、12、酷、台灯、小熨斗、预冷、金属环、混合玻璃、极限、铃儿响叮当、棉床单、木柱、伊斯坦布尔、勒伦、牛皮纸盒、香料盒</x:v>
       </x:c>
       <x:c r="Q12" s="32" t="n">
         <x:v>871</x:v>
@@ -1532,7 +1538,9 @@
         <x:v>Seattle, Washington</x:v>
       </x:c>
       <x:c r="O13" s="30" t="str"/>
-      <x:c r="P13" s="30" t="str"/>
+      <x:c r="P13" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q13" s="32" t="n">
         <x:v>690</x:v>
       </x:c>
@@ -1630,7 +1638,7 @@
       </x:c>
       <x:c r="O14" s="30" t="str"/>
       <x:c r="P14" s="30" t="str">
-        <x:v>ct a,towel,al bl,cutlery fork,smt,clear bowl,e cut,barmops,dish cloth,wash cloth,cutlery,socks</x:v>
+        <x:v>毛巾、、餐具叉、、透明碗、、拖把、洗碗布、洗碗布、餐具、袜子</x:v>
       </x:c>
       <x:c r="Q14" s="32" t="n">
         <x:v>633</x:v>
@@ -1728,7 +1736,9 @@
         <x:v>chicago, illinois, united states 1950 innovation parkway suite 100</x:v>
       </x:c>
       <x:c r="O15" s="30" t="str"/>
-      <x:c r="P15" s="30" t="str"/>
+      <x:c r="P15" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q15" s="32" t="n">
         <x:v>172</x:v>
       </x:c>
@@ -1819,7 +1829,9 @@
         <x:v>Hampshire, Illinois</x:v>
       </x:c>
       <x:c r="O16" s="30" t="str"/>
-      <x:c r="P16" s="30" t="str"/>
+      <x:c r="P16" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q16" s="32" t="n">
         <x:v>153</x:v>
       </x:c>
@@ -1911,7 +1923,7 @@
       </x:c>
       <x:c r="O17" s="30" t="str"/>
       <x:c r="P17" s="30" t="str">
-        <x:v>sol,wood,cradle,carrier,surfboard,used yacht,ipm,packing material</x:v>
+        <x:v>溶胶、木材、摇篮、载体、冲浪板、二手游艇、、包装材料</x:v>
       </x:c>
       <x:c r="Q17" s="32" t="n">
         <x:v>121</x:v>
@@ -2022,7 +2034,7 @@
       </x:c>
       <x:c r="O18" s="30" t="str"/>
       <x:c r="P18" s="30" t="str">
-        <x:v>6 oz,t rib,ilp,trigger sprayer,frost,kala chana,husk,spice jar,packaging material,chas,bottles,dropper,hkm,diamond,non medical,tin box,bottle,jar pet,foma,spray</x:v>
+        <x:v>6盎司，肋，触发喷雾器，霜，卡拉查纳，果壳，香料罐，包装材料，瓶子，滴管，钻石，非医疗，铁盒，瓶子，罐子宠物，福马，喷雾</x:v>
       </x:c>
       <x:c r="Q18" s="32" t="n">
         <x:v>90</x:v>
@@ -2128,7 +2140,9 @@
         <x:v>New York City, New York</x:v>
       </x:c>
       <x:c r="O19" s="30" t="str"/>
-      <x:c r="P19" s="30" t="str"/>
+      <x:c r="P19" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q19" s="32" t="n">
         <x:v>73</x:v>
       </x:c>
@@ -2236,7 +2250,7 @@
       </x:c>
       <x:c r="O20" s="30" t="str"/>
       <x:c r="P20" s="30" t="str">
-        <x:v>drying rack,plastic bath mat,polyester shower curtain,bamboo fiber roll,kit,board,spring link,aluminium nonstick cookware,cap to,knob,foot,plastic spray,tato,tong,liner,plastic clothes hanger,picture hanging,hooks shower curtain,cement adhesive,nns</x:v>
+        <x:v>晾衣架，塑料浴垫，涤纶浴帘，竹纤维卷，套件，木板，弹簧连杆，铝制不粘炊具，帽盖，旋钮，脚，喷塑，塔托，钳，内胆，塑料衣架，挂画，挂钩浴帘，水泥胶</x:v>
       </x:c>
       <x:c r="Q20" s="32" t="n">
         <x:v>57</x:v>
@@ -2342,7 +2356,9 @@
         <x:v>Fresh Meadows, New York</x:v>
       </x:c>
       <x:c r="O21" s="30" t="str"/>
-      <x:c r="P21" s="30" t="str"/>
+      <x:c r="P21" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q21" s="32" t="n">
         <x:v>56</x:v>
       </x:c>
@@ -2447,7 +2463,9 @@
         <x:v>Ontario, California</x:v>
       </x:c>
       <x:c r="O22" s="30" t="str"/>
-      <x:c r="P22" s="30" t="str"/>
+      <x:c r="P22" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q22" s="32" t="n">
         <x:v>45</x:v>
       </x:c>
@@ -2542,7 +2560,9 @@
         <x:v>Diamond Bar, California</x:v>
       </x:c>
       <x:c r="O23" s="30" t="str"/>
-      <x:c r="P23" s="30" t="str"/>
+      <x:c r="P23" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q23" s="32" t="n">
         <x:v>44</x:v>
       </x:c>
@@ -2637,7 +2657,9 @@
         <x:v>Torrance, California</x:v>
       </x:c>
       <x:c r="O24" s="30" t="str"/>
-      <x:c r="P24" s="30" t="str"/>
+      <x:c r="P24" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q24" s="32" t="n">
         <x:v>24</x:v>
       </x:c>
@@ -2732,7 +2754,9 @@
         <x:v>Monterey Park, California</x:v>
       </x:c>
       <x:c r="O25" s="30" t="str"/>
-      <x:c r="P25" s="30" t="str"/>
+      <x:c r="P25" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q25" s="32" t="n">
         <x:v>23</x:v>
       </x:c>
@@ -2840,7 +2864,7 @@
       </x:c>
       <x:c r="O26" s="30" t="str"/>
       <x:c r="P26" s="30" t="str">
-        <x:v>plastic pail,iron,toys,decoration,wheel,sinter,electro plated,grinding wheels,welding rods,fin,lids,electroplat,wheel plastic,core bits,welding wire,p profile,sky,core blade,fence finials,polishing pads</x:v>
+        <x:v>塑料桶、铁、玩具、装饰、砂轮、烧结、电镀、砂轮、焊条、翅片、盖子、电镀、轮塑料、芯钻头、焊丝、型材、天空、芯刀片、栅栏尖头、抛光垫</x:v>
       </x:c>
       <x:c r="Q26" s="32" t="n">
         <x:v>19</x:v>
@@ -2936,7 +2960,9 @@
         <x:v>macon, georgia, united states 723 Joe Tamplin Industria</x:v>
       </x:c>
       <x:c r="O27" s="30" t="str"/>
-      <x:c r="P27" s="30" t="str"/>
+      <x:c r="P27" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q27" s="32" t="n">
         <x:v>19</x:v>
       </x:c>
@@ -3034,7 +3060,7 @@
       </x:c>
       <x:c r="O28" s="30" t="str"/>
       <x:c r="P28" s="30" t="str">
-        <x:v>cat,ra c,pole,nido,rolls,lye,ys,altamira,d 300,alta,printed film,shipping mark,tin,polyethylene,white po,umber,ion,polyethylene film,roof,adhesivo</x:v>
+        <x:v>猫，杆，卷，碱液，阿尔塔米拉，300，阿尔塔，印刷薄膜，运输唛头，锡，聚乙烯，白粉，琥珀色，离子，聚乙烯薄膜，屋顶，粘合剂</x:v>
       </x:c>
       <x:c r="Q28" s="32" t="n">
         <x:v>17</x:v>
@@ -3126,7 +3152,9 @@
         <x:v>Baldwin Park, California</x:v>
       </x:c>
       <x:c r="O29" s="30" t="str"/>
-      <x:c r="P29" s="30" t="str"/>
+      <x:c r="P29" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q29" s="32" t="n">
         <x:v>16</x:v>
       </x:c>
@@ -3220,7 +3248,7 @@
       </x:c>
       <x:c r="O30" s="30" t="str"/>
       <x:c r="P30" s="30" t="str">
-        <x:v>ev,gg,plc,cane,pata,kit,t 23,board,chakki atta,jasmine,pen,peanuts inshell,invoice no ex,teen,freight prepaid,vat,tuff,25kg plastic bag,ppe bags,big bags 1000kg</x:v>
+        <x:v>甘蔗，套件，23，板，茉莉花，钢笔，带壳花生，无发票，青少年，运费预付，增值税，凝灰岩，25公斤塑料袋，个人防护用品袋，大袋1000公斤</x:v>
       </x:c>
       <x:c r="Q30" s="32" t="n">
         <x:v>15</x:v>
@@ -3328,7 +3356,9 @@
         <x:v>Arcadia, California</x:v>
       </x:c>
       <x:c r="O31" s="30" t="str"/>
-      <x:c r="P31" s="30" t="str"/>
+      <x:c r="P31" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q31" s="32" t="n">
         <x:v>11</x:v>
       </x:c>
@@ -3430,7 +3460,7 @@
         <x:v>7 HARBOR PARK DR, PORT WASHINGTON, NY 11050, USA</x:v>
       </x:c>
       <x:c r="P32" s="30" t="str">
-        <x:v>handtools,caulking gun,trap,cable ties,industrial plastic,clamp,paint roller,cod,ion,hammer,hawk,ratchet tie down,paint grid,trowel aluminum,pole,wood pole,bungee cord,hex key,xt,roller frame</x:v>
+        <x:v>手动工具，填缝枪，陷阱，扎带，工业塑料，夹子，油漆滚轮，鳕鱼，离子，锤子，鹰，棘轮绑带，油漆网格，抹子铝，杆，木杆，弹力绳，六角扳手，滚轮架</x:v>
       </x:c>
       <x:c r="Q32" s="32" t="n">
         <x:v>11</x:v>
@@ -3538,7 +3568,9 @@
         <x:v>Walnut, California</x:v>
       </x:c>
       <x:c r="O33" s="30" t="str"/>
-      <x:c r="P33" s="30" t="str"/>
+      <x:c r="P33" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q33" s="32" t="n">
         <x:v>10</x:v>
       </x:c>
@@ -3638,7 +3670,7 @@
         <x:v>420 Route 17 South, Mahwah, NJ 07430, USA</x:v>
       </x:c>
       <x:c r="P34" s="30" t="str">
-        <x:v>garage,ev,rubber insert,floor,high cube,un no,black vinyl,weather strip,foil duct,sheet,count,sunrise,kit,tool cart,y 100,irene,replacement seal,garage door,seal kit,a1</x:v>
+        <x:v>车库，电动车，橡胶插件，地板，高立方体，联合国编号，黑色乙烯基，密封条，铝箔管道，片材，计数，日出，套件，工具车，100，艾琳，替换密封件，车库门，密封套件，1</x:v>
       </x:c>
       <x:c r="Q34" s="32" t="n">
         <x:v>10</x:v>
@@ -3749,7 +3781,7 @@
       </x:c>
       <x:c r="O35" s="30" t="str"/>
       <x:c r="P35" s="30" t="str">
-        <x:v>adult snorkel,blush brush,straw,student,w ma,zet,dow,clip fan,bed sheet pillow,cleaning set,light dome,mahjong,paper stationery,sketchbook,cub,mail car,clpl,bands,puppy training pads,nitrile</x:v>
+        <x:v>成人通气管、腮红刷、吸管、学生、、、陶氏、夹扇、床单枕、清洁套装、灯罩、麻将、纸文具、素描本、幼崽、邮车、、乐队、小狗训练垫、丁腈</x:v>
       </x:c>
       <x:c r="Q35" s="32" t="n">
         <x:v>10</x:v>
@@ -3847,7 +3879,9 @@
         <x:v>Pomona, California</x:v>
       </x:c>
       <x:c r="O36" s="30" t="str"/>
-      <x:c r="P36" s="30" t="str"/>
+      <x:c r="P36" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q36" s="32" t="n">
         <x:v>9</x:v>
       </x:c>
@@ -3952,7 +3986,9 @@
         <x:v>Covina, California</x:v>
       </x:c>
       <x:c r="O37" s="30" t="str"/>
-      <x:c r="P37" s="30" t="str"/>
+      <x:c r="P37" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q37" s="32" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -4050,7 +4086,7 @@
       </x:c>
       <x:c r="O38" s="30" t="str"/>
       <x:c r="P38" s="30" t="str">
-        <x:v>ev,vag,t 80,k2,count,t 23,ore,rite,kr,alkyl alcohol,tar,sulphonic acid,moulds,m50,drum,marshall,yu,lanco,stanc,diamond</x:v>
+        <x:v>80，2，23，矿石，烷基醇，焦油，磺酸，模具，50，鼓，马歇尔，钻石</x:v>
       </x:c>
       <x:c r="Q38" s="32" t="n">
         <x:v>7</x:v>
@@ -4151,7 +4187,7 @@
       </x:c>
       <x:c r="O39" s="30" t="str"/>
       <x:c r="P39" s="30" t="str">
-        <x:v>Grocery products</x:v>
+        <x:v>杂货产品</x:v>
       </x:c>
       <x:c r="Q39" s="32" t="n">
         <x:v>7</x:v>
@@ -4251,7 +4287,9 @@
       <x:c r="O40" s="30" t="str">
         <x:v>1901 HARRISON ST STE 1100, OAKLAND, CA 94612-3648, USA</x:v>
       </x:c>
-      <x:c r="P40" s="30" t="str"/>
+      <x:c r="P40" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q40" s="32" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -4356,7 +4394,9 @@
         <x:v>Boston, Massachusetts</x:v>
       </x:c>
       <x:c r="O41" s="30" t="str"/>
-      <x:c r="P41" s="30" t="str"/>
+      <x:c r="P41" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q41" s="32" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -4464,7 +4504,7 @@
       </x:c>
       <x:c r="O42" s="30" t="str"/>
       <x:c r="P42" s="30" t="str">
-        <x:v>ev,pp pe bag,solar module,el box,fine crystal,gf,board,urit,y 100,d can,invoice no ex,l way,tapioca maltodextrin,drum,white pepper powder,freight prepaid,stylus pro,mater,crystal,hulled sesame seed</x:v>
+        <x:v>袋，太阳能组件，盒，细晶，板，100，罐，无发票，方式，木薯麦芽糊精，桶，白胡椒粉，运费预付，材料，水晶，去壳芝麻</x:v>
       </x:c>
       <x:c r="Q42" s="32" t="n">
         <x:v>6</x:v>
@@ -4562,7 +4602,9 @@
         <x:v>Itasca, Illinois</x:v>
       </x:c>
       <x:c r="O43" s="30" t="str"/>
-      <x:c r="P43" s="30" t="str"/>
+      <x:c r="P43" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q43" s="32" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -4660,7 +4702,7 @@
       </x:c>
       <x:c r="O44" s="30" t="str"/>
       <x:c r="P44" s="30" t="str">
-        <x:v>floor,pc plate,stainless steel mug,bicycle lock,kit,ore,st b,head light,knob,brush pet,tuff,tong,y post,cucumber,dog collar,stackable desk,liner,velvet,cleaning brush,pastel</x:v>
+        <x:v>地板，板，不锈钢杯，自行车锁，套件，矿石，头灯，旋钮，宠物刷，凝灰岩，通，柱，黄瓜，狗项圈，可堆叠桌子，衬垫，天鹅绒，清洁刷，粉彩</x:v>
       </x:c>
       <x:c r="Q44" s="32" t="n">
         <x:v>6</x:v>
@@ -4766,7 +4808,9 @@
         <x:v>Covina, California</x:v>
       </x:c>
       <x:c r="O45" s="30" t="str"/>
-      <x:c r="P45" s="30" t="str"/>
+      <x:c r="P45" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q45" s="32" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -4865,7 +4909,9 @@
         <x:v>1149 N PATT ST , BLDG B</x:v>
       </x:c>
       <x:c r="O46" s="30" t="str"/>
-      <x:c r="P46" s="30" t="str"/>
+      <x:c r="P46" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q46" s="32" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -4962,7 +5008,9 @@
         <x:v>Irwindale, California</x:v>
       </x:c>
       <x:c r="O47" s="30" t="str"/>
-      <x:c r="P47" s="30" t="str"/>
+      <x:c r="P47" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q47" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -5059,7 +5107,9 @@
         <x:v>Elmont, New York</x:v>
       </x:c>
       <x:c r="O48" s="30" t="str"/>
-      <x:c r="P48" s="30" t="str"/>
+      <x:c r="P48" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q48" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -5164,7 +5214,9 @@
         <x:v>Wood Dale, Illinois</x:v>
       </x:c>
       <x:c r="O49" s="30" t="str"/>
-      <x:c r="P49" s="30" t="str"/>
+      <x:c r="P49" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q49" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -5257,7 +5309,9 @@
         <x:v>Broomfield, Colorado</x:v>
       </x:c>
       <x:c r="O50" s="30" t="str"/>
-      <x:c r="P50" s="30" t="str"/>
+      <x:c r="P50" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q50" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -5358,7 +5412,9 @@
         <x:v>City of Industry, California</x:v>
       </x:c>
       <x:c r="O51" s="30" t="str"/>
-      <x:c r="P51" s="30" t="str"/>
+      <x:c r="P51" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q51" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -5458,7 +5514,7 @@
       </x:c>
       <x:c r="O52" s="30" t="str"/>
       <x:c r="P52" s="30" t="str">
-        <x:v>house plan,electrical control,ev,t2,pvc,electronic control,pipe fitting,ale,180 degree,electrical symbol,wooden,straight edge,som,house furnishing,design art,count,plastic pa,rasin,foam,board</x:v>
+        <x:v>房屋平面图，电气控制，2，聚氯乙烯，电子控制，管件，麦芽酒，180度，电气符号，木制，直边，家居装饰，设计艺术，计数，塑料帕，泡沫，板</x:v>
       </x:c>
       <x:c r="Q52" s="32" t="n">
         <x:v>4</x:v>
@@ -5559,7 +5615,7 @@
       </x:c>
       <x:c r="O53" s="30" t="str"/>
       <x:c r="P53" s="30" t="str">
-        <x:v>ev,mist spray,nonwoven,large car,un no,black vinyl,hair products,non woven roll,plastic bottle pump,down timer,collapsible bowl,cure,cuticle,fir,accessories hair,styling cap,holder plastic,divi,kit,t 23</x:v>
+        <x:v>电动车，喷雾，无纺布，大型汽车，联合国编号，黑色乙烯基，发制品，无纺布卷，塑料瓶泵，倒计时器，折叠碗，治疗，角质层，冷杉，配件头发，造型帽，塑料支架，迪维，套件，23</x:v>
       </x:c>
       <x:c r="Q53" s="32" t="n">
         <x:v>3</x:v>
@@ -5657,7 +5713,9 @@
         <x:v>San Francisco, California</x:v>
       </x:c>
       <x:c r="O54" s="30" t="str"/>
-      <x:c r="P54" s="30" t="str"/>
+      <x:c r="P54" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q54" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -5754,7 +5812,9 @@
         <x:v>Schiller Park, Illinois</x:v>
       </x:c>
       <x:c r="O55" s="30" t="str"/>
-      <x:c r="P55" s="30" t="str"/>
+      <x:c r="P55" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q55" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -5849,7 +5909,9 @@
         <x:v>la vergne, tennessee, united states 1 ingram boulevard</x:v>
       </x:c>
       <x:c r="O56" s="30" t="str"/>
-      <x:c r="P56" s="30" t="str"/>
+      <x:c r="P56" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q56" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -5952,7 +6014,9 @@
         <x:v>Kansas City, Missouri</x:v>
       </x:c>
       <x:c r="O57" s="30" t="str"/>
-      <x:c r="P57" s="30" t="str"/>
+      <x:c r="P57" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q57" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -6047,7 +6111,9 @@
         <x:v>Corona, California</x:v>
       </x:c>
       <x:c r="O58" s="30" t="str"/>
-      <x:c r="P58" s="30" t="str"/>
+      <x:c r="P58" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q58" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -6145,7 +6211,7 @@
       </x:c>
       <x:c r="O59" s="30" t="str"/>
       <x:c r="P59" s="30" t="str">
-        <x:v>printing paste,blu,t 24,top,cod,acrylic resin,water,ice,ink,vine,printing ink,8k,pigment dispersion,decoration,textile,ting,orange,rubi,d 21,d 300</x:v>
+        <x:v>印花色浆，蓝色，24，顶部，鳕鱼，丙烯酸树脂，水，冰，油墨，藤蔓，印刷油墨，8，颜料分散体，装饰，纺织，丁，橙色，21，300</x:v>
       </x:c>
       <x:c r="Q59" s="32" t="n">
         <x:v>3</x:v>
@@ -6245,7 +6311,9 @@
         <x:v>san diego, california, united states 6695 rasha street</x:v>
       </x:c>
       <x:c r="O60" s="30" t="str"/>
-      <x:c r="P60" s="30" t="str"/>
+      <x:c r="P60" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q60" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -6342,7 +6410,9 @@
         <x:v>Flushing, New York</x:v>
       </x:c>
       <x:c r="O61" s="30" t="str"/>
-      <x:c r="P61" s="30" t="str"/>
+      <x:c r="P61" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q61" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -6450,7 +6520,7 @@
       </x:c>
       <x:c r="O62" s="30" t="str"/>
       <x:c r="P62" s="30" t="str">
-        <x:v>huang jin,talbe,ale,clamp,sichuan,som,sweet sour sauce,pads machine,labe,vine,flavor,sos,soy sauce sweet,ginger,ppe,baby cucumber,hang,d can,lathe machine,2 ch</x:v>
+        <x:v>黄进，塔贝，麦芽酒，夹子，四川，甜酸酱，垫机，藤，风味，酱油甜，姜，小黄瓜，挂，罐，车床机，2通道</x:v>
       </x:c>
       <x:c r="Q62" s="32" t="n">
         <x:v>3</x:v>
@@ -6551,7 +6621,7 @@
       </x:c>
       <x:c r="O63" s="30" t="str"/>
       <x:c r="P63" s="30" t="str">
-        <x:v>tin lid,crt,ns a,tin cans,anillos,pre painted,pail,sheet,tinplate sheet,packaging material,handle,t san,metal pail,cube,metal ring,alambre de cobre,camp,paint,galvanized wire,as e</x:v>
+        <x:v>马口铁盖，马口铁罐，预涂，桶，片材，马口铁片，包装材料，手柄，金属桶，立方体，金属环，营地，油漆，镀锌丝</x:v>
       </x:c>
       <x:c r="Q63" s="32" t="n">
         <x:v>2</x:v>
@@ -6660,7 +6730,7 @@
       </x:c>
       <x:c r="O64" s="30" t="str"/>
       <x:c r="P64" s="30" t="str">
-        <x:v>np c,psl,ev,t2,shaft hose,wooden,epi,lever block,grease fitting,rivet,clutch cover,sea a,arm,casting clutch,flywheel assembly,unit,cy door,e ring,count,e pi</x:v>
+        <x:v>2，轴软管，木制，杠杆块，黄油嘴，铆钉，离合器盖，海，臂，铸造离合器，飞轮组件，单元，门，环，计数</x:v>
       </x:c>
       <x:c r="Q64" s="32" t="n">
         <x:v>2</x:v>
@@ -6766,7 +6836,9 @@
         <x:v>Monterey Park, California</x:v>
       </x:c>
       <x:c r="O65" s="30" t="str"/>
-      <x:c r="P65" s="30" t="str"/>
+      <x:c r="P65" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q65" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -6864,7 +6936,7 @@
       </x:c>
       <x:c r="O66" s="30" t="str"/>
       <x:c r="P66" s="30" t="str">
-        <x:v>saa,bathmats,crafts item,bath,place mat,coat,aluminium light,student,mdf wood,decorative item,cotton hand,hand woven,store bag,amb,ems,mat,apple juice,table,feet,festivities</x:v>
+        <x:v>浴室垫，工艺品，浴室，餐垫，外套，铝灯，学生，木，装饰物品，棉质手，手工编织，储物袋，垫子，苹果汁，桌子，脚，节日</x:v>
       </x:c>
       <x:c r="Q66" s="32" t="n">
         <x:v>2</x:v>
@@ -6965,7 +7037,7 @@
       </x:c>
       <x:c r="O67" s="30" t="str"/>
       <x:c r="P67" s="30" t="str">
-        <x:v>ev,ale,inflatable boat,consol,unit,bra,packaging material,kit,handle,oxygen hose,ore,differential,piston ring,non medical,lp,gear,aluminium,piston,disposable cap,tial</x:v>
+        <x:v>电动车，啤酒，充气船，控制台，单位，胸罩，包装材料，套件，手柄，氧气软管，矿石，差速器，活塞环，非医疗，齿轮，铝，活塞，一次性帽，迪亚</x:v>
       </x:c>
       <x:c r="Q67" s="32" t="n">
         <x:v>2</x:v>
@@ -7063,7 +7135,9 @@
         <x:v>Lebec, California</x:v>
       </x:c>
       <x:c r="O68" s="30" t="str"/>
-      <x:c r="P68" s="30" t="str"/>
+      <x:c r="P68" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q68" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -7158,7 +7232,9 @@
         <x:v>El Monte, California</x:v>
       </x:c>
       <x:c r="O69" s="30" t="str"/>
-      <x:c r="P69" s="30" t="str"/>
+      <x:c r="P69" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q69" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -7251,7 +7327,9 @@
         <x:v>Howard, Washington</x:v>
       </x:c>
       <x:c r="O70" s="30" t="str"/>
-      <x:c r="P70" s="30" t="str"/>
+      <x:c r="P70" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q70" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -7345,7 +7423,7 @@
       </x:c>
       <x:c r="O71" s="30" t="str"/>
       <x:c r="P71" s="30" t="str">
-        <x:v>garlic s,bamboo shoot,wood,mustard powder,red horse,esp,mat,led pl,paging machine,sea,cod,ion,cy cy,ice,salt,rdp,pickle,plant,sky,packing material</x:v>
+        <x:v>大蒜、竹笋、木材、芥末粉、红马、、垫子、发光二极管、分页机、海、鳕鱼、离子、、冰、盐、、泡菜、植物、天空、包装材料</x:v>
       </x:c>
       <x:c r="Q71" s="32" t="n">
         <x:v>2</x:v>
@@ -7456,7 +7534,7 @@
       </x:c>
       <x:c r="O72" s="30" t="str"/>
       <x:c r="P72" s="30" t="str">
-        <x:v>white cable,metal gal,glass flute,gg,nonwoven,sewing part,tradi,happy strap,needle sewing,leather art,buckle,fabric snap,e steel,kit,pap,aron,fabric,s stap,mechanical pencils,silk</x:v>
+        <x:v>白色电缆，金属加仑，玻璃笛，无纺布，缝纫部分，传统，快乐带，针缝，皮革艺术，带扣，织物按扣，钢，套件，阿伦，织物，自动铅笔，丝绸</x:v>
       </x:c>
       <x:c r="Q72" s="32" t="n">
         <x:v>2</x:v>
@@ -7565,7 +7643,7 @@
       </x:c>
       <x:c r="O73" s="30" t="str"/>
       <x:c r="P73" s="30" t="str">
-        <x:v>Hand tool bargain bin displays, impulse table displays, camo displays, four price points, box displays, pocket knife displays, eyewear displays, cargo tie-down displays, clip strip displays, peg hook displays, glasses displays, fish bowl displays, bargain bucket trees and other catalog items</x:v>
+        <x:v>手动工具特价箱展示、脉冲桌展示、迷彩展示、四个价格点、盒子展示、小刀展示、眼镜展示、货物系紧展示、夹条展示、挂钩展示、眼镜展示、鱼缸展示、特价桶树和其他目录项目</x:v>
       </x:c>
       <x:c r="Q73" s="32" t="n">
         <x:v>2</x:v>
@@ -7672,7 +7750,7 @@
       </x:c>
       <x:c r="O74" s="30" t="str"/>
       <x:c r="P74" s="30" t="str">
-        <x:v>starter,e 31,blu,delivery,mop,mop pole,large frame,wood,kraft liner,c 14,l brand,paper bag,microfiber cleaning pad,wooden,cod,ion,one pc,mala,aluminum,pole</x:v>
+        <x:v>启动器，31，蓝色，送货，拖把，拖把杆，大框架，木质，牛皮纸内衬，14，品牌，纸袋，超细纤维清洁垫，木质，鳕鱼，离子，一件，马拉，铝，杆</x:v>
       </x:c>
       <x:c r="Q74" s="32" t="n">
         <x:v>2</x:v>
@@ -7777,7 +7855,7 @@
       </x:c>
       <x:c r="O75" s="30" t="str"/>
       <x:c r="P75" s="30" t="str">
-        <x:v>hunting blind,sanshui,saa,enzyme,color glass,hook set,pe jar,seat cushion,top pet,smast,w ma,m5,foldable wagon,y68,n seal,n spotlight,w re,al bar,platform truck,poultry</x:v>
+        <x:v>狩猎百叶窗，三水，酶，彩色玻璃，挂钩组，罐，座垫，顶宠，5，折叠车，68，密封，聚光灯，平台车，家禽</x:v>
       </x:c>
       <x:c r="Q75" s="32" t="n">
         <x:v>2</x:v>
@@ -7886,7 +7964,7 @@
       </x:c>
       <x:c r="O76" s="30" t="str"/>
       <x:c r="P76" s="30" t="str">
-        <x:v>top print,blu,pet preform,pc,t 24,cod,ion,resin,ticl,arm,color bl,pellet,t 23,olo,gh,handle,recycled pet,neck,pet bottle,caps</x:v>
+        <x:v>顶部打印，蓝色，宠物预成型件，24，鳕鱼，离子，树脂，手臂，颜色，颗粒，23，手柄，再生宠物，颈部，宠物瓶，盖子</x:v>
       </x:c>
       <x:c r="Q76" s="32" t="n">
         <x:v>2</x:v>
@@ -7994,7 +8072,9 @@
         <x:v>140 E POND DR</x:v>
       </x:c>
       <x:c r="O77" s="30" t="str"/>
-      <x:c r="P77" s="30" t="str"/>
+      <x:c r="P77" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q77" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -8094,7 +8174,7 @@
       </x:c>
       <x:c r="O78" s="30" t="str"/>
       <x:c r="P78" s="30" t="str">
-        <x:v>believe,caulking gun,mowing line,hammock,ale,roller paint brush,xch,pole,safety glasses,xt,count,4 piece,hole saw kit,ledge,painting,cable clip,knife,irene,water sprayer,ppe</x:v>
+        <x:v>相信，填缝枪，割草线，吊床，啤酒，滚筒油漆刷，杆，安全眼镜，计数，4件，孔锯套件，壁架，绘画，电缆夹，刀，艾琳，喷水器，个人防护用品</x:v>
       </x:c>
       <x:c r="Q78" s="32" t="n">
         <x:v>1</x:v>
@@ -8203,7 +8283,7 @@
       </x:c>
       <x:c r="O79" s="30" t="str"/>
       <x:c r="P79" s="30" t="str">
-        <x:v>A range of kitchen and bath cabinets</x:v>
+        <x:v>一系列厨房和浴室柜</x:v>
       </x:c>
       <x:c r="Q79" s="32" t="n">
         <x:v>1</x:v>
@@ -8314,7 +8394,7 @@
       </x:c>
       <x:c r="O80" s="30" t="str"/>
       <x:c r="P80" s="30" t="str">
-        <x:v>s 10,s 15,dauber brush,cap dauber,nozzle,brush,s cap,s14,s5,brushes,s10,cap,wool dauber,tube brush,s tube,cotton swabs,510 c,s7,s 140,led cap</x:v>
+        <x:v>10，15，涂抹刷，帽涂抹，喷嘴，刷子，帽，14，5，刷子，10，帽，羊毛涂抹器，管刷，管，棉签，510，7，140，发光二极管帽</x:v>
       </x:c>
       <x:c r="Q80" s="32" t="n">
         <x:v>1</x:v>
@@ -8412,7 +8492,9 @@
         <x:v>South Carolina, USA</x:v>
       </x:c>
       <x:c r="O81" s="30" t="str"/>
-      <x:c r="P81" s="30" t="str"/>
+      <x:c r="P81" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q81" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -8507,7 +8589,9 @@
         <x:v>Santa Fe Springs, California</x:v>
       </x:c>
       <x:c r="O82" s="30" t="str"/>
-      <x:c r="P82" s="30" t="str"/>
+      <x:c r="P82" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q82" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -8610,7 +8694,9 @@
         <x:v>Diamond Bar, California</x:v>
       </x:c>
       <x:c r="O83" s="30" t="str"/>
-      <x:c r="P83" s="30" t="str"/>
+      <x:c r="P83" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q83" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -8714,7 +8800,7 @@
       </x:c>
       <x:c r="O84" s="30" t="str"/>
       <x:c r="P84" s="30" t="str">
-        <x:v>plastic plant,ev,l file,calculator,gg,cyclone,flower bath mat,sheet,pata,bicycle lock,count,fir,rubber hammer,compac,food container,locking plier,welcome mat,kit,board,peg</x:v>
+        <x:v>塑料厂，文件，计算器，旋风分离器，花浴垫，片材，自行车锁，计数，冷杉，橡胶锤，食品容器，锁钳，迎宾垫，套件，木板，钉子</x:v>
       </x:c>
       <x:c r="Q84" s="32" t="n">
         <x:v>1</x:v>
@@ -8820,7 +8906,9 @@
         <x:v>Carson, California</x:v>
       </x:c>
       <x:c r="O85" s="30" t="str"/>
-      <x:c r="P85" s="30" t="str"/>
+      <x:c r="P85" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q85" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -8928,7 +9016,7 @@
       </x:c>
       <x:c r="O86" s="30" t="str"/>
       <x:c r="P86" s="30" t="str">
-        <x:v>marble candle,flower can,angel decor,artificial flower,articles of iron,metal plant stand,ink paper,leopard,iron glass,metal and glass,wood metal art,fabric,mang,pen,tar,d can,christmas decorative item,decorative hand,round foot,wooden hand</x:v>
+        <x:v>大理石蜡烛，花罐，天使装饰，人造花，铁制品，金属植物架，墨纸，豹子，铁玻璃，金属玻璃，木金属艺术，布料，芒，钢笔，焦油，罐，圣诞装饰品，装饰手，圆脚，木手</x:v>
       </x:c>
       <x:c r="Q86" s="32" t="n">
         <x:v>1</x:v>
@@ -9034,7 +9122,9 @@
         <x:v>Moreno Valley, California</x:v>
       </x:c>
       <x:c r="O87" s="30" t="str"/>
-      <x:c r="P87" s="30" t="str"/>
+      <x:c r="P87" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q87" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -9131,7 +9221,9 @@
         <x:v>South El Monte, California</x:v>
       </x:c>
       <x:c r="O88" s="30" t="str"/>
-      <x:c r="P88" s="30" t="str"/>
+      <x:c r="P88" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q88" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -9239,7 +9331,7 @@
       </x:c>
       <x:c r="O89" s="30" t="str"/>
       <x:c r="P89" s="30" t="str">
-        <x:v>rolls,mop,yarn,reef,r 12,ale,c 14,fcl container,tin,r 11,cod,ion,r pet,brushes,s wire,s form,ice,20gp container,cotton mop head,door delivery</x:v>
+        <x:v>卷，拖把，纱线，珊瑚礁，12，啤酒，14，整箱集装箱，锡，11，鳕鱼，离子，宠物，刷子，线，表格，冰，20集装箱，棉拖把头，送货上门</x:v>
       </x:c>
       <x:c r="Q89" s="32" t="n">
         <x:v>1</x:v>
@@ -9345,7 +9437,9 @@
         <x:v>Garden City, New York</x:v>
       </x:c>
       <x:c r="O90" s="30" t="str"/>
-      <x:c r="P90" s="30" t="str"/>
+      <x:c r="P90" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q90" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -9440,7 +9534,9 @@
         <x:v>Blackstone, Massachusetts</x:v>
       </x:c>
       <x:c r="O91" s="30" t="str"/>
-      <x:c r="P91" s="30" t="str"/>
+      <x:c r="P91" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q91" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -9545,7 +9641,9 @@
         <x:v>La Mirada, California</x:v>
       </x:c>
       <x:c r="O92" s="30" t="str"/>
-      <x:c r="P92" s="30" t="str"/>
+      <x:c r="P92" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q92" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -9643,7 +9741,7 @@
       </x:c>
       <x:c r="O93" s="30" t="str"/>
       <x:c r="P93" s="30" t="str">
-        <x:v>wooden matches,carton,baby oil,made of pp,safety matche,wooden,plastic household article,kitchen match,k 400,s 155,bbq</x:v>
+        <x:v>木制火柴，纸盒，婴儿油，制成，安全火柴，木制，塑料家居用品，厨房火柴，400，155，烧烤</x:v>
       </x:c>
       <x:c r="Q93" s="32" t="n">
         <x:v>1</x:v>
@@ -9749,7 +9847,9 @@
         <x:v>Ontario, California</x:v>
       </x:c>
       <x:c r="O94" s="30" t="str"/>
-      <x:c r="P94" s="30" t="str"/>
+      <x:c r="P94" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q94" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -9844,7 +9944,9 @@
         <x:v>El Monte, California</x:v>
       </x:c>
       <x:c r="O95" s="30" t="str"/>
-      <x:c r="P95" s="30" t="str"/>
+      <x:c r="P95" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q95" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -9939,7 +10041,9 @@
         <x:v>Itasca, Illinois</x:v>
       </x:c>
       <x:c r="O96" s="30" t="str"/>
-      <x:c r="P96" s="30" t="str"/>
+      <x:c r="P96" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q96" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -10037,7 +10141,7 @@
       </x:c>
       <x:c r="O97" s="30" t="str"/>
       <x:c r="P97" s="30" t="str">
-        <x:v>stainless steel fryer,50 fan,casual set,bar set,arm,wicker,drill bit,hand tool,aed,s 158,surge,ioi,slat,s14,power cords,cock,electrica,hang,sprayer,moving blanket</x:v>
+        <x:v>不锈钢炸锅，50风扇，休闲套装，吧台套装，手臂，柳条，钻头，手动工具，158，浪涌，板条，14，电源线，旋塞，电动，挂，喷雾器，移动毯</x:v>
       </x:c>
       <x:c r="Q97" s="32" t="n">
         <x:v>1</x:v>
@@ -10145,7 +10249,9 @@
         <x:v>3428 SW 15TH ST</x:v>
       </x:c>
       <x:c r="O98" s="30" t="str"/>
-      <x:c r="P98" s="30" t="str"/>
+      <x:c r="P98" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q98" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -10245,7 +10351,7 @@
       </x:c>
       <x:c r="O99" s="30" t="str"/>
       <x:c r="P99" s="30" t="str">
-        <x:v>cod,chain,chain part,sprocket,roller chain</x:v>
+        <x:v>鳕鱼，链条，链条零件，链轮，滚子链条</x:v>
       </x:c>
       <x:c r="Q99" s="32" t="n">
         <x:v>1</x:v>
@@ -10344,7 +10450,7 @@
       </x:c>
       <x:c r="O100" s="30" t="str"/>
       <x:c r="P100" s="30" t="str">
-        <x:v>hmi,wooden,giant,mats,card,count,packaging material,model,static cling,board,cene,ppe,st b,brass,tar,s 10,family,plastic game,elvie,freeze</x:v>
+        <x:v>木制，巨人，垫子，卡片，计数，包装材料，模型，静电吸附，板，黄铜，焦油，10，家庭，塑料游戏，埃尔维，冻结</x:v>
       </x:c>
       <x:c r="Q100" s="32" t="n">
         <x:v>1</x:v>
@@ -10440,7 +10546,9 @@
         <x:v>Pomona, California</x:v>
       </x:c>
       <x:c r="O101" s="30" t="str"/>
-      <x:c r="P101" s="30" t="str"/>
+      <x:c r="P101" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q101" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -10538,7 +10646,7 @@
       </x:c>
       <x:c r="O102" s="30" t="str"/>
       <x:c r="P102" s="30" t="str">
-        <x:v>shell,fork,wood,fittings,pipe,pump part,ingco,ceramic filter,cod,cylinder,slurry tank,e motor,shackle,e gear,base engine,unit,submersible pump parts,base valve,aker,packaging material</x:v>
+        <x:v>外壳、叉子、木材、配件、管道、泵零件、、陶瓷过滤器、鳕鱼、气缸、浆料罐、电机、卸扣、齿轮、基础发动机、单元、潜水泵零件、底阀、阿克、包装材料</x:v>
       </x:c>
       <x:c r="Q102" s="32" t="n">
         <x:v>1</x:v>
@@ -10648,7 +10756,9 @@
         <x:v>PO BOX 3</x:v>
       </x:c>
       <x:c r="O103" s="30" t="str"/>
-      <x:c r="P103" s="30" t="str"/>
+      <x:c r="P103" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q103" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -10757,7 +10867,9 @@
         <x:v>14943 DESMAN RD</x:v>
       </x:c>
       <x:c r="O104" s="30" t="str"/>
-      <x:c r="P104" s="30" t="str"/>
+      <x:c r="P104" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q104" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -10867,7 +10979,7 @@
       </x:c>
       <x:c r="O105" s="30" t="str"/>
       <x:c r="P105" s="30" t="str">
-        <x:v>Toilet preparations, such as perfumes, shaving preparations, hair preparations, face creams, lotions, and other cosmetic preparations</x:v>
+        <x:v>盥洗用品，例如香水、剃须用品、护发用品、面霜、乳液和其他化妆品制剂</x:v>
       </x:c>
       <x:c r="Q105" s="32" t="n">
         <x:v>1</x:v>
@@ -10975,7 +11087,9 @@
         <x:v>Chino, California</x:v>
       </x:c>
       <x:c r="O106" s="30" t="str"/>
-      <x:c r="P106" s="30" t="str"/>
+      <x:c r="P106" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q106" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -11073,7 +11187,7 @@
       </x:c>
       <x:c r="O107" s="30" t="str"/>
       <x:c r="P107" s="30" t="str">
-        <x:v>ether,front axle beam,g al,motor v,wood box,no n,machine,durable torch,60 cbm,card,electric towel,williams,count,unit,14k,d box,asb,kit,truck,board</x:v>
+        <x:v>乙醚，前轴梁，电机，木箱，无，机，耐用手电筒，60立方米，卡，电热毛巾，威廉姆斯，计数，单位，14，盒，套件，卡车，板</x:v>
       </x:c>
       <x:c r="Q107" s="32" t="n">
         <x:v>1</x:v>
@@ -11179,7 +11293,9 @@
         <x:v>02160, г.киев, пр.воссоединения 7а, оф.212а</x:v>
       </x:c>
       <x:c r="O108" s="30" t="str"/>
-      <x:c r="P108" s="30" t="str"/>
+      <x:c r="P108" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q108" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -11273,7 +11389,7 @@
       </x:c>
       <x:c r="O109" s="30" t="str"/>
       <x:c r="P109" s="30" t="str">
-        <x:v>storage card,mechnical seals,latch hook,heat engine,apparatus for measuring the flow of gases,self-adhesive tape,extractor,plastic lamp,optical reader,label of paper,plastic cap,electromagnet,explorer,trucks,trash can,frame,expansion valve,hand shank,light emitting diodes,lock parts</x:v>
+        <x:v>存储卡、机械密封件、插销钩、热机、气体流量测量仪、自粘胶带、提取器、塑料灯、光学阅读器、纸标签、塑料盖、电磁铁、探险家、卡车、垃圾桶、框架、膨胀阀、手柄、发光二极管、锁部件</x:v>
       </x:c>
       <x:c r="Q109" s="32" t="n">
         <x:v>9024</x:v>
@@ -11379,7 +11495,9 @@
         <x:v>B-14 &amp; 15 , NOIDA PHASE II</x:v>
       </x:c>
       <x:c r="O110" s="30" t="str"/>
-      <x:c r="P110" s="30" t="str"/>
+      <x:c r="P110" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q110" s="32" t="n">
         <x:v>7587</x:v>
       </x:c>
@@ -11488,7 +11606,9 @@
         <x:v>GRUPO LAAR , DE LOS CIPRESES N26 , CARCELEN INDUSTRIAL</x:v>
       </x:c>
       <x:c r="O111" s="30" t="str"/>
-      <x:c r="P111" s="30" t="str"/>
+      <x:c r="P111" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q111" s="32" t="n">
         <x:v>6944</x:v>
       </x:c>
@@ -11588,7 +11708,7 @@
       </x:c>
       <x:c r="O112" s="30" t="str"/>
       <x:c r="P112" s="30" t="str">
-        <x:v>Offers industrial and commercial electric apparatus and other equipment which include power converters (i.E., AC to DC and DC to AC), power supplies, surge suppressors, and similar equipment for industrial-type and consumer-type equipment</x:v>
+        <x:v>提供工业和商业电气设备和其他设备，包括电源转换器（即交流到直流和直流到交流）、电源、浪涌抑制器以及适用于工业型和消费型设备的类似设备</x:v>
       </x:c>
       <x:c r="Q112" s="32" t="n">
         <x:v>5800</x:v>
@@ -11691,7 +11811,7 @@
       </x:c>
       <x:c r="O113" s="30" t="str"/>
       <x:c r="P113" s="30" t="str">
-        <x:v>Wireless communications products</x:v>
+        <x:v>无线通讯产品</x:v>
       </x:c>
       <x:c r="Q113" s="32" t="n">
         <x:v>4462</x:v>
@@ -11790,7 +11910,7 @@
       </x:c>
       <x:c r="O114" s="30" t="str"/>
       <x:c r="P114" s="30" t="str">
-        <x:v>elastan,arrow,al bl,8 gsm,shirts,manmade fiber,cotton organic,bra size,structure,knit fabric,ciq,knitted fabric,hand tag,cacique,dow,cacl,table,twill,rubber yarn,blu</x:v>
+        <x:v>弹性纤维，箭头，8，衬衫，化学纤维，有机棉，胸罩尺寸，结构，针织面料，针织面料，手牌，酋长，陶氏化学，桌子，斜纹布，橡胶纱，蓝色</x:v>
       </x:c>
       <x:c r="Q114" s="32" t="n">
         <x:v>4245</x:v>
@@ -11885,7 +12005,7 @@
       </x:c>
       <x:c r="O115" s="30" t="str"/>
       <x:c r="P115" s="30" t="str">
-        <x:v>granules of pig iron,record sleeves,wires,display,fire fighting truck,cu products,glues based on starches,air filter,coupler cable,hydraulic machine,cotters,wrench sockets,panel,plastic bag,steel parts,tyre,light emitting diodes,stoppers,gemalto,camera</x:v>
+        <x:v>生铁颗粒、唱片套、电线、显示器、消防车、铜产品、淀粉胶、空气过滤器、耦合电缆、液压机、开口销、扳手套筒、面板、塑料袋、钢件、轮胎、发光二极管、塞子、金雅拓、相机</x:v>
       </x:c>
       <x:c r="Q115" s="32" t="n">
         <x:v>3623</x:v>
@@ -11992,7 +12112,7 @@
       </x:c>
       <x:c r="O116" s="30" t="str"/>
       <x:c r="P116" s="30" t="str">
-        <x:v>three hole,taping machine,mmmm,5w power supply,instruction,pressure switch,housing pcb,format,h pin,ssd 256gb,70w street light,teflon,remo,wash machine,printing,insulated pad,machine,insula,locking sleeve,12w bulb</x:v>
+        <x:v>三孔，编带机，5电源，说明书，压力开关，外壳，格式，针，256，70路灯，铁氟龙，雷莫，洗衣机，印刷，绝缘垫，机器，绝缘体，锁紧套，12灯泡</x:v>
       </x:c>
       <x:c r="Q116" s="32" t="n">
         <x:v>2538</x:v>
@@ -12095,7 +12215,7 @@
       </x:c>
       <x:c r="O117" s="30" t="str"/>
       <x:c r="P117" s="30" t="str">
-        <x:v>ticl,ceo,yan,other textile,products</x:v>
+        <x:v>其他纺织，产品</x:v>
       </x:c>
       <x:c r="Q117" s="32" t="n">
         <x:v>2442</x:v>
@@ -12194,7 +12314,7 @@
       </x:c>
       <x:c r="O118" s="30" t="str"/>
       <x:c r="P118" s="30" t="str">
-        <x:v>plastic core-rubber-tires,rubber product,printing ink,vitriol,textile fabrics,deco film,aluminum paper,tester,butyl,plastic,gearing,electrical machinery,semi-colloidal graphite,plastics,stamping punching,plastic polyester resin,coil,acrylic resin,web,printer</x:v>
+        <x:v>胶芯橡胶轮胎、橡胶制品、印刷油墨、硫酸、纺织面料、装饰膜、铝纸、测试仪、丁基、塑料、齿轮、电机、半胶体石墨、塑料、冲压冲孔、塑料聚酯树脂、卷材、丙烯酸树脂、卷筒纸、打印机</x:v>
       </x:c>
       <x:c r="Q118" s="32" t="n">
         <x:v>2311</x:v>
@@ -12295,7 +12415,7 @@
       </x:c>
       <x:c r="O119" s="30" t="str"/>
       <x:c r="P119" s="30" t="str">
-        <x:v>arm,latch,relay box,pinion,manifold,rear view,rear hub,x7,rain,spring pad,cyl head,sas,fork,nks,anten,seat rear,alum,knob,erco,signal</x:v>
+        <x:v>臂，闩锁，继电器盒，小齿轮，歧管，后视图，后轮毂，7，雨，弹簧垫，气缸头，叉，座椅后部，明矾，旋钮，信号</x:v>
       </x:c>
       <x:c r="Q119" s="32" t="n">
         <x:v>2061</x:v>
@@ -12396,7 +12516,7 @@
       </x:c>
       <x:c r="O120" s="30" t="str"/>
       <x:c r="P120" s="30" t="str">
-        <x:v>cam part,gum,rys,connect parts,partition board,harness,opal,demo kit,t series,kick,brown carton,side board,pin mould,alfa,dry reed,damping spring,shock,deep gray,front cover,t seal</x:v>
+        <x:v>凸轮部件，口香糖，连接部件，隔板，线束，蛋白石，演示套件，系列，踢脚，棕色纸箱，侧板，销模，阿尔法，干簧片，阻尼弹簧，减震，深灰色，前盖，型密封</x:v>
       </x:c>
       <x:c r="Q120" s="32" t="n">
         <x:v>1941</x:v>
@@ -12505,7 +12625,7 @@
       </x:c>
       <x:c r="O121" s="30" t="str"/>
       <x:c r="P121" s="30" t="str">
-        <x:v>Women's lingerie, as well as clothing products for in-house and leisure purposes</x:v>
+        <x:v>女士内衣以及室内和休闲服装产品</x:v>
       </x:c>
       <x:c r="Q121" s="32" t="n">
         <x:v>1878</x:v>
@@ -12599,7 +12719,9 @@
         <x:v>DONG AN QUARTER , TAN DONG HIEP WARD , DI AN DIST</x:v>
       </x:c>
       <x:c r="O122" s="30" t="str"/>
-      <x:c r="P122" s="30" t="str"/>
+      <x:c r="P122" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q122" s="32" t="n">
         <x:v>1828</x:v>
       </x:c>
@@ -12697,7 +12819,7 @@
       </x:c>
       <x:c r="O123" s="30" t="str"/>
       <x:c r="P123" s="30" t="str">
-        <x:v>1 8m,lye,ice,wheel,8k,metal slide,wired bra,white po,micromesh,keyboard,simplex,iu,s20,cod,5d,c printed fabric,ribbon item,spb,laminated foam,board</x:v>
+        <x:v>18、碱液、冰、轮、8、金属滑轨、钢丝文胸、白宝、微网、键盘、单面、、20、、5、印花织物、丝带项目、、层压泡沫、板</x:v>
       </x:c>
       <x:c r="Q123" s="32" t="n">
         <x:v>1677</x:v>
@@ -12796,7 +12918,7 @@
       </x:c>
       <x:c r="O124" s="30" t="str"/>
       <x:c r="P124" s="30" t="str">
-        <x:v>plated circuit,deco film,printed circuits,electronic intergrated circuits,industrial steel material,loudspeaker,pressing punching,stamping punching,sticker,plastic product,plastics,connector</x:v>
+        <x:v>电镀电路、装饰膜、印刷电路、电子集成电路、工业钢材、扬声器、冲压冲孔、冲压冲孔、不干胶、塑料制品、塑料、连接器</x:v>
       </x:c>
       <x:c r="Q124" s="32" t="n">
         <x:v>1517</x:v>
@@ -12905,7 +13027,7 @@
       </x:c>
       <x:c r="O125" s="30" t="str"/>
       <x:c r="P125" s="30" t="str">
-        <x:v>cot,plastic machine,plastic product,crochd,synthetic fibres,stitch-bonded fibre fabrics,textile fabrics,composition leather,dyed woven cotton fabric,waterproof paper,rey,twine,cables of abaca,texturd polyester,dresses,sewing thread of synthetic staple fibres,rayon,statuettes of plastics,fabrics of synthetic fibres,tailoring machine</x:v>
+        <x:v>胶床、塑料机械、塑料制品、鳄鱼布、合纤、缝编布、纺织面料、合成革、色织棉布、防水纸、雷、麻线、蕉麻线、聚酯纤维、连衣裙、合纤短纤缝纫线、人造丝、塑料雕像、合纤织物、裁缝机</x:v>
       </x:c>
       <x:c r="Q125" s="32" t="n">
         <x:v>1476</x:v>
@@ -13005,7 +13127,9 @@
         <x:v>NETAJI SUBHASH PLACE, OPPOSITE WAZIRPUR DTC DEPOT, PITAMPURA , 414, 4TH FLOOR, D MALL</x:v>
       </x:c>
       <x:c r="O126" s="30" t="str"/>
-      <x:c r="P126" s="30" t="str"/>
+      <x:c r="P126" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q126" s="32" t="n">
         <x:v>1440</x:v>
       </x:c>
@@ -13114,7 +13238,9 @@
         <x:v>Miami, Florida</x:v>
       </x:c>
       <x:c r="O127" s="30" t="str"/>
-      <x:c r="P127" s="30" t="str"/>
+      <x:c r="P127" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q127" s="32" t="n">
         <x:v>1398</x:v>
       </x:c>
@@ -13208,7 +13334,7 @@
       </x:c>
       <x:c r="O128" s="30" t="str"/>
       <x:c r="P128" s="30" t="str">
-        <x:v>production line,compac,qsfp,wifi router,md,display s,clean table,cable fixing,back camera,1 sim,cutter device,lumi,defoam,easel,color box,crown,bbl,battery connector,hook connector,al cable</x:v>
+        <x:v>生产线，无线网络路由器，显示器，清洁台，电缆固定，后置摄像头，1，切割装置，消泡，画架，彩盒，皇冠，电池连接器，挂钩连接器，铝电缆</x:v>
       </x:c>
       <x:c r="Q128" s="32" t="n">
         <x:v>1379</x:v>
@@ -13311,7 +13437,7 @@
       </x:c>
       <x:c r="O129" s="30" t="str"/>
       <x:c r="P129" s="30" t="str">
-        <x:v>Self-adhesive·products·and·solutions</x:v>
+        <x:v>自粘·产品·和·解决方案</x:v>
       </x:c>
       <x:c r="Q129" s="32" t="n">
         <x:v>1322</x:v>
@@ -13418,7 +13544,7 @@
       </x:c>
       <x:c r="O130" s="30" t="str"/>
       <x:c r="P130" s="30" t="str">
-        <x:v>bits,accesorios,export document,agent,abro,13 pocket,a 60,caja de,le par,tipo,vin,carton,e 12,yt,hot rolled,packaged,moisture content,water tank,s 140,inco</x:v>
+        <x:v>钻头，配件，出口文件，代理，13口袋，60，纸箱，12，热轧，包装，水分含量，水箱，140</x:v>
       </x:c>
       <x:c r="Q130" s="32" t="n">
         <x:v>1247</x:v>
@@ -13519,7 +13645,7 @@
       </x:c>
       <x:c r="O131" s="30" t="str"/>
       <x:c r="P131" s="30" t="str">
-        <x:v>torc,k 12,cat,t 16,e 200,rtp,sva,d 13,cle,sulfuric acid,caza,open version,facture,silver,blu,bajaj auto,belo,he i,scooters,abs black</x:v>
+        <x:v>12，16，200，13，硫酸，开放版，银色，蓝色，贝洛，踏板车，工程塑料黑色</x:v>
       </x:c>
       <x:c r="Q131" s="32" t="n">
         <x:v>1011</x:v>
@@ -13620,7 +13746,7 @@
       </x:c>
       <x:c r="O132" s="30" t="str"/>
       <x:c r="P132" s="30" t="str">
-        <x:v>oil spec,troll,polyester film,thermocouple,bmc injection machine,varnish,support unit,magnetic sensor,black sf,connector housing,bearing holder,standard a,protec,hydraulic pump,nut runner,m5,key,solenoid valve,lank,diode lead</x:v>
+        <x:v>油规格，巨魔，聚酯薄膜，热电偶，注射机，清漆，支撑单元，磁性传感器，黑色，连接器外壳，轴承座，标准，液压泵，螺母扳手，5，钥匙，电磁阀，兰克，二极管引线</x:v>
       </x:c>
       <x:c r="Q132" s="32" t="n">
         <x:v>1008</x:v>
@@ -13718,7 +13844,9 @@
         <x:v>NOKIA TELECOM SEZ , SIPCOT INDUSTRIAL PARK , PHASE III, SRIPERUMBUDUR</x:v>
       </x:c>
       <x:c r="O133" s="30" t="str"/>
-      <x:c r="P133" s="30" t="str"/>
+      <x:c r="P133" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q133" s="32" t="n">
         <x:v>941</x:v>
       </x:c>
@@ -13820,7 +13948,7 @@
       </x:c>
       <x:c r="O134" s="30" t="str"/>
       <x:c r="P134" s="30" t="str">
-        <x:v>Cleaning equipment</x:v>
+        <x:v>清洁设备</x:v>
       </x:c>
       <x:c r="Q134" s="32" t="n">
         <x:v>713</x:v>
@@ -13925,7 +14053,7 @@
       </x:c>
       <x:c r="O135" s="30" t="str"/>
       <x:c r="P135" s="30" t="str">
-        <x:v>Leather goods</x:v>
+        <x:v>皮具</x:v>
       </x:c>
       <x:c r="Q135" s="32" t="n">
         <x:v>633</x:v>
@@ -14030,7 +14158,7 @@
       </x:c>
       <x:c r="O136" s="30" t="str"/>
       <x:c r="P136" s="30" t="str">
-        <x:v>Motor vehicle parts and accessories</x:v>
+        <x:v>机动车辆零配件</x:v>
       </x:c>
       <x:c r="Q136" s="32" t="n">
         <x:v>530</x:v>
@@ -14128,7 +14256,9 @@
         <x:v>NO. 27, GROUND FLOOR RECTANGLE-1, SAKET DISTRICT CENTRE , NO. D-4 , SAKET</x:v>
       </x:c>
       <x:c r="O137" s="30" t="str"/>
-      <x:c r="P137" s="30" t="str"/>
+      <x:c r="P137" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q137" s="32" t="n">
         <x:v>375</x:v>
       </x:c>
@@ -14235,7 +14365,9 @@
         <x:v>SIKKIM COMMERCE HOUSE, SIXTH FLOOR, NO. 4/1, MIDDLETON STREET</x:v>
       </x:c>
       <x:c r="O138" s="30" t="str"/>
-      <x:c r="P138" s="30" t="str"/>
+      <x:c r="P138" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q138" s="32" t="n">
         <x:v>220</x:v>
       </x:c>
@@ -14337,7 +14469,7 @@
       </x:c>
       <x:c r="O139" s="30" t="str"/>
       <x:c r="P139" s="30" t="str">
-        <x:v>Operation of a shopping mall; Consumer goods and services</x:v>
+        <x:v>经营购物中心；消费品和服务</x:v>
       </x:c>
       <x:c r="Q139" s="32" t="n">
         <x:v>126</x:v>
@@ -14446,7 +14578,7 @@
       </x:c>
       <x:c r="O140" s="30" t="str"/>
       <x:c r="P140" s="30" t="str">
-        <x:v>Machinery and equipment for the construction, infrastructure, quarrying, mining, shipping, transportation, refining, and utility industries</x:v>
+        <x:v>用于建筑、基础设施、采石、采矿、航运、运输、炼油和公用事业行业的机械和设备</x:v>
       </x:c>
       <x:c r="Q140" s="32" t="n">
         <x:v>87</x:v>
@@ -14557,7 +14689,7 @@
       </x:c>
       <x:c r="O141" s="30" t="str"/>
       <x:c r="P141" s="30" t="str">
-        <x:v>double side,nozzle plastic,straight type,aspire,cock,r 12,big clip,brochure,waist support,big core,plunger,carton,r bra,water tank,bharat,heavy belt,w re,automat,plastic stand,drill</x:v>
+        <x:v>双面，吸嘴塑料，直型，公鸡，12，大夹子，宣传册，护腰，大芯，柱塞，纸箱，胸罩，水箱，巴拉特，重型皮带，自动机，塑料支架，钻头</x:v>
       </x:c>
       <x:c r="Q141" s="32" t="n">
         <x:v>81</x:v>
@@ -14656,7 +14788,7 @@
       </x:c>
       <x:c r="O142" s="30" t="str"/>
       <x:c r="P142" s="30" t="str">
-        <x:v>Biological and medical products, botanical drugs and herbs, and pharmaceutical products intended for internal and external consumption in such forms as ampoules, tablets, capsules, vials, ointments, powders, solutions, and suspensions; Bandages, beauty preparations, colognes, cosmetics, dentifrices, deodorants, diagnostic reagents, first-aid supplies, hair preparations, toilet soaps, and toiletries</x:v>
+        <x:v>生物和医疗产品、植物药物和草药，以及供内部和外部消费的安瓿、片剂、胶囊、小瓶、软膏、粉末、溶液和悬浮液等形式的药品；绷带、美容用品、古龙水、化妆品、牙膏、除臭剂、诊断试剂、急救用品、护发剂、香皂和盥洗用品</x:v>
       </x:c>
       <x:c r="Q142" s="32" t="n">
         <x:v>72</x:v>
@@ -14756,7 +14888,9 @@
         <x:v>SEVENTH FLOOR, PARAS TWIN TOWER , GOLF COURSE ROAD , SECTOR-54</x:v>
       </x:c>
       <x:c r="O143" s="30" t="str"/>
-      <x:c r="P143" s="30" t="str"/>
+      <x:c r="P143" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q143" s="32" t="n">
         <x:v>66</x:v>
       </x:c>
@@ -14854,7 +14988,7 @@
       </x:c>
       <x:c r="O144" s="30" t="str"/>
       <x:c r="P144" s="30" t="str">
-        <x:v>made up article,cotton terry towel,bath towel,8 inc</x:v>
+        <x:v>化妆用品、棉毛巾、浴巾、8件</x:v>
       </x:c>
       <x:c r="Q144" s="32" t="n">
         <x:v>64</x:v>
@@ -14961,7 +15095,7 @@
       </x:c>
       <x:c r="O145" s="30" t="str"/>
       <x:c r="P145" s="30" t="str">
-        <x:v>coat,m5,vechi,cam shaft,digital finger counter,led bulb 11w,cotton buds,table,sn 99,brake shoe,makeup,piston,steel nail,electric shaver,electroplat,hair shaver,lipgloss,plastic,steel pot,u bra</x:v>
+        <x:v>外套，5，凸轮轴，数指计数器，发光二极管灯泡11，棉签，桌子，99，刹车蹄，化妆，活塞，钢钉，电动剃须刀，电镀，剃须刀，唇彩，塑料，钢锅，胸罩</x:v>
       </x:c>
       <x:c r="Q145" s="32" t="n">
         <x:v>59</x:v>
@@ -15069,7 +15203,9 @@
         <x:v>FLAT NO. 203 &amp; 204 , 2ND FLOOR , A-WING, DELPHI BLDG CENTRAL AVENUE, HIRANANDANI BUSINESS PARK,POWAI MUMBAI</x:v>
       </x:c>
       <x:c r="O146" s="30" t="str"/>
-      <x:c r="P146" s="30" t="str"/>
+      <x:c r="P146" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q146" s="32" t="n">
         <x:v>41</x:v>
       </x:c>
@@ -15179,7 +15315,7 @@
       </x:c>
       <x:c r="O147" s="30" t="str"/>
       <x:c r="P147" s="30" t="str">
-        <x:v>Plastic bottles, blow moulding multilayer bottles, injection moulding articals, measuring cups, multiwall polycarbonate sheets, and ultra lite multiwall polycobonate sheet</x:v>
+        <x:v>塑料瓶、吹塑多层瓶、注塑制品、量杯、多层聚碳酸酯片材和超轻多层聚碳酸酯片材</x:v>
       </x:c>
       <x:c r="Q147" s="32" t="n">
         <x:v>28</x:v>
@@ -15288,7 +15424,7 @@
       </x:c>
       <x:c r="O148" s="30" t="str"/>
       <x:c r="P148" s="30" t="str">
-        <x:v>Pharmaceuticals, prescriptions, over-the-counter drugs, health and beauty products, and general merchandise</x:v>
+        <x:v>药品、处方药、非处方药、保健和美容产品以及日用商品</x:v>
       </x:c>
       <x:c r="Q148" s="32" t="n">
         <x:v>26</x:v>
@@ -15399,7 +15535,7 @@
       </x:c>
       <x:c r="O149" s="30" t="str"/>
       <x:c r="P149" s="30" t="str">
-        <x:v>Cosmetics and other related products (skin care, hair care, hair coloring, make-up and styling products)</x:v>
+        <x:v>化妆品及其他相关产品（护肤、护发、染发、彩妆及造型产品）</x:v>
       </x:c>
       <x:c r="Q149" s="32" t="n">
         <x:v>26</x:v>
@@ -15512,7 +15648,7 @@
       </x:c>
       <x:c r="O150" s="30" t="str"/>
       <x:c r="P150" s="30" t="str">
-        <x:v>Wire harnesses and related products</x:v>
+        <x:v>线束及相关产品</x:v>
       </x:c>
       <x:c r="Q150" s="32" t="n">
         <x:v>23</x:v>
@@ -15613,7 +15749,7 @@
       </x:c>
       <x:c r="O151" s="30" t="str"/>
       <x:c r="P151" s="30" t="str">
-        <x:v>Cosmetic products</x:v>
+        <x:v>化妆品</x:v>
       </x:c>
       <x:c r="Q151" s="32" t="n">
         <x:v>23</x:v>
@@ -15722,7 +15858,7 @@
       </x:c>
       <x:c r="O152" s="30" t="str"/>
       <x:c r="P152" s="30" t="str">
-        <x:v>Oil and gas field machinery and equipment, and other related petroleum exploring special equipment</x:v>
+        <x:v>油气田机械设备及其他相关石油勘探专用设备</x:v>
       </x:c>
       <x:c r="Q152" s="32" t="n">
         <x:v>22</x:v>
@@ -15833,7 +15969,7 @@
       </x:c>
       <x:c r="O153" s="30" t="str"/>
       <x:c r="P153" s="30" t="str">
-        <x:v>Motorcycles and motorcycle accessories</x:v>
+        <x:v>摩托车及摩托车配件</x:v>
       </x:c>
       <x:c r="Q153" s="32" t="n">
         <x:v>19</x:v>
@@ -15946,7 +16082,7 @@
       </x:c>
       <x:c r="O154" s="30" t="str"/>
       <x:c r="P154" s="30" t="str">
-        <x:v>Women's clothing</x:v>
+        <x:v>女装</x:v>
       </x:c>
       <x:c r="Q154" s="32" t="n">
         <x:v>18</x:v>
@@ -16055,7 +16191,7 @@
       </x:c>
       <x:c r="O155" s="30" t="str"/>
       <x:c r="P155" s="30" t="str">
-        <x:v>Yarn and textile fibers</x:v>
+        <x:v>纱线和纺织纤维</x:v>
       </x:c>
       <x:c r="Q155" s="32" t="n">
         <x:v>18</x:v>
@@ -16154,7 +16290,7 @@
       </x:c>
       <x:c r="O156" s="30" t="str"/>
       <x:c r="P156" s="30" t="str">
-        <x:v>Home furnishings and other related products</x:v>
+        <x:v>家居用品及其他相关产品</x:v>
       </x:c>
       <x:c r="Q156" s="32" t="n">
         <x:v>17</x:v>
@@ -16263,7 +16399,7 @@
       </x:c>
       <x:c r="O157" s="30" t="str"/>
       <x:c r="P157" s="30" t="str">
-        <x:v>Offers aircraft management, business and general aviation MRO, commercial aviation MRO, and avionics upgrade and retrofit services</x:v>
+        <x:v>提供飞机管理、公务和通用航空维护维修运行、商业航空维护维修运行以及航电升级和改造服务</x:v>
       </x:c>
       <x:c r="Q157" s="32" t="n">
         <x:v>16</x:v>
@@ -16374,7 +16510,7 @@
       </x:c>
       <x:c r="O158" s="30" t="str"/>
       <x:c r="P158" s="30" t="str">
-        <x:v>Cars, trucks, vans and mini vans, and SUVs (sport utility vehicles)</x:v>
+        <x:v>汽车、卡车、货车和小型货车以及运动型多用途汽车（运动型多用途车）</x:v>
       </x:c>
       <x:c r="Q158" s="32" t="n">
         <x:v>16</x:v>
@@ -16485,7 +16621,7 @@
       </x:c>
       <x:c r="O159" s="30" t="str"/>
       <x:c r="P159" s="30" t="str">
-        <x:v>New and used automobiles and light trucks, such as sport utility vehicles, and passenger and cargo vans; Motor vehicle supplies, tires and new and used parts, as well as its accessories, tools and equipment; Provision of repair and maintenance services</x:v>
+        <x:v>新车和二手汽车和轻型卡车，例如运动型多用途车、客货车和货车；机动车辆用品、轮胎、新旧零件及其配件、工具和设备；提供维修和保养服务</x:v>
       </x:c>
       <x:c r="Q159" s="32" t="n">
         <x:v>15</x:v>
@@ -16596,7 +16732,7 @@
       </x:c>
       <x:c r="O160" s="30" t="str"/>
       <x:c r="P160" s="30" t="str">
-        <x:v>Medical supplies (Access Device: Dilatation; Access Device: Sheath; Antiretropulsion; Atherectomy Systems; Balloons: Dilation and Extraction; Band Ligator; Baskets; Bronchial Thermoplasty; Capital Equipment: Diagnostic; Capital Equipment: Mapping &amp; Navigation; Capital Equipment: Therapy; Catheters: Ablation; Catheters: Balloon; Catheters: Diagnostic; Catheters: Drainage; Catheters: Guide; Catheters: Mapping; Catheters: Ureteral; Clips; Cytology Brushes; Defibrillators; Direct Visualization Systems; Embolic Protection; Embolization; Forceps; Guidewires; Imaging Systems; Introducer Sheaths; Laser Fibers &amp; Accessories; Lasers &amp; Lithotripsy; Leads; Left Atrial Appendage Closure System; Needles; Pacemakers; Pelvic Floor Reconstruction; Plaque Modification; Probes; Remote Patient Monitoring; Renal Denervation; Retrieval Devices; Slings: Mid-Urethral; Snares; Sphincterotomes; Spinal Cord Stimulator Systems; Stents: Coronary; Stents: Gastrointestinal; Stents: Pulmonary; Stents: Ureteral; Stent</x:v>
+        <x:v>医疗用品（接入装置：扩张；接入装置：护套；抗后推；斑块切除系统；球囊：扩张和提取；束带结扎器；篮子；支气管热成形术；资本设备：诊断；资本设备：测绘和导航；资本设备：治疗；导管：消融；导管：球囊；导管：诊断；导管：引流；导管：引导；导管：测绘；：；&amp;；&amp;；去神经术；吊带；括约肌刺激器系统；支架：肺支架</x:v>
       </x:c>
       <x:c r="Q160" s="32" t="n">
         <x:v>15</x:v>
@@ -16707,7 +16843,7 @@
       </x:c>
       <x:c r="O161" s="30" t="str"/>
       <x:c r="P161" s="30" t="str">
-        <x:v>Agricultural and farm machinery and equipment, and other turf and grounds care equipment, including planting, harvesting, and grass mowing equipment</x:v>
+        <x:v>农业机械和设备，以及其他草坪和场地护理设备，包括种植、收割和割草设备</x:v>
       </x:c>
       <x:c r="Q161" s="32" t="n">
         <x:v>15</x:v>
@@ -16819,7 +16955,9 @@
         <x:v>PLOT NO. 71/2/B , PIMPRI INDUSTRIAL AREA , MIDC BHOSARI</x:v>
       </x:c>
       <x:c r="O162" s="30" t="str"/>
-      <x:c r="P162" s="30" t="str"/>
+      <x:c r="P162" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q162" s="32" t="n">
         <x:v>14</x:v>
       </x:c>
@@ -16921,7 +17059,7 @@
       </x:c>
       <x:c r="O163" s="30" t="str"/>
       <x:c r="P163" s="30" t="str">
-        <x:v>Cotton knitwear (bodysuits; sleepsuits; caps, mittens and booties; blankets; bibs; hooded towels, washcloths; fitted sheets for bassinets / cradles / cribs / cots; t-shirts; thermal nightwear; and long johns (pyjama sets))</x:v>
+        <x:v>棉针织品（连体衣；睡衣；帽子、手套和靴子；毛毯；围兜；连帽毛巾、面巾；摇篮/摇篮/婴儿床/婴儿床床笠；恤；保暖睡衣；以及秋裤（睡衣套装））</x:v>
       </x:c>
       <x:c r="Q163" s="32" t="n">
         <x:v>13</x:v>
@@ -17018,7 +17156,7 @@
       </x:c>
       <x:c r="O164" s="30" t="str"/>
       <x:c r="P164" s="30" t="str">
-        <x:v>Precision instruments and services for many applications in research and development, quality control, production, logistics and retail to customers around the world</x:v>
+        <x:v>为全球客户提供研发、质量控制、生产、物流和零售等多种应用的精密仪器和服务</x:v>
       </x:c>
       <x:c r="Q164" s="32" t="n">
         <x:v>13</x:v>
@@ -17112,7 +17250,9 @@
         <x:v>SM 64 MZA 83 LOTE 7 Y 8 CHICHEN ITZA</x:v>
       </x:c>
       <x:c r="O165" s="30" t="str"/>
-      <x:c r="P165" s="30" t="str"/>
+      <x:c r="P165" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q165" s="32" t="n">
         <x:v>13</x:v>
       </x:c>
@@ -17218,7 +17358,7 @@
       </x:c>
       <x:c r="O166" s="30" t="str"/>
       <x:c r="P166" s="30" t="str">
-        <x:v>ferrite,cable,knives,springs,trunki suitcase,hand shank,rivets,electromagnet,decorative band,mesh fabric,punching machine,sealing strip,seat,base metal,ynthetic filament spinning jets,transmission shafts,assembling machine,chamois leather,power line,eyes</x:v>
+        <x:v>铁氧体、电缆、刀具、弹簧、行李箱、手柄、铆钉、电磁铁、装饰带、网布、冲孔机、密封条、座椅、贱金属、化纤喷丝头、传动轴、装配机、麂皮、电源线、眼睛</x:v>
       </x:c>
       <x:c r="Q166" s="32" t="n">
         <x:v>12</x:v>
@@ -17314,7 +17454,9 @@
         <x:v>CERRO EL PLOMO 5420 1304 , LAS CONDES</x:v>
       </x:c>
       <x:c r="O167" s="30" t="str"/>
-      <x:c r="P167" s="30" t="str"/>
+      <x:c r="P167" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q167" s="32" t="n">
         <x:v>12</x:v>
       </x:c>
@@ -17424,7 +17566,7 @@
       </x:c>
       <x:c r="O168" s="30" t="str"/>
       <x:c r="P168" s="30" t="str">
-        <x:v>Fragrances and cosmetics and treatment products</x:v>
+        <x:v>香水、化妆品和护理产品</x:v>
       </x:c>
       <x:c r="Q168" s="32" t="n">
         <x:v>12</x:v>
@@ -17535,7 +17677,7 @@
       </x:c>
       <x:c r="O169" s="30" t="str"/>
       <x:c r="P169" s="30" t="str">
-        <x:v>Hardware and other related products</x:v>
+        <x:v>硬件及其他相关产品</x:v>
       </x:c>
       <x:c r="Q169" s="32" t="n">
         <x:v>12</x:v>
@@ -17645,7 +17787,9 @@
         <x:v>D-3/3, OKHLA INDUSTRIAL AREA , PHASE-II , NEW  SOUTH</x:v>
       </x:c>
       <x:c r="O170" s="30" t="str"/>
-      <x:c r="P170" s="30" t="str"/>
+      <x:c r="P170" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q170" s="32" t="n">
         <x:v>12</x:v>
       </x:c>
@@ -17744,7 +17888,9 @@
         <x:v>NO. 45 , SHANTHI NIKETHAN COLONY, MAHENDRA HILLS , EAST MARREDPALLY</x:v>
       </x:c>
       <x:c r="O171" s="30" t="str"/>
-      <x:c r="P171" s="30" t="str"/>
+      <x:c r="P171" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q171" s="32" t="n">
         <x:v>12</x:v>
       </x:c>
@@ -17852,7 +17998,7 @@
       </x:c>
       <x:c r="O172" s="30" t="str"/>
       <x:c r="P172" s="30" t="str">
-        <x:v>Motor vehicles</x:v>
+        <x:v>机动车辆</x:v>
       </x:c>
       <x:c r="Q172" s="32" t="n">
         <x:v>11</x:v>
@@ -17962,7 +18108,9 @@
         <x:v>CALLE BOSQUES DE BOLOGNIA 121</x:v>
       </x:c>
       <x:c r="O173" s="30" t="str"/>
-      <x:c r="P173" s="30" t="str"/>
+      <x:c r="P173" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q173" s="32" t="n">
         <x:v>11</x:v>
       </x:c>
@@ -18070,7 +18218,7 @@
       </x:c>
       <x:c r="O174" s="30" t="str"/>
       <x:c r="P174" s="30" t="str">
-        <x:v>orange,lows,coating head,perma,teli,foil,harness,h pin,tape slitting,50 micron,slot die,type m,g25,color blue,black print,pen,plain core,e11,machine,self adhesive transfer</x:v>
+        <x:v>橙色，低速，涂布头，铝箔，线束，针，胶带分切，50微米，槽模，型，25，蓝色，黑色打印，笔，平芯，11，机器，自粘转印</x:v>
       </x:c>
       <x:c r="Q174" s="32" t="n">
         <x:v>10</x:v>
@@ -18170,7 +18318,9 @@
         <x:v>bhopal, madhya pradesh, india</x:v>
       </x:c>
       <x:c r="O175" s="30" t="str"/>
-      <x:c r="P175" s="30" t="str"/>
+      <x:c r="P175" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q175" s="32" t="n">
         <x:v>10</x:v>
       </x:c>
@@ -18281,7 +18431,9 @@
         <x:v>PLOT NO 209/1436 ESBC WILSON BUSINESS PARK , BLOCK BRAVO 12ND FLOOR OFF LANGATA ROAD</x:v>
       </x:c>
       <x:c r="O176" s="30" t="str"/>
-      <x:c r="P176" s="30" t="str"/>
+      <x:c r="P176" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q176" s="32" t="n">
         <x:v>10</x:v>
       </x:c>
@@ -18391,7 +18543,7 @@
       </x:c>
       <x:c r="O177" s="30" t="str"/>
       <x:c r="P177" s="30" t="str">
-        <x:v>Adhesives, abrasives, laminates, passive fire protection, dental and orthodontic products, electronic materials, medical products, car-care products (sun films, polish, wax, car shampoo, treatment for the exterior, interior and the under chassis rust protection), electronic circuits, and optical films</x:v>
+        <x:v>粘合剂、磨料、层压板、被动防火、牙科和正畸产品、电子材料、医疗产品、汽车护理产品（太阳膜、上光剂、蜡、洗车液、外部、内部和底盘防锈处理）、电子电路和光学薄膜</x:v>
       </x:c>
       <x:c r="Q177" s="32" t="n">
         <x:v>9</x:v>
@@ -18501,7 +18653,9 @@
         <x:v>69 B 27, CALLE 17 A</x:v>
       </x:c>
       <x:c r="O178" s="30" t="str"/>
-      <x:c r="P178" s="30" t="str"/>
+      <x:c r="P178" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q178" s="32" t="n">
         <x:v>8</x:v>
       </x:c>
@@ -18610,7 +18764,9 @@
         <x:v>CALLE NUEVA CARRETERA PROGRESO-CHELEM 5155</x:v>
       </x:c>
       <x:c r="O179" s="30" t="str"/>
-      <x:c r="P179" s="30" t="str"/>
+      <x:c r="P179" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q179" s="32" t="n">
         <x:v>8</x:v>
       </x:c>
@@ -18720,7 +18876,7 @@
       </x:c>
       <x:c r="O180" s="30" t="str"/>
       <x:c r="P180" s="30" t="str">
-        <x:v>Membership warehouse club (Consumer electronics; Computers; Baby products; Automotive supplies; Sporting goods; Outdoor equipment; Hardware products; Toys and games; Household appliances; Housewares; Bed and bath products; Luggage; Healthcare products; Furniture; Office supplies; Fashion accessories; Restaurant/institutional products)</x:v>
+        <x:v>会员仓俱乐部（消费电子；电脑；婴儿用品；汽车用品；体育用品；户外装备；五金制品；玩具游戏；家用电器；家庭用品；床浴用品；箱包；保健品；家具；办公用品；时尚配饰；餐厅/机构产品）</x:v>
       </x:c>
       <x:c r="Q180" s="32" t="n">
         <x:v>8</x:v>
@@ -18828,7 +18984,9 @@
         <x:v>4695, LANE RAZIA BEGUM HAUS QAZI</x:v>
       </x:c>
       <x:c r="O181" s="30" t="str"/>
-      <x:c r="P181" s="30" t="str"/>
+      <x:c r="P181" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q181" s="32" t="n">
         <x:v>8</x:v>
       </x:c>
@@ -18934,7 +19092,7 @@
       <x:c r="N182" s="30" t="str"/>
       <x:c r="O182" s="30" t="str"/>
       <x:c r="P182" s="30" t="str">
-        <x:v>vehicle,wheel,8k,cma cgm,a tool,cutting tools,pa pallet,auto spare,polish pad,cod,brush,ring,freight prepaid,fans,disco,custom,mobil,brushes,discs,k machine</x:v>
+        <x:v>车辆，车轮，8，工具，切削工具，托盘，汽车备件，抛光垫，鳕鱼，刷子，环，运费预付，风扇，迪斯科，定制，美孚，刷子，光盘，机</x:v>
       </x:c>
       <x:c r="Q182" s="32" t="n">
         <x:v>7</x:v>
@@ -19039,7 +19197,7 @@
       </x:c>
       <x:c r="O183" s="30" t="str"/>
       <x:c r="P183" s="30" t="str">
-        <x:v>felt tipped,polyurethane,bags,hardened plastic,polyester,aluminium alloy,insulation board,medium density fiberboard,sacks,aluminium bar,laminated wood salon table,plastic plate,wood furniture,porous-tipped pens,trade advertising material,stainless steel,fibreboard,board fireproofing</x:v>
+        <x:v>毛毡、聚氨酯、箱包、硬质塑料、聚酯、铝合金、保温板、中密度纤维板、麻袋、铝棒、层压木沙龙桌、塑料板、木制家具、多孔笔、商业广告材料、不锈钢、纤维板、防火板</x:v>
       </x:c>
       <x:c r="Q183" s="32" t="n">
         <x:v>7</x:v>
@@ -19144,7 +19302,7 @@
       </x:c>
       <x:c r="O184" s="30" t="str"/>
       <x:c r="P184" s="30" t="str">
-        <x:v>Abrasives, ceramics, and plastic products</x:v>
+        <x:v>磨料、陶瓷、塑料制品</x:v>
       </x:c>
       <x:c r="Q184" s="32" t="n">
         <x:v>7</x:v>
@@ -19255,7 +19413,7 @@
       </x:c>
       <x:c r="O185" s="30" t="str"/>
       <x:c r="P185" s="30" t="str">
-        <x:v>inserted nut,nuts,arm,drill bit,dressing stick,x7,rain,hand tool,expansion foam,aed,reis,80 mesh,dag,bright raw white,s type,elma,brewery hose,smooth cover,polyethylene wax emulsion,type f</x:v>
+        <x:v>插入螺母，螺母，臂，钻头，敷料棒，7，雨，手动工具，膨胀泡沫，80目，亮原白色，型，啤酒厂软管，光滑盖，聚乙烯蜡乳液，型</x:v>
       </x:c>
       <x:c r="Q185" s="32" t="n">
         <x:v>7</x:v>
@@ -19364,7 +19522,7 @@
       </x:c>
       <x:c r="O186" s="30" t="str"/>
       <x:c r="P186" s="30" t="str">
-        <x:v>Motor vehicles and motor vehicle parts and supplies (brand new cars, pre-owned vehicles, car mats, headlights, gear knobs, leather gaiters, handbrake handles, stainless sill protectors, seat covers, car point roof boxes, side repeaters and indicators, car body kits, and car care products)</x:v>
+        <x:v>机动车辆和机动车辆零部件和用品（全新汽车、二手车、汽车脚垫、车头灯、档位旋钮、皮革护腿、手刹手柄、不锈钢门槛保护装置、座套、汽车点车顶盒、侧中继器和指示灯、车身套件和汽车护理产品）</x:v>
       </x:c>
       <x:c r="Q186" s="32" t="n">
         <x:v>7</x:v>
@@ -19474,7 +19632,9 @@
         <x:v>NO. 824/825/826/827, EIGHH FLOOR, TOWER A, EMMAR DIGITAL GREEN, SECTOR-61, GOLF EXTENSION</x:v>
       </x:c>
       <x:c r="O187" s="30" t="str"/>
-      <x:c r="P187" s="30" t="str"/>
+      <x:c r="P187" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q187" s="32" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -19584,7 +19744,7 @@
       </x:c>
       <x:c r="O188" s="30" t="str"/>
       <x:c r="P188" s="30" t="str">
-        <x:v>Motor vehicles and motor vehicle parts and supplies; Maintenance and repair of motor vehicles</x:v>
+        <x:v>机动车辆及机动车辆零部件和用品；机动车辆的保养和维修</x:v>
       </x:c>
       <x:c r="Q188" s="32" t="n">
         <x:v>7</x:v>
@@ -19693,7 +19853,7 @@
       </x:c>
       <x:c r="O189" s="30" t="str"/>
       <x:c r="P189" s="30" t="str">
-        <x:v>Sheets and strips with paper and cloth backing for all hand sanding and portable machine sanding applications</x:v>
+        <x:v>带有纸和布背衬的片材和条带，适用于所有手动打磨和便携式机器打磨应用</x:v>
       </x:c>
       <x:c r="Q189" s="32" t="n">
         <x:v>7</x:v>
@@ -19787,7 +19947,9 @@
         <x:v>delhi, delhi, india</x:v>
       </x:c>
       <x:c r="O190" s="30" t="str"/>
-      <x:c r="P190" s="30" t="str"/>
+      <x:c r="P190" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q190" s="32" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -19903,7 +20065,7 @@
       </x:c>
       <x:c r="O191" s="30" t="str"/>
       <x:c r="P191" s="30" t="str">
-        <x:v>barcode scanner</x:v>
+        <x:v>条码扫描仪</x:v>
       </x:c>
       <x:c r="Q191" s="32" t="n">
         <x:v>6</x:v>
@@ -20010,7 +20172,7 @@
       </x:c>
       <x:c r="O192" s="30" t="str"/>
       <x:c r="P192" s="30" t="str">
-        <x:v>Bending machines, shears, manual machines, folder, sheet processing machines, folding machines, cutting, graphical, shearer, control, hydraulic shears, schroeder, folder, and other special machineries</x:v>
+        <x:v>折弯机、剪板机、手动机、折页机、板材加工机、折页机、切割机、图形剪板机、控制机、液压剪板机、施罗德、折页机、等特种机械</x:v>
       </x:c>
       <x:c r="Q192" s="32" t="n">
         <x:v>6</x:v>
@@ -20111,7 +20273,7 @@
       </x:c>
       <x:c r="O193" s="30" t="str"/>
       <x:c r="P193" s="30" t="str">
-        <x:v>food grade,r 12,slide,polyisobutylene,polyolefin,offset,atta,bio,propylene copolymer,type load cell,dos,bat,hopper,synthetic rubber,g lock,conveyor,cover,manua,elite,polyethylen</x:v>
+        <x:v>食品级，12，幻灯片，聚异丁烯，聚烯烃，胶印，生物，丙烯共聚物，称重传感器，蝙蝠，料斗，合成橡胶，输送机，盖子，精英，聚乙烯</x:v>
       </x:c>
       <x:c r="Q193" s="32" t="n">
         <x:v>6</x:v>
@@ -20207,7 +20369,9 @@
         <x:v>GABRIEL RAMOS MILLAN 383 VILLASENOR</x:v>
       </x:c>
       <x:c r="O194" s="30" t="str"/>
-      <x:c r="P194" s="30" t="str"/>
+      <x:c r="P194" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q194" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -20316,7 +20480,9 @@
         <x:v>PLOT NUMBER 209/5443 ,  ADDIS ABABA ROAD ,  INDUSTRIAL AREA</x:v>
       </x:c>
       <x:c r="O195" s="30" t="str"/>
-      <x:c r="P195" s="30" t="str"/>
+      <x:c r="P195" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q195" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -20426,7 +20592,7 @@
       </x:c>
       <x:c r="O196" s="30" t="str"/>
       <x:c r="P196" s="30" t="str">
-        <x:v>Automotive and industrial paints</x:v>
+        <x:v>汽车和工业涂料</x:v>
       </x:c>
       <x:c r="Q196" s="32" t="n">
         <x:v>5</x:v>
@@ -20526,7 +20692,9 @@
         <x:v>NO. 80-B , YESHWANTHPUR INDUSTRIAL SUBURBS</x:v>
       </x:c>
       <x:c r="O197" s="30" t="str"/>
-      <x:c r="P197" s="30" t="str"/>
+      <x:c r="P197" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q197" s="32" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -20634,7 +20802,7 @@
       </x:c>
       <x:c r="O198" s="30" t="str"/>
       <x:c r="P198" s="30" t="str">
-        <x:v>Decorative, floor, wall, swimming pool, and floor/wall tiles; sanitary wares, such as toilet products, lavatories, and faucets; and other products for building projects</x:v>
+        <x:v>装饰、地板、墙壁、游泳池、地砖/墙砖；卫生洁具，例如盥洗用品、盥洗盆和水龙头；和其他建筑项目产品</x:v>
       </x:c>
       <x:c r="Q198" s="32" t="n">
         <x:v>5</x:v>
@@ -20734,7 +20902,9 @@
         <x:v>SALVADOR QUEZADA LIMON NO. 1512 , CURTIDORES</x:v>
       </x:c>
       <x:c r="O199" s="30" t="str"/>
-      <x:c r="P199" s="30" t="str"/>
+      <x:c r="P199" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q199" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -20842,7 +21012,7 @@
       </x:c>
       <x:c r="O200" s="30" t="str"/>
       <x:c r="P200" s="30" t="str">
-        <x:v>connector,malleable cast iron,bluetooth headset,cable,builders' ware of plastics,polymers of ethylene,voltage stabilized suppliers,electronic scale,plug cord,printer,account balances,cast steel products,interphone,equilibristat,regulated power supply,plates,wires</x:v>
+        <x:v>连接器、可锻铸铁、蓝牙耳机、电缆、塑料建筑用品、乙烯聚合物、稳压供应商、电子秤、插头线、打印机、账户余额、铸钢产品、对讲机、平衡器、稳压电源、板材、电线</x:v>
       </x:c>
       <x:c r="Q200" s="32" t="n">
         <x:v>4</x:v>
@@ -20947,7 +21117,7 @@
       </x:c>
       <x:c r="O201" s="30" t="str"/>
       <x:c r="P201" s="30" t="str">
-        <x:v>Hardware, plumbing and heating equipment and supplies (steam and hot water boilers, bathtubs, sinks, lavatories, shower stalls, and whirlpool baths, fittings, flanges, pipes and other related products)</x:v>
+        <x:v>五金、管道和供暖设备及用品（蒸汽和热水锅炉、浴缸、水槽、盥洗室、淋浴间和漩涡浴缸、配件、法兰、管道和其他相关产品）</x:v>
       </x:c>
       <x:c r="Q201" s="32" t="n">
         <x:v>4</x:v>
@@ -21059,7 +21229,9 @@
         <x:v>NO. A-4 , NARAINA INDUSTRIAL AREA, PHASE-I</x:v>
       </x:c>
       <x:c r="O202" s="30" t="str"/>
-      <x:c r="P202" s="30" t="str"/>
+      <x:c r="P202" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q202" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -21159,7 +21331,7 @@
       </x:c>
       <x:c r="O203" s="30" t="str"/>
       <x:c r="P203" s="30" t="str">
-        <x:v>Yarn and fabrics</x:v>
+        <x:v>纱线和面料</x:v>
       </x:c>
       <x:c r="Q203" s="32" t="n">
         <x:v>4</x:v>
@@ -21269,7 +21441,9 @@
         <x:v>36 A 71, CARRERA 4 B</x:v>
       </x:c>
       <x:c r="O204" s="30" t="str"/>
-      <x:c r="P204" s="30" t="str"/>
+      <x:c r="P204" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q204" s="32" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -21378,7 +21552,9 @@
         <x:v>PLOT NO.LR NO 24393</x:v>
       </x:c>
       <x:c r="O205" s="30" t="str"/>
-      <x:c r="P205" s="30" t="str"/>
+      <x:c r="P205" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q205" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -21486,7 +21662,7 @@
       </x:c>
       <x:c r="O206" s="30" t="str"/>
       <x:c r="P206" s="30" t="str">
-        <x:v>Belts and belting products</x:v>
+        <x:v>皮带及皮带产品</x:v>
       </x:c>
       <x:c r="Q206" s="32" t="n">
         <x:v>3</x:v>
@@ -21597,7 +21773,7 @@
       </x:c>
       <x:c r="O207" s="30" t="str"/>
       <x:c r="P207" s="30" t="str">
-        <x:v>bars,pipes,cotters,plastic caps,stainless steel tube,cold rolled stainless steel sheet,alloy steel seamless circular section tube,scavenge trunk,tubes,butterfly auto valve,check valve,glass fibres,plated steel,washers,knives,inox,stainless steel rods,stainless steel ornament pipe,alloy steel,spring</x:v>
+        <x:v>棒材、管材、开口销、塑料帽、不锈钢管、冷轧不锈钢板、合金钢无缝圆截面管、扫气箱、管材、蝶式自动阀、止回阀、玻璃纤维、镀钢、垫圈、刀具、不锈钢、不锈钢棒、不锈钢装饰管、合金钢、弹簧</x:v>
       </x:c>
       <x:c r="Q207" s="32" t="n">
         <x:v>3</x:v>
@@ -21701,7 +21877,9 @@
         <x:v>EL-91, TTC Industrial Area,</x:v>
       </x:c>
       <x:c r="O208" s="30" t="str"/>
-      <x:c r="P208" s="30" t="str"/>
+      <x:c r="P208" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q208" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -21811,7 +21989,7 @@
       </x:c>
       <x:c r="O209" s="30" t="str"/>
       <x:c r="P209" s="30" t="str">
-        <x:v>tools,violet red bill agar,domestic,label tape,vitrified,antiparasitic,personal hot cup,floor,culture medium,glucose,buje rueda,glass cleaning,machine,crayones,needle for suturing,copier,manganese dioxide,lubricant,catcher,blue respirator</x:v>
+        <x:v>工具，紫红嘴琼脂，国产，标签胶带，玻璃化，抗寄生虫，个人热杯，地板，培养基，葡萄糖，玻璃清洁，机器，蜡笔，缝合针，复印机，二氧化锰，润滑剂，捕手，蓝色呼吸器</x:v>
       </x:c>
       <x:c r="Q209" s="32" t="n">
         <x:v>3</x:v>
@@ -21910,7 +22088,7 @@
       </x:c>
       <x:c r="O210" s="30" t="str"/>
       <x:c r="P210" s="30" t="str">
-        <x:v>blu,pvc,silicone nipple,frame,moulding machine,t 80,iron and steel,machine,two burner,brown oxide,feeder,grill,titi,used injection molding machine,bowl,unit,spiral screen,model,e pi,made of glass</x:v>
+        <x:v>蓝光，聚氯乙烯，硅胶奶嘴，框架，成型机，80，钢铁，机，两个燃烧器，棕色氧化物，进料器，烤架，蒂蒂，二手注塑机，碗，单位，螺旋筛，模型，玻璃制成</x:v>
       </x:c>
       <x:c r="Q210" s="32" t="n">
         <x:v>2</x:v>
@@ -22010,7 +22188,9 @@
         <x:v>F-402, 4TH FLOOR PLOT NO. D-1 , DISTRICT CENTRE "RAS VILAS" , SAKET</x:v>
       </x:c>
       <x:c r="O211" s="30" t="str"/>
-      <x:c r="P211" s="30" t="str"/>
+      <x:c r="P211" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q211" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -22120,7 +22300,7 @@
       </x:c>
       <x:c r="O212" s="30" t="str"/>
       <x:c r="P212" s="30" t="str">
-        <x:v>Chemicals and allied products</x:v>
+        <x:v>化学品及相关产品</x:v>
       </x:c>
       <x:c r="Q212" s="32" t="n">
         <x:v>2</x:v>
@@ -22221,7 +22401,7 @@
       </x:c>
       <x:c r="O213" s="30" t="str"/>
       <x:c r="P213" s="30" t="str">
-        <x:v>Tires and tubes</x:v>
+        <x:v>轮胎和内胎</x:v>
       </x:c>
       <x:c r="Q213" s="32" t="n">
         <x:v>2</x:v>
@@ -22331,7 +22511,9 @@
         <x:v>NO. SF-11, SECOND FLOOR, VASANT SQUARE MALL, COMMUNITY CENTRE, VAST KUNJ</x:v>
       </x:c>
       <x:c r="O214" s="30" t="str"/>
-      <x:c r="P214" s="30" t="str"/>
+      <x:c r="P214" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q214" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -22441,7 +22623,7 @@
       </x:c>
       <x:c r="O215" s="30" t="str"/>
       <x:c r="P215" s="30" t="str">
-        <x:v>The authorized distributor and service provider for GE’s gas engines in India, supplying both the Jenbacher and Waukesha product ranges for power generation and gas compression respectively</x:v>
+        <x:v>燃气发动机在印度的授权经销商和服务提供商，分别供应用于发电和气体压缩的和产品系列</x:v>
       </x:c>
       <x:c r="Q215" s="32" t="n">
         <x:v>2</x:v>
@@ -22550,7 +22732,7 @@
       </x:c>
       <x:c r="O216" s="30" t="str"/>
       <x:c r="P216" s="30" t="str">
-        <x:v>bag dryer,430 s,gh,fork,spiral shaped,coating,abs plastic,ape,ring,table,brush,lily flower,remover,hot,h4,oven mitt,spatula,rolli,marble roll,adeo</x:v>
+        <x:v>袋式烘干机，430，叉子，螺旋形，涂层，工程塑料塑料，猿，环，桌子，刷子，百合花，去除剂，热，4，烤箱手套，抹刀，大理石卷</x:v>
       </x:c>
       <x:c r="Q216" s="32" t="n">
         <x:v>2</x:v>
@@ -22643,7 +22825,7 @@
       </x:c>
       <x:c r="O217" s="30" t="str"/>
       <x:c r="P217" s="30" t="str">
-        <x:v>cotters,boards,stainless steel tube,feed additive,grill,bolt,lubricant,tubes,articles of copper,glass fibres,washers,non-alloy steel coil,section steel,carbon steel pipe,ordinary steel h-beam,inox,rotary knob,stainless steel rods,spring,nettng</x:v>
+        <x:v>开口销、板材、不锈钢管、饲料添加剂、格栅、螺栓、润滑油、管材、铜制品、玻璃纤维、垫圈、非合金钢卷、型钢、碳钢管、普通钢型钢、不锈钢、旋钮、不锈钢棒、弹簧、网</x:v>
       </x:c>
       <x:c r="Q217" s="32" t="n">
         <x:v>2</x:v>
@@ -22748,7 +22930,7 @@
       </x:c>
       <x:c r="O218" s="30" t="str"/>
       <x:c r="P218" s="30" t="str">
-        <x:v>coil,boards,checking instruments,grill,rivet,glass fibres,carbon  brushes,washers,heat sensor,section steel,electricity meters,knives,ordinary steel h-beam,inox,metal wire,clamps,springs,processors,alloy steel,thermometer</x:v>
+        <x:v>线圈、板材、检测仪器、烤架、铆钉、玻璃纤维、碳刷、垫圈、热传感器、型钢、电度表、刀具、普通钢型钢、不锈钢、金属丝、夹具、弹簧、处理器、合金钢、温度计</x:v>
       </x:c>
       <x:c r="Q218" s="32" t="n">
         <x:v>2</x:v>
@@ -22861,7 +23043,7 @@
       </x:c>
       <x:c r="O219" s="30" t="str"/>
       <x:c r="P219" s="30" t="str">
-        <x:v>roof tile,expander plug,steel sleeve,steel ball,xtr,sleeve,arg,mm st,clay roofing tile,expansion plug,10mm</x:v>
+        <x:v>屋顶瓦，膨胀塞，钢套，钢球，套筒，粘土屋顶瓦，膨胀塞，10</x:v>
       </x:c>
       <x:c r="Q219" s="32" t="n">
         <x:v>2</x:v>
@@ -22962,7 +23144,7 @@
       </x:c>
       <x:c r="O220" s="30" t="str"/>
       <x:c r="P220" s="30" t="str">
-        <x:v>Cut and sew apparel</x:v>
+        <x:v>裁剪和缝制服装</x:v>
       </x:c>
       <x:c r="Q220" s="32" t="n">
         <x:v>2</x:v>
@@ -23060,7 +23242,9 @@
         <x:v>DIAGONAL REFORMA NO. 2583 ORIENTE, MOCTEZUMA</x:v>
       </x:c>
       <x:c r="O221" s="30" t="str"/>
-      <x:c r="P221" s="30" t="str"/>
+      <x:c r="P221" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q221" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -23170,7 +23354,7 @@
       </x:c>
       <x:c r="O222" s="30" t="str"/>
       <x:c r="P222" s="30" t="str">
-        <x:v>bobbin,superbolt,anilox roll,ev,lubricating grease,ares,cable connecting,frequency converter,belt,propylene copolymer,manometer,talen,g5,ldpe granule,moulding machine,machine,pneumatic cylinder,v belt,paper bag machine,card</x:v>
+        <x:v>线轴，超级螺栓，网纹辊，润滑油脂，战神，电缆连接，变频器，皮带，丙烯共聚物，压力计，塔伦，5，低密度聚乙烯颗粒，成型机，机，气缸，带，纸袋机，卡</x:v>
       </x:c>
       <x:c r="Q222" s="32" t="n">
         <x:v>2</x:v>
@@ -23269,7 +23453,7 @@
       </x:c>
       <x:c r="O223" s="30" t="str"/>
       <x:c r="P223" s="30" t="str">
-        <x:v>rolls,blu,reels,graphtol,t yellow,pigment,bare pump,pv f,g 15,esbo,bb,tano,sheet,hood,80 gsm,roll,stabilizer,man made fabric,blowing agent,pvc stabilizer</x:v>
+        <x:v>卷，蓝色，卷轴，黄色，颜料，裸泵，15，片材，罩，80，卷，稳定剂，人造织物，发泡剂，聚氯乙烯稳定剂</x:v>
       </x:c>
       <x:c r="Q223" s="32" t="n">
         <x:v>2</x:v>
@@ -23374,7 +23558,7 @@
       </x:c>
       <x:c r="O224" s="30" t="str"/>
       <x:c r="P224" s="30" t="str">
-        <x:v>Automated teller machines and other cash processing equipment (various types of ATMs including stand-alone, desktop, drive-up, and through-the-wall models)</x:v>
+        <x:v>自动柜员机和其他现金处理设备（各种类型的自动柜员机，包括独立式、台式、驾车式和穿墙式自动柜员机）</x:v>
       </x:c>
       <x:c r="Q224" s="32" t="n">
         <x:v>2</x:v>
@@ -23475,7 +23659,7 @@
       </x:c>
       <x:c r="O225" s="30" t="str"/>
       <x:c r="P225" s="30" t="str">
-        <x:v>perlita expandida,insta,puerto rico,black b,cone,ail,sacks and bags,party,methyl hydroxyethyl cellulose,t 90,e 44,pla,acrylic polymer,pvc corner bead,white po,polyisocyanate,ale,reef,paper kraft bag,gat</x:v>
+        <x:v>波多黎各，黑色，锥体，麻袋和袋子，派对，甲基羟乙基纤维素，90，44，丙烯酸聚合物，聚氯乙烯角珠，白色，多异氰酸酯，啤酒，礁石，牛皮纸袋</x:v>
       </x:c>
       <x:c r="Q225" s="32" t="n">
         <x:v>2</x:v>
@@ -23575,7 +23759,9 @@
         <x:v>NO. R-22, FIRST FLOOR, RITA BLOCK , SHAKAR PUR</x:v>
       </x:c>
       <x:c r="O226" s="30" t="str"/>
-      <x:c r="P226" s="30" t="str"/>
+      <x:c r="P226" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q226" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -23686,7 +23872,9 @@
         <x:v>ACAHAY C/ RUTA TRANSCHACO</x:v>
       </x:c>
       <x:c r="O227" s="30" t="str"/>
-      <x:c r="P227" s="30" t="str"/>
+      <x:c r="P227" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q227" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -23795,7 +23983,9 @@
         <x:v>SERVIS HOUSE , 2- MAIN GULBERG , 54662</x:v>
       </x:c>
       <x:c r="O228" s="30" t="str"/>
-      <x:c r="P228" s="30" t="str"/>
+      <x:c r="P228" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q228" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -23903,7 +24093,7 @@
       </x:c>
       <x:c r="O229" s="30" t="str"/>
       <x:c r="P229" s="30" t="str">
-        <x:v>Home furnishings, furniture and household products</x:v>
+        <x:v>家居摆设、家具及家居用品</x:v>
       </x:c>
       <x:c r="Q229" s="32" t="n">
         <x:v>2</x:v>
@@ -24011,7 +24201,9 @@
         <x:v>nairobi, nairobi area, kenya p/o box 47540</x:v>
       </x:c>
       <x:c r="O230" s="30" t="str"/>
-      <x:c r="P230" s="30" t="str"/>
+      <x:c r="P230" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q230" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -24113,7 +24305,7 @@
       </x:c>
       <x:c r="O231" s="30" t="str"/>
       <x:c r="P231" s="30" t="str">
-        <x:v>Offers speakers, car stereo mechanisms, factory automation systems, optical disc manufacturing systems, organic light-emitting diode displays, microphones, headphones, precision pressed parts, precision resin-molded parts, and precision molds/dies; Provides studio monitor speakers and home speakers, as well as ultralight mini-speakers that are used in cell phones and notebook computers; audio visual accessories; and mechanisms for car audio systems, such as CD, DVD, MD, and cassette players</x:v>
+        <x:v>提供扬声器、汽车音响机构、工厂自动化系统、光盘制造系统、有机发光二极管显示器、麦克风、耳机、精密冲压件、精密树脂成型件、精密模具；提供录音室监听音箱和家用音箱，以及用于手机和笔记本电脑的超轻迷你音箱；视听配件；以及汽车音响系统的机构，例如、、和盒式磁带播放器</x:v>
       </x:c>
       <x:c r="Q231" s="32" t="n">
         <x:v>2</x:v>
@@ -24223,7 +24415,9 @@
         <x:v>TUUSHIN BLDG , AMAR STREET , 8TH KHOROO , SUKHBAATAR DISTRICT</x:v>
       </x:c>
       <x:c r="O232" s="30" t="str"/>
-      <x:c r="P232" s="30" t="str"/>
+      <x:c r="P232" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q232" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -24323,7 +24517,7 @@
       </x:c>
       <x:c r="O233" s="30" t="str"/>
       <x:c r="P233" s="30" t="str">
-        <x:v>Millwork, veneer, plywood and structural wood, and other related products</x:v>
+        <x:v>木制品、单板、胶合板和结构木材以及其他相关产品</x:v>
       </x:c>
       <x:c r="Q233" s="32" t="n">
         <x:v>1</x:v>
@@ -24431,7 +24625,9 @@
         <x:v>calle 1era, el carmen, atras de la caja de ahorros de via espa�a entrando por la calle de eterna plaque, chalet #137.</x:v>
       </x:c>
       <x:c r="O234" s="30" t="str"/>
-      <x:c r="P234" s="30" t="str"/>
+      <x:c r="P234" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q234" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -24534,7 +24730,9 @@
         <x:v>21/3, SECTOR NO. 22, KORANGI INDUSTRIAL AREA, KARACHI</x:v>
       </x:c>
       <x:c r="O235" s="30" t="str"/>
-      <x:c r="P235" s="30" t="str"/>
+      <x:c r="P235" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q235" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -24644,7 +24842,7 @@
       </x:c>
       <x:c r="O236" s="30" t="str"/>
       <x:c r="P236" s="30" t="str">
-        <x:v>Complete solutions in all of its fields of horticulture and floriculture, telecommunications, water purification, solar energy, and generators</x:v>
+        <x:v>园艺花卉、电信、水净化、太阳能和发电机等所有领域的完整解决方案</x:v>
       </x:c>
       <x:c r="Q236" s="32" t="n">
         <x:v>1</x:v>
@@ -24755,7 +24953,7 @@
       </x:c>
       <x:c r="O237" s="30" t="str"/>
       <x:c r="P237" s="30" t="str">
-        <x:v>numerical control panels,coil,air filter,dryer,acrylic resin,gate,check valve,gloves of vulcanized rubber,machinery,amalgam lead,caps,stroboscopes,jet projecting machines,connectors,robot,floodlight,oil pump,life-jackets,plastic tubing,inox</x:v>
+        <x:v>数控面板、线圈、空气过滤器、干燥机、丙烯酸树脂、闸门、止回阀、硫化橡胶手套、机械、汞合金铅、帽子、频闪仪、喷射投影机、连接器、机器人、泛光灯、油泵、救生衣、塑料管、不锈钢</x:v>
       </x:c>
       <x:c r="Q237" s="32" t="n">
         <x:v>1</x:v>
@@ -24864,7 +25062,7 @@
       </x:c>
       <x:c r="O238" s="30" t="str"/>
       <x:c r="P238" s="30" t="str">
-        <x:v>steel parts,springs,stainless steel cable,railway vehicles,seat,electric multi-testing machines for testing metals,industrial steel material,stainless steel strip,plastic,steel pipe,screws,stainless steel square tube,paper,steel tube,u-steel,styrene butadiene rubber,regrind rubber,bolts,screw</x:v>
+        <x:v>钢件、弹簧、不锈钢拉索、轨道车辆、座椅、金属电动万能试验机、工业钢材、不锈钢带、塑料、钢管、螺钉、不锈钢方管、纸张、钢管、型钢、丁苯橡胶、再生橡胶、螺栓、螺钉</x:v>
       </x:c>
       <x:c r="Q238" s="32" t="n">
         <x:v>1</x:v>
@@ -24968,7 +25166,9 @@
         <x:v>Gut No 262, Lavale Road,</x:v>
       </x:c>
       <x:c r="O239" s="30" t="str"/>
-      <x:c r="P239" s="30" t="str"/>
+      <x:c r="P239" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q239" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -25077,7 +25277,9 @@
         <x:v>aguirre 611 y boyacá guayaquil guayas</x:v>
       </x:c>
       <x:c r="O240" s="30" t="str"/>
-      <x:c r="P240" s="30" t="str"/>
+      <x:c r="P240" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q240" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -25169,7 +25371,7 @@
       </x:c>
       <x:c r="O241" s="30" t="str"/>
       <x:c r="P241" s="30" t="str">
-        <x:v>ice,ev,lightweight panel,8k,metal frame,cod,board,granite slab,k ar,s p a,freight prepaid,custom,impro,ip p,w 10 28,chains,ether,melamine faced chipboard,ed panel,electrotherm</x:v>
+        <x:v>冰，轻质面板，8，金属框架，鳕鱼，板，花岗岩板，运费预付，定制，即兴，1028，链条，乙醚，三聚氰胺饰面刨花板，面板</x:v>
       </x:c>
       <x:c r="Q241" s="32" t="n">
         <x:v>1</x:v>
@@ -25273,7 +25475,9 @@
         <x:v>63/ 64 , 6TH FLOOR , MEHERZIN BLDG, 109/ A WOOD HOUSE ROAD, COLABA MUMBAI</x:v>
       </x:c>
       <x:c r="O242" s="30" t="str"/>
-      <x:c r="P242" s="30" t="str"/>
+      <x:c r="P242" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q242" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -25375,7 +25579,7 @@
       </x:c>
       <x:c r="O243" s="30" t="str"/>
       <x:c r="P243" s="30" t="str">
-        <x:v>pvc,kluber,analysis timer,dashboard,contactor,calar,dryer,crayones,cutting tool,aquaculture,gas scrubber,bandsaw,control panel contactor,double dinger wood,walnut laminated flooring,machinery,wooden flooring,strawberry,distribution band,particle board</x:v>
+        <x:v>聚氯乙烯、克鲁勃、分析定时器、仪表板、接触器、卡拉、干燥机、蜡笔、切削工具、水产养殖、气体洗涤器、带锯、控制面板接触器、双丁格木、胡桃木强化地板、机械、木地板、草莓、配电带、刨花板</x:v>
       </x:c>
       <x:c r="Q243" s="32" t="n">
         <x:v>1</x:v>
@@ -25479,7 +25683,9 @@
         <x:v>CAMINO DE LA COLINA 1447 , HUECHURABA</x:v>
       </x:c>
       <x:c r="O244" s="30" t="str"/>
-      <x:c r="P244" s="30" t="str"/>
+      <x:c r="P244" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q244" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -25588,7 +25794,9 @@
         <x:v>1/374 BHARATHI NAGAR FIRST STREET VENGAIVASAL</x:v>
       </x:c>
       <x:c r="O245" s="30" t="str"/>
-      <x:c r="P245" s="30" t="str"/>
+      <x:c r="P245" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q245" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -25686,7 +25894,7 @@
       </x:c>
       <x:c r="O246" s="30" t="str"/>
       <x:c r="P246" s="30" t="str">
-        <x:v>t 16,box,teja,loop cap,wall spike,f clamp,arm,tension bar,iec,outdoor,door,bolt,lv,steel rebars,tension band,gh,ceramic roofing tile,tiles,t cap,ce f1</x:v>
+        <x:v>16，盒子，环帽，墙钉，夹，臂，张力杆，户外，门，螺栓，钢筋，张力带，陶瓷屋面瓦，瓷砖，帽，1</x:v>
       </x:c>
       <x:c r="Q246" s="32" t="n">
         <x:v>1</x:v>
@@ -25791,7 +25999,7 @@
       </x:c>
       <x:c r="O247" s="30" t="str"/>
       <x:c r="P247" s="30" t="str">
-        <x:v>Pharmaceutical preparations</x:v>
+        <x:v>药物制剂</x:v>
       </x:c>
       <x:c r="Q247" s="32" t="n">
         <x:v>1</x:v>
@@ -25901,7 +26109,9 @@
         <x:v>PLOT NO1870/1/569 , APOLLO CENTRE ,  VALE CLOSE , RING ROAD</x:v>
       </x:c>
       <x:c r="O248" s="30" t="str"/>
-      <x:c r="P248" s="30" t="str"/>
+      <x:c r="P248" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q248" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -26000,7 +26210,9 @@
         <x:v>111, GROUND FLOOR , NAVSARJAN INDUSTRIAL SOCIETY , UDHNA MAGDALLA ROAD</x:v>
       </x:c>
       <x:c r="O249" s="30" t="str"/>
-      <x:c r="P249" s="30" t="str"/>
+      <x:c r="P249" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q249" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -26108,7 +26320,7 @@
       </x:c>
       <x:c r="O250" s="30" t="str"/>
       <x:c r="P250" s="30" t="str">
-        <x:v>noel,baking,cuti,travel passport,pod,cle,mult,glove,wavy,lunch bag,ketchup,meal prep,75 liter,skin brush,silicone kitchenware,watermelon,cone ice,avocado,wood packing,butter stick</x:v>
+        <x:v>诺埃尔、烘焙、、旅行护照、、、、手套、波浪形、午餐袋、番茄酱、膳食准备、75升、皮肤刷、硅胶厨具、西瓜、圆锥冰、鳄梨、木质包装、黄油棒</x:v>
       </x:c>
       <x:c r="Q250" s="32" t="n">
         <x:v>1</x:v>
@@ -26204,7 +26416,9 @@
         <x:v>25 TO 74 HOANG CAU, WARD O CHO DUA, DISTRICT DONG DA</x:v>
       </x:c>
       <x:c r="O251" s="30" t="str"/>
-      <x:c r="P251" s="30" t="str"/>
+      <x:c r="P251" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q251" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -26301,7 +26515,9 @@
         <x:v>PERIFERICO ECOLOGICO LATERAL OTRA (ESPECIFICAR) OTRA (ESPECIFICAR) OTRA (ESPECIFICAR) 2 A  0</x:v>
       </x:c>
       <x:c r="O252" s="30" t="str"/>
-      <x:c r="P252" s="30" t="str"/>
+      <x:c r="P252" s="30" t="str">
+        <x:v>暂无经营范围信息</x:v>
+      </x:c>
       <x:c r="Q252" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -26411,7 +26627,7 @@
       </x:c>
       <x:c r="O253" s="30" t="str"/>
       <x:c r="P253" s="30" t="str">
-        <x:v>Drilling and well services</x:v>
+        <x:v>钻井和油井服务</x:v>
       </x:c>
       <x:c r="Q253" s="32" t="n">
         <x:v>1</x:v>
@@ -26520,7 +26736,7 @@
       </x:c>
       <x:c r="O254" s="30" t="str"/>
       <x:c r="P254" s="30" t="str">
-        <x:v>Biological and medical products; botanical drugs and herbs; and pharmaceutical products</x:v>
+        <x:v>生物及医药产品；植物药和草药；和医药产品</x:v>
       </x:c>
       <x:c r="Q254" s="32" t="n">
         <x:v>1</x:v>
@@ -26633,7 +26849,7 @@
       </x:c>
       <x:c r="O255" s="30" t="str"/>
       <x:c r="P255" s="30" t="str">
-        <x:v>Metalworking machinery and equipment</x:v>
+        <x:v>金属加工机械及设备</x:v>
       </x:c>
       <x:c r="Q255" s="32" t="n">
         <x:v>1</x:v>
@@ -26728,7 +26944,7 @@
       </x:c>
       <x:c r="O256" s="30" t="str"/>
       <x:c r="P256" s="30" t="str">
-        <x:v>screw,gym accessory,android,tripod stand,exercise,small basket,cycle,skating board,mobile back cover,sunglasses,shoe accessory,body massager,pill box,magnet button,gag,microphone,shoes with light,small glass,ladies umbrella,mmi</x:v>
+        <x:v>螺丝，健身配件，安卓，三脚架，运动，小篮子，周期，滑板，手机后盖，墨镜，鞋配件，身体按摩器，药盒，磁力按钮，堵嘴，麦克风，带灯鞋，小玻璃，女士雨伞</x:v>
       </x:c>
       <x:c r="Q256" s="32" t="n">
         <x:v>1</x:v>
@@ -26819,7 +27035,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5483580c7b574dae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13e37fd9ccb64422"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27468,10 +27684,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="41" t="str">
-        <x:v>经营范围（原文）</x:v>
+        <x:v>经营范围（中文）</x:v>
       </x:c>
       <x:c r="B19" s="41" t="str">
-        <x:v>API返回的公司经营或产品范围原文</x:v>
+        <x:v>API经营或产品范围的中文译文；原文保留在结构化主数据和原始证据中</x:v>
       </x:c>
       <x:c r="C19" s="41" t="str">
         <x:v>API、官网或公式</x:v>

</xml_diff>